<commit_message>
ERD: add SIM-8 (SORT_SEQ, partial send and re-cut of the open qty)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-5" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-6" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-7" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-8" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Column Definition'!$A$3:$H$467</definedName>
@@ -15272,6 +15273,2185 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SIM-8 SORT_SEQ: H0253 lines into scan order, partial send and re-cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="33" t="inlineStr">
+        <is>
+          <t>BPF F2 · Functions: XD09, XD10 (ASN Option, Create ASN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="34" t="inlineStr">
+        <is>
+          <t>• PART-B, 6 pcs/case. H0253 is stored in any order; XD09 numbers the lines of a unit by the scan keys (SORT_SEQ): Customer Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>• Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>• 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>• 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="inlineStr">
+        <is>
+          <t>NEW row</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>UPD row</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>DEL row</t>
+        </is>
+      </c>
+      <c r="E8" s="39" t="inlineStr">
+        <is>
+          <t>READ row</t>
+        </is>
+      </c>
+      <c r="F8" s="40" t="inlineStr">
+        <is>
+          <t>TEMP row</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>Changed cell</t>
+        </is>
+      </c>
+      <c r="H8" s="42" t="inlineStr">
+        <is>
+          <t>PK column</t>
+        </is>
+      </c>
+      <c r="I8" s="36" t="inlineStr">
+        <is>
+          <t>Status OK</t>
+        </is>
+      </c>
+      <c r="J8" s="43" t="inlineStr">
+        <is>
+          <t>Status attention</t>
+        </is>
+      </c>
+      <c r="K8" s="44" t="inlineStr">
+        <is>
+          <t>Status NG / cancel</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="45" t="inlineStr">
+        <is>
+          <t>1. H0253 lines as stored (not sorted)</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="n"/>
+      <c r="C10" s="46" t="n"/>
+      <c r="D10" s="46" t="n"/>
+      <c r="E10" s="46" t="n"/>
+      <c r="F10" s="46" t="n"/>
+      <c r="G10" s="46" t="n"/>
+      <c r="H10" s="46" t="n"/>
+      <c r="I10" s="46" t="n"/>
+      <c r="J10" s="46" t="n"/>
+      <c r="K10" s="46" t="n"/>
+      <c r="L10" s="46" t="n"/>
+      <c r="M10" s="46" t="n"/>
+      <c r="N10" s="46" t="n"/>
+      <c r="O10" s="46" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C12" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D12" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E12" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F12" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G12" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>CANCEL_STATUS</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B13" s="51" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="C13" s="51" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="D13" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E13" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F13" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G13" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H13" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I13" s="52" t="n">
+        <v>14</v>
+      </c>
+      <c r="J13" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K13" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L13" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M13" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N13" s="51" t="inlineStr">
+        <is>
+          <t>Order time 07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B14" s="51" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="C14" s="51" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="D14" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E14" s="51" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F14" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G14" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H14" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I14" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K14" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L14" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M14" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="51" t="inlineStr">
+        <is>
+          <t>Order time 09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B15" s="51" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C15" s="51" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="D15" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E15" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F15" s="51" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G15" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H15" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I15" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K15" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L15" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M15" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N15" s="51" t="inlineStr">
+        <is>
+          <t>Order time 08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B16" s="51" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C16" s="51" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="D16" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E16" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F16" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G16" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H16" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I16" s="52" t="n">
+        <v>8</v>
+      </c>
+      <c r="J16" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K16" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L16" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M16" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N16" s="51" t="inlineStr">
+        <is>
+          <t>Order time 08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B17" s="51" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C17" s="51" t="inlineStr">
+        <is>
+          <t>A-0201</t>
+        </is>
+      </c>
+      <c r="D17" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E17" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F17" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G17" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H17" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I17" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K17" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L17" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M17" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N17" s="51" t="inlineStr">
+        <is>
+          <t>Next unit (15-Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="45" t="inlineStr">
+        <is>
+          <t>2. [Search] 15-Oct (PO1 20 pcs) → XD09: SORT_SEQ, cases, blocks</t>
+        </is>
+      </c>
+      <c r="B19" s="46" t="n"/>
+      <c r="C19" s="46" t="n"/>
+      <c r="D19" s="46" t="n"/>
+      <c r="E19" s="46" t="n"/>
+      <c r="F19" s="46" t="n"/>
+      <c r="G19" s="46" t="n"/>
+      <c r="H19" s="46" t="n"/>
+      <c r="I19" s="46" t="n"/>
+      <c r="J19" s="46" t="n"/>
+      <c r="K19" s="46" t="n"/>
+      <c r="L19" s="46" t="n"/>
+      <c r="M19" s="46" t="n"/>
+      <c r="N19" s="46" t="n"/>
+      <c r="O19" s="46" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>#TEMP_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D20" s="47" t="inlineStr">
+        <is>
+          <t>Temporary (session)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>SORT_SEQ</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>OPEN_ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>ASSIGNED_QTY</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>CUM_DEST_QTY</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>CUT_FLAG</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>GROUP_SEQ</t>
+        </is>
+      </c>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>CROSSDOCK_STATUS</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B22" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D22" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E22" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F22" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G22" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I22" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M22" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O22" s="64" t="inlineStr">
+        <is>
+          <t>SORT_SEQ 1 = 9715300 / A-0101 / item 001</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B23" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D23" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E23" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F23" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G23" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="H23" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I23" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="L23" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M23" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N23" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O23" s="64" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D24" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E24" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F24" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="L24" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N24" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O24" s="64" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B25" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="64" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="D25" s="64" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="E25" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F25" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G25" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I25" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L25" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M25" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N25" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O25" s="64" t="inlineStr">
+        <is>
+          <t>Case 2 = VN 2 + VN 2 + TH 2: no cut (VN 10, TH 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B26" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="64" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="D26" s="64" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="E26" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F26" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G26" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I26" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J26" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L26" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M26" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N26" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O26" s="64" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B27" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D27" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E27" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F27" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G27" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H27" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I27" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="L27" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M27" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N27" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O27" s="64" t="inlineStr">
+        <is>
+          <t>Cut: VN 12, TH 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B28" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D28" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E28" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F28" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G28" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H28" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I28" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="K28" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="L28" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M28" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="N28" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O28" s="64" t="inlineStr">
+        <is>
+          <t>Case 4: only 2 of 6 pcs with PO1 → block 3 Not Ready, block 4 too</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B29" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D29" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E29" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F29" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G29" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H29" s="64" t="n"/>
+      <c r="I29" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J29" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" s="63" t="n">
+        <v>18</v>
+      </c>
+      <c r="L29" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M29" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="N29" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O29" s="64" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B30" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D30" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E30" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F30" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G30" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H30" s="64" t="n"/>
+      <c r="I30" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J30" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="K30" s="63" t="n">
+        <v>24</v>
+      </c>
+      <c r="L30" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M30" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="N30" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O30" s="64" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="45" t="inlineStr">
+        <is>
+          <t>3. Supplier chooses option 1 case → [Create ASN]</t>
+        </is>
+      </c>
+      <c r="B32" s="46" t="n"/>
+      <c r="C32" s="46" t="n"/>
+      <c r="D32" s="46" t="n"/>
+      <c r="E32" s="46" t="n"/>
+      <c r="F32" s="46" t="n"/>
+      <c r="G32" s="46" t="n"/>
+      <c r="H32" s="46" t="n"/>
+      <c r="I32" s="46" t="n"/>
+      <c r="J32" s="46" t="n"/>
+      <c r="K32" s="46" t="n"/>
+      <c r="L32" s="46" t="n"/>
+      <c r="M32" s="46" t="n"/>
+      <c r="N32" s="46" t="n"/>
+      <c r="O32" s="46" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B35" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="49" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="F35" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G35" s="49" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="H35" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I35" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J35" s="49" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="K35" s="49" t="inlineStr">
+        <is>
+          <t>3126035921</t>
+        </is>
+      </c>
+      <c r="L35" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M35" s="49" t="n"/>
+      <c r="N35" s="49" t="n"/>
+      <c r="O35" s="49" t="inlineStr">
+        <is>
+          <t>Item 001: 6 of 8, open 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B38" s="42" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="C38" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="D38" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>MAPPED_QTY</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="C39" s="49" t="inlineStr">
+        <is>
+          <t>3126035921</t>
+        </is>
+      </c>
+      <c r="D39" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="E39" s="49" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="F39" s="53" t="n">
+        <v>20</v>
+      </c>
+      <c r="G39" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="H39" s="49" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="45" t="inlineStr">
+        <is>
+          <t>4. [Search] 16-Oct (PO1 open 14 + PO2 10) → open qty cut again from case 1</t>
+        </is>
+      </c>
+      <c r="B41" s="46" t="n"/>
+      <c r="C41" s="46" t="n"/>
+      <c r="D41" s="46" t="n"/>
+      <c r="E41" s="46" t="n"/>
+      <c r="F41" s="46" t="n"/>
+      <c r="G41" s="46" t="n"/>
+      <c r="H41" s="46" t="n"/>
+      <c r="I41" s="46" t="n"/>
+      <c r="J41" s="46" t="n"/>
+      <c r="K41" s="46" t="n"/>
+      <c r="L41" s="46" t="n"/>
+      <c r="M41" s="46" t="n"/>
+      <c r="N41" s="46" t="n"/>
+      <c r="O41" s="46" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="35" t="inlineStr">
+        <is>
+          <t>#TEMP_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D42" s="47" t="inlineStr">
+        <is>
+          <t>Temporary (session)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>SORT_SEQ</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>OPEN_ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="I43" s="9" t="inlineStr">
+        <is>
+          <t>ASSIGNED_QTY</t>
+        </is>
+      </c>
+      <c r="J43" s="9" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="K43" s="9" t="inlineStr">
+        <is>
+          <t>CUM_DEST_QTY</t>
+        </is>
+      </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>CUT_FLAG</t>
+        </is>
+      </c>
+      <c r="M43" s="9" t="inlineStr">
+        <is>
+          <t>GROUP_SEQ</t>
+        </is>
+      </c>
+      <c r="N43" s="9" t="inlineStr">
+        <is>
+          <t>CROSSDOCK_STATUS</t>
+        </is>
+      </c>
+      <c r="O43" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B44" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D44" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E44" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F44" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G44" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I44" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J44" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L44" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M44" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N44" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O44" s="64" t="inlineStr">
+        <is>
+          <t>Open qty 8 - 6 = 2; case 1 = the same physical case as case 2 on 15-Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B45" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D45" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E45" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F45" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G45" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I45" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J45" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="L45" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M45" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N45" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O45" s="64" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B46" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" s="64" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="D46" s="64" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="E46" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F46" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G46" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H46" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I46" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J46" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L46" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M46" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N46" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O46" s="64" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B47" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" s="64" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="D47" s="64" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="E47" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F47" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G47" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H47" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I47" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J47" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K47" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L47" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M47" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N47" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O47" s="64" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B48" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C48" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D48" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E48" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F48" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G48" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H48" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I48" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J48" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L48" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M48" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N48" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O48" s="64" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B49" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D49" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E49" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F49" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G49" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H49" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I49" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J49" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K49" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="L49" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M49" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N49" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O49" s="64" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B50" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D50" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E50" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F50" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G50" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H50" s="64" t="inlineStr">
+        <is>
+          <t>T0410021</t>
+        </is>
+      </c>
+      <c r="I50" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J50" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="L50" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M50" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N50" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O50" s="64" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B51" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C51" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D51" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E51" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F51" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G51" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H51" s="64" t="inlineStr">
+        <is>
+          <t>T0410021</t>
+        </is>
+      </c>
+      <c r="I51" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J51" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="K51" s="63" t="n">
+        <v>18</v>
+      </c>
+      <c r="L51" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M51" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="N51" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O51" s="64" t="inlineStr">
+        <is>
+          <t>Unit 14-Oct: all 3 blocks Ready (options 2 / 3 / 4 cases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B52" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D52" s="64" t="inlineStr">
+        <is>
+          <t>A-0201</t>
+        </is>
+      </c>
+      <c r="E52" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F52" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H52" s="64" t="n"/>
+      <c r="I52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J52" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L52" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M52" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O52" s="64" t="inlineStr">
+        <is>
+          <t>Unit 15-Oct after unit 14-Oct (way B): no PO left</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -15594,7 +17774,7 @@
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7</t>
+          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8</t>
         </is>
       </c>
     </row>
@@ -15654,7 +17834,7 @@
       </c>
       <c r="F14" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7</t>
+          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8</t>
         </is>
       </c>
     </row>
@@ -15684,7 +17864,7 @@
       </c>
       <c r="F15" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-3, SIM-4, SIM-7</t>
+          <t>SIM-2, SIM-3, SIM-4, SIM-7, SIM-8</t>
         </is>
       </c>
     </row>
@@ -15774,7 +17954,7 @@
       </c>
       <c r="F18" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-5, SIM-6, SIM-7</t>
+          <t>SIM-2, SIM-5, SIM-6, SIM-7, SIM-8</t>
         </is>
       </c>
     </row>
@@ -31978,7 +34158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -32256,6 +34436,38 @@
       <c r="F11" s="32" t="inlineStr">
         <is>
           <t>PART-A 14-Oct, 6 pcs/case: V01 VN 10, T01 TH 6, V02 VN 14 (dummy customer codes CUST-A / B / C give this scan order). p1 (24 pcs) is released 15-Oct, p2 (6 pcs) 16-Oct. Cuts are valid after cases 1, 3, 4 and 5 (VN / TH multiples of 6): blocks case 1 | 2-3 | 4 | 5. 15-Oct: blocks 1-3 Ready, the supplier chooses option 4 cases (blocks 1-3, 24 pcs). 16-Oct: the open 6 pcs of V02 get p2 and go in a second ASN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="32" t="inlineStr">
+        <is>
+          <t>SIM-8</t>
+        </is>
+      </c>
+      <c r="B12" s="32" t="inlineStr">
+        <is>
+          <t>SORT_SEQ: H0253 lines into scan order, partial send and re-cut</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>BPF F2</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>XD09, XD10 (ASN Option, Create ASN)</t>
+        </is>
+      </c>
+      <c r="E12" s="32" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE, #TEMP_INSTRUCTION, TB_R_INSTRUCTION, TB_R_PRA_DAILY_ORDER_MAPPED</t>
+        </is>
+      </c>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>PART-B, 6 pcs/case. H0253 is stored in any order; XD09 numbers the lines of a unit by the scan keys (SORT_SEQ): Customer Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No. Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only. 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
XD09 / SIM-8: scan order = PK order of the H0253 replicate (ORDER BY per unit)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -15316,7 +15316,7 @@
     <row r="3">
       <c r="A3" s="34" t="inlineStr">
         <is>
-          <t>• PART-B, 6 pcs/case. H0253 is stored in any order; XD09 numbers the lines of a unit by the scan keys (SORT_SEQ): Customer Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No.</t>
+          <t>• PART-B, 6 pcs/case. The PK of the H0253 replicate is the 7 scan keys (Customer Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No), so the rows are kept in scan order; the order of the whole table is global (all parts and dates), so XD09 filters the unit and reads it with ORDER BY Part, Order Date + the PK columns. SORT_SEQ = row number in this order.</t>
         </is>
       </c>
     </row>
@@ -15401,7 +15401,7 @@
     <row r="10">
       <c r="A10" s="45" t="inlineStr">
         <is>
-          <t>1. H0253 lines as stored (not sorted)</t>
+          <t>1. H0253 lines in PK order (PK = the 7 scan keys)</t>
         </is>
       </c>
       <c r="B10" s="46" t="n"/>
@@ -15511,12 +15511,12 @@
       </c>
       <c r="B13" s="51" t="inlineStr">
         <is>
-          <t>9730000</t>
+          <t>9715300</t>
         </is>
       </c>
       <c r="C13" s="51" t="inlineStr">
         <is>
-          <t>C-0103</t>
+          <t>A-0101</t>
         </is>
       </c>
       <c r="D13" s="51" t="inlineStr">
@@ -15545,7 +15545,7 @@
         </is>
       </c>
       <c r="I13" s="52" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="J13" s="51" t="inlineStr">
         <is>
@@ -15569,7 +15569,7 @@
       </c>
       <c r="N13" s="51" t="inlineStr">
         <is>
-          <t>Order time 07:00</t>
+          <t>Order time 08:00</t>
         </is>
       </c>
     </row>
@@ -15581,12 +15581,12 @@
       </c>
       <c r="B14" s="51" t="inlineStr">
         <is>
-          <t>9722D00</t>
+          <t>9715300</t>
         </is>
       </c>
       <c r="C14" s="51" t="inlineStr">
         <is>
-          <t>B-0102</t>
+          <t>A-0101</t>
         </is>
       </c>
       <c r="D14" s="51" t="inlineStr">
@@ -15596,12 +15596,12 @@
       </c>
       <c r="E14" s="51" t="inlineStr">
         <is>
-          <t>9722D10</t>
+          <t>9715310</t>
         </is>
       </c>
       <c r="F14" s="51" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G14" s="51" t="inlineStr">
@@ -15615,7 +15615,7 @@
         </is>
       </c>
       <c r="I14" s="52" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J14" s="51" t="inlineStr">
         <is>
@@ -15639,7 +15639,7 @@
       </c>
       <c r="N14" s="51" t="inlineStr">
         <is>
-          <t>Order time 09:00</t>
+          <t>Order time 08:00</t>
         </is>
       </c>
     </row>
@@ -15656,12 +15656,12 @@
       </c>
       <c r="C15" s="51" t="inlineStr">
         <is>
-          <t>A-0101</t>
+          <t>A-0201</t>
         </is>
       </c>
       <c r="D15" s="51" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E15" s="51" t="inlineStr">
@@ -15671,7 +15671,7 @@
       </c>
       <c r="F15" s="51" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G15" s="51" t="inlineStr">
@@ -15685,7 +15685,7 @@
         </is>
       </c>
       <c r="I15" s="52" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J15" s="51" t="inlineStr">
         <is>
@@ -15709,7 +15709,7 @@
       </c>
       <c r="N15" s="51" t="inlineStr">
         <is>
-          <t>Order time 08:00</t>
+          <t>Other unit (15-Oct) between the lines: XD09 splits per unit</t>
         </is>
       </c>
     </row>
@@ -15721,12 +15721,12 @@
       </c>
       <c r="B16" s="51" t="inlineStr">
         <is>
-          <t>9715300</t>
+          <t>9722D00</t>
         </is>
       </c>
       <c r="C16" s="51" t="inlineStr">
         <is>
-          <t>A-0101</t>
+          <t>B-0102</t>
         </is>
       </c>
       <c r="D16" s="51" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="E16" s="51" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>9722D10</t>
         </is>
       </c>
       <c r="F16" s="51" t="inlineStr">
@@ -15755,7 +15755,7 @@
         </is>
       </c>
       <c r="I16" s="52" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J16" s="51" t="inlineStr">
         <is>
@@ -15779,7 +15779,7 @@
       </c>
       <c r="N16" s="51" t="inlineStr">
         <is>
-          <t>Order time 08:00</t>
+          <t>Order time 09:00</t>
         </is>
       </c>
     </row>
@@ -15791,17 +15791,17 @@
       </c>
       <c r="B17" s="51" t="inlineStr">
         <is>
-          <t>9715300</t>
+          <t>9730000</t>
         </is>
       </c>
       <c r="C17" s="51" t="inlineStr">
         <is>
-          <t>A-0201</t>
+          <t>C-0103</t>
         </is>
       </c>
       <c r="D17" s="51" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E17" s="51" t="inlineStr">
@@ -15825,7 +15825,7 @@
         </is>
       </c>
       <c r="I17" s="52" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="J17" s="51" t="inlineStr">
         <is>
@@ -15849,7 +15849,7 @@
       </c>
       <c r="N17" s="51" t="inlineStr">
         <is>
-          <t>Next unit (15-Oct)</t>
+          <t>Order time 07:00: still last (Customer Code first)</t>
         </is>
       </c>
     </row>
@@ -34467,7 +34467,7 @@
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>PART-B, 6 pcs/case. H0253 is stored in any order; XD09 numbers the lines of a unit by the scan keys (SORT_SEQ): Customer Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No. Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only. 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
+          <t>PART-B, 6 pcs/case. The PK of the H0253 replicate is the 7 scan keys (Customer Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No), so the rows are kept in scan order; the order of the whole table is global (all parts and dates), so XD09 filters the unit and reads it with ORDER BY Part, Order Date + the PK columns. SORT_SEQ = row number in this order. Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only. 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
XD09 / ERD: Allocation Priority = Customer Order Date in the scan order, query in XD09 Appendix, SIM-8 step 1b
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -15279,7 +15279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -15316,14 +15316,14 @@
     <row r="3">
       <c r="A3" s="34" t="inlineStr">
         <is>
-          <t>• PART-B, 6 pcs/case. The PK of the H0253 replicate is the 7 scan keys (Customer Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No), so the rows are kept in scan order; the order of the whole table is global (all parts and dates), so XD09 filters the unit and reads it with ORDER BY Part, Order Date + the PK columns. SORT_SEQ = row number in this order.</t>
+          <t>• PART-B, 6 pcs/case. Scan order = G-System allocation order with Allocation Priority = Customer Order Date: 1) Allocation Priority, 2) Customer Code, 3) Customer Order No, 4) Order Date, 5) Order Time, 6) Destination, 7) Detailed Item No, 8) Serial No. Keys 2-8 are the PK of the H0253 replicate; XD09 reads with ORDER BY Part, Allocation Priority + the PK columns (query in XD09 Appendix). SORT_SEQ = row number per unit.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="34" t="inlineStr">
         <is>
-          <t>• Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first.</t>
+          <t>• Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. A-0201 (15-Oct) is in the middle of the PK order but after all 14-Oct lines in the scan order (Allocation Priority).</t>
         </is>
       </c>
     </row>
@@ -15709,7 +15709,7 @@
       </c>
       <c r="N15" s="51" t="inlineStr">
         <is>
-          <t>Other unit (15-Oct) between the lines: XD09 splits per unit</t>
+          <t>15-Oct between the 14-Oct lines in PK order: moved down by the Allocation Priority (1b)</t>
         </is>
       </c>
     </row>
@@ -15856,7 +15856,7 @@
     <row r="19">
       <c r="A19" s="45" t="inlineStr">
         <is>
-          <t>2. [Search] 15-Oct (PO1 20 pcs) → XD09: SORT_SEQ, cases, blocks</t>
+          <t>1b. XD09 read order: ORDER BY Part, Allocation Priority (= Order Date), PK columns</t>
         </is>
       </c>
       <c r="B19" s="46" t="n"/>
@@ -15877,912 +15877,1108 @@
     <row r="20">
       <c r="A20" s="35" t="inlineStr">
         <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D20" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E21" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F21" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G21" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>CANCEL_STATUS</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B22" s="51" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C22" s="51" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="D22" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E22" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F22" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G22" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H22" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I22" s="52" t="n">
+        <v>8</v>
+      </c>
+      <c r="J22" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K22" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L22" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M22" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N22" s="51" t="inlineStr">
+        <is>
+          <t>Priority 14-Oct · SORT_SEQ 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B23" s="51" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C23" s="51" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="D23" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E23" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F23" s="51" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G23" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H23" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I23" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K23" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L23" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M23" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N23" s="51" t="inlineStr">
+        <is>
+          <t>Priority 14-Oct · SORT_SEQ 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="C24" s="51" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="D24" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E24" s="51" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F24" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G24" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H24" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I24" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="J24" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K24" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L24" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M24" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" s="51" t="inlineStr">
+        <is>
+          <t>Priority 14-Oct · SORT_SEQ 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B25" s="51" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="C25" s="51" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="D25" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E25" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F25" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G25" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H25" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I25" s="52" t="n">
+        <v>14</v>
+      </c>
+      <c r="J25" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K25" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L25" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M25" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" s="51" t="inlineStr">
+        <is>
+          <t>Priority 14-Oct · SORT_SEQ 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B26" s="51" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C26" s="51" t="inlineStr">
+        <is>
+          <t>A-0201</t>
+        </is>
+      </c>
+      <c r="D26" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E26" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F26" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G26" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H26" s="51" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="I26" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="J26" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K26" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L26" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M26" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N26" s="51" t="inlineStr">
+        <is>
+          <t>Priority 15-Oct: after all 14-Oct lines (unit 15-Oct, SORT_SEQ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="45" t="inlineStr">
+        <is>
+          <t>2. [Search] 15-Oct (PO1 20 pcs) → XD09: SORT_SEQ, cases, blocks</t>
+        </is>
+      </c>
+      <c r="B28" s="46" t="n"/>
+      <c r="C28" s="46" t="n"/>
+      <c r="D28" s="46" t="n"/>
+      <c r="E28" s="46" t="n"/>
+      <c r="F28" s="46" t="n"/>
+      <c r="G28" s="46" t="n"/>
+      <c r="H28" s="46" t="n"/>
+      <c r="I28" s="46" t="n"/>
+      <c r="J28" s="46" t="n"/>
+      <c r="K28" s="46" t="n"/>
+      <c r="L28" s="46" t="n"/>
+      <c r="M28" s="46" t="n"/>
+      <c r="N28" s="46" t="n"/>
+      <c r="O28" s="46" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
           <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
-      <c r="D20" s="47" t="inlineStr">
+      <c r="D29" s="47" t="inlineStr">
         <is>
           <t>Temporary (session)</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>SORT_SEQ</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>CUSTOMER_CD</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>DESTINATION_CD</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>PART_NO</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>OPEN_ORDER_QTY</t>
         </is>
       </c>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="H30" s="9" t="inlineStr">
         <is>
           <t>PO_NO</t>
         </is>
       </c>
-      <c r="I21" s="9" t="inlineStr">
+      <c r="I30" s="9" t="inlineStr">
         <is>
           <t>ASSIGNED_QTY</t>
         </is>
       </c>
-      <c r="J21" s="9" t="inlineStr">
+      <c r="J30" s="9" t="inlineStr">
         <is>
           <t>CASE_SEQ</t>
         </is>
       </c>
-      <c r="K21" s="9" t="inlineStr">
+      <c r="K30" s="9" t="inlineStr">
         <is>
           <t>CUM_DEST_QTY</t>
         </is>
       </c>
-      <c r="L21" s="9" t="inlineStr">
+      <c r="L30" s="9" t="inlineStr">
         <is>
           <t>CUT_FLAG</t>
         </is>
       </c>
-      <c r="M21" s="9" t="inlineStr">
+      <c r="M30" s="9" t="inlineStr">
         <is>
           <t>GROUP_SEQ</t>
         </is>
       </c>
-      <c r="N21" s="9" t="inlineStr">
+      <c r="N30" s="9" t="inlineStr">
         <is>
           <t>CROSSDOCK_STATUS</t>
         </is>
       </c>
-      <c r="O21" s="9" t="inlineStr">
+      <c r="O30" s="9" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="62" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B22" s="63" t="n">
+      <c r="B31" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="64" t="inlineStr">
+      <c r="C31" s="64" t="inlineStr">
         <is>
           <t>9715300</t>
         </is>
       </c>
-      <c r="D22" s="64" t="inlineStr">
+      <c r="D31" s="64" t="inlineStr">
         <is>
           <t>A-0101</t>
         </is>
       </c>
-      <c r="E22" s="64" t="inlineStr">
+      <c r="E31" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F22" s="64" t="inlineStr">
+      <c r="F31" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G22" s="63" t="n">
+      <c r="G31" s="63" t="n">
         <v>8</v>
       </c>
-      <c r="H22" s="64" t="inlineStr">
+      <c r="H31" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I22" s="63" t="n">
+      <c r="I31" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="J22" s="63" t="n">
+      <c r="J31" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="K22" s="63" t="n">
+      <c r="K31" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="L22" s="65" t="inlineStr">
+      <c r="L31" s="65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M22" s="63" t="n">
+      <c r="M31" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="N22" s="49" t="inlineStr">
+      <c r="N31" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O22" s="64" t="inlineStr">
+      <c r="O31" s="64" t="inlineStr">
         <is>
           <t>SORT_SEQ 1 = 9715300 / A-0101 / item 001</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="62" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B23" s="63" t="n">
+      <c r="B32" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="64" t="inlineStr">
+      <c r="C32" s="64" t="inlineStr">
         <is>
           <t>9715300</t>
         </is>
       </c>
-      <c r="D23" s="64" t="inlineStr">
+      <c r="D32" s="64" t="inlineStr">
         <is>
           <t>A-0101</t>
         </is>
       </c>
-      <c r="E23" s="64" t="inlineStr">
+      <c r="E32" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F23" s="64" t="inlineStr">
+      <c r="F32" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G23" s="63" t="n">
+      <c r="G32" s="63" t="n">
         <v>8</v>
       </c>
-      <c r="H23" s="64" t="inlineStr">
+      <c r="H32" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I23" s="63" t="n">
+      <c r="I32" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J23" s="63" t="n">
+      <c r="J32" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="K23" s="63" t="n">
+      <c r="K32" s="63" t="n">
         <v>8</v>
       </c>
-      <c r="L23" s="64" t="inlineStr">
+      <c r="L32" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M23" s="63" t="n">
+      <c r="M32" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="N23" s="49" t="inlineStr">
+      <c r="N32" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O23" s="64" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="62" t="inlineStr">
+      <c r="O32" s="64" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B24" s="63" t="n">
+      <c r="B33" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="C24" s="64" t="inlineStr">
+      <c r="C33" s="64" t="inlineStr">
         <is>
           <t>9715300</t>
         </is>
       </c>
-      <c r="D24" s="64" t="inlineStr">
+      <c r="D33" s="64" t="inlineStr">
         <is>
           <t>A-0101</t>
         </is>
       </c>
-      <c r="E24" s="64" t="inlineStr">
+      <c r="E33" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F24" s="64" t="inlineStr">
+      <c r="F33" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G24" s="63" t="n">
+      <c r="G33" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="H24" s="64" t="inlineStr">
+      <c r="H33" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I24" s="63" t="n">
+      <c r="I33" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J24" s="63" t="n">
+      <c r="J33" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="K24" s="63" t="n">
+      <c r="K33" s="63" t="n">
         <v>10</v>
       </c>
-      <c r="L24" s="64" t="inlineStr">
+      <c r="L33" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M24" s="63" t="n">
+      <c r="M33" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="N24" s="49" t="inlineStr">
+      <c r="N33" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O24" s="64" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="62" t="inlineStr">
+      <c r="O33" s="64" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B25" s="63" t="n">
+      <c r="B34" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="C25" s="64" t="inlineStr">
+      <c r="C34" s="64" t="inlineStr">
         <is>
           <t>9722D00</t>
         </is>
       </c>
-      <c r="D25" s="64" t="inlineStr">
+      <c r="D34" s="64" t="inlineStr">
         <is>
           <t>B-0102</t>
         </is>
       </c>
-      <c r="E25" s="64" t="inlineStr">
+      <c r="E34" s="64" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="F25" s="64" t="inlineStr">
+      <c r="F34" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G25" s="63" t="n">
+      <c r="G34" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="H25" s="64" t="inlineStr">
+      <c r="H34" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I25" s="63" t="n">
+      <c r="I34" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J25" s="63" t="n">
+      <c r="J34" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="K25" s="63" t="n">
+      <c r="K34" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="L25" s="64" t="inlineStr">
+      <c r="L34" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M25" s="63" t="n">
+      <c r="M34" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="N25" s="49" t="inlineStr">
+      <c r="N34" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O25" s="64" t="inlineStr">
+      <c r="O34" s="64" t="inlineStr">
         <is>
           <t>Case 2 = VN 2 + VN 2 + TH 2: no cut (VN 10, TH 2)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="62" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B26" s="63" t="n">
+      <c r="B35" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="C26" s="64" t="inlineStr">
+      <c r="C35" s="64" t="inlineStr">
         <is>
           <t>9722D00</t>
         </is>
       </c>
-      <c r="D26" s="64" t="inlineStr">
+      <c r="D35" s="64" t="inlineStr">
         <is>
           <t>B-0102</t>
         </is>
       </c>
-      <c r="E26" s="64" t="inlineStr">
+      <c r="E35" s="64" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="F26" s="64" t="inlineStr">
+      <c r="F35" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G26" s="63" t="n">
+      <c r="G35" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="H26" s="64" t="inlineStr">
+      <c r="H35" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I26" s="63" t="n">
+      <c r="I35" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="J26" s="63" t="n">
+      <c r="J35" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="K26" s="63" t="n">
+      <c r="K35" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="L26" s="64" t="inlineStr">
+      <c r="L35" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M26" s="63" t="n">
+      <c r="M35" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="N26" s="49" t="inlineStr">
+      <c r="N35" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O26" s="64" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="62" t="inlineStr">
+      <c r="O35" s="64" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B27" s="63" t="n">
+      <c r="B36" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="C27" s="64" t="inlineStr">
+      <c r="C36" s="64" t="inlineStr">
         <is>
           <t>9730000</t>
         </is>
       </c>
-      <c r="D27" s="64" t="inlineStr">
+      <c r="D36" s="64" t="inlineStr">
         <is>
           <t>C-0103</t>
         </is>
       </c>
-      <c r="E27" s="64" t="inlineStr">
+      <c r="E36" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F27" s="64" t="inlineStr">
+      <c r="F36" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G27" s="63" t="n">
+      <c r="G36" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="H27" s="64" t="inlineStr">
+      <c r="H36" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I27" s="63" t="n">
+      <c r="I36" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J27" s="63" t="n">
+      <c r="J36" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="K27" s="63" t="n">
+      <c r="K36" s="63" t="n">
         <v>12</v>
       </c>
-      <c r="L27" s="65" t="inlineStr">
+      <c r="L36" s="65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M27" s="63" t="n">
+      <c r="M36" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="N27" s="49" t="inlineStr">
+      <c r="N36" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O27" s="64" t="inlineStr">
+      <c r="O36" s="64" t="inlineStr">
         <is>
           <t>Cut: VN 12, TH 6</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="62" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B28" s="63" t="n">
+      <c r="B37" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="C28" s="64" t="inlineStr">
+      <c r="C37" s="64" t="inlineStr">
         <is>
           <t>9730000</t>
         </is>
       </c>
-      <c r="D28" s="64" t="inlineStr">
+      <c r="D37" s="64" t="inlineStr">
         <is>
           <t>C-0103</t>
         </is>
       </c>
-      <c r="E28" s="64" t="inlineStr">
+      <c r="E37" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F28" s="64" t="inlineStr">
+      <c r="F37" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G28" s="63" t="n">
+      <c r="G37" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="H28" s="64" t="inlineStr">
+      <c r="H37" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I28" s="63" t="n">
+      <c r="I37" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J28" s="63" t="n">
+      <c r="J37" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="K28" s="63" t="n">
+      <c r="K37" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="L28" s="64" t="inlineStr">
+      <c r="L37" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M28" s="63" t="n">
+      <c r="M37" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="N28" s="66" t="inlineStr">
+      <c r="N37" s="66" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="O28" s="64" t="inlineStr">
+      <c r="O37" s="64" t="inlineStr">
         <is>
           <t>Case 4: only 2 of 6 pcs with PO1 → block 3 Not Ready, block 4 too</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="62" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B29" s="63" t="n">
+      <c r="B38" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="C29" s="64" t="inlineStr">
+      <c r="C38" s="64" t="inlineStr">
         <is>
           <t>9730000</t>
         </is>
       </c>
-      <c r="D29" s="64" t="inlineStr">
+      <c r="D38" s="64" t="inlineStr">
         <is>
           <t>C-0103</t>
         </is>
       </c>
-      <c r="E29" s="64" t="inlineStr">
+      <c r="E38" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F29" s="64" t="inlineStr">
+      <c r="F38" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G29" s="63" t="n">
+      <c r="G38" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="H29" s="64" t="n"/>
-      <c r="I29" s="63" t="n">
+      <c r="H38" s="64" t="n"/>
+      <c r="I38" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="J29" s="63" t="n">
+      <c r="J38" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="K29" s="63" t="n">
+      <c r="K38" s="63" t="n">
         <v>18</v>
       </c>
-      <c r="L29" s="65" t="inlineStr">
+      <c r="L38" s="65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M29" s="63" t="n">
+      <c r="M38" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="N29" s="66" t="inlineStr">
+      <c r="N38" s="66" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="O29" s="64" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="62" t="inlineStr">
+      <c r="O38" s="64" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B30" s="63" t="n">
+      <c r="B39" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="C30" s="64" t="inlineStr">
+      <c r="C39" s="64" t="inlineStr">
         <is>
           <t>9730000</t>
         </is>
       </c>
-      <c r="D30" s="64" t="inlineStr">
+      <c r="D39" s="64" t="inlineStr">
         <is>
           <t>C-0103</t>
         </is>
       </c>
-      <c r="E30" s="64" t="inlineStr">
+      <c r="E39" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F30" s="64" t="inlineStr">
+      <c r="F39" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G30" s="63" t="n">
+      <c r="G39" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="H30" s="64" t="n"/>
-      <c r="I30" s="63" t="n">
+      <c r="H39" s="64" t="n"/>
+      <c r="I39" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="J30" s="63" t="n">
+      <c r="J39" s="63" t="n">
         <v>5</v>
       </c>
-      <c r="K30" s="63" t="n">
+      <c r="K39" s="63" t="n">
         <v>24</v>
       </c>
-      <c r="L30" s="65" t="inlineStr">
+      <c r="L39" s="65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M30" s="63" t="n">
+      <c r="M39" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="N30" s="66" t="inlineStr">
+      <c r="N39" s="66" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="O30" s="64" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="45" t="inlineStr">
-        <is>
-          <t>3. Supplier chooses option 1 case → [Create ASN]</t>
-        </is>
-      </c>
-      <c r="B32" s="46" t="n"/>
-      <c r="C32" s="46" t="n"/>
-      <c r="D32" s="46" t="n"/>
-      <c r="E32" s="46" t="n"/>
-      <c r="F32" s="46" t="n"/>
-      <c r="G32" s="46" t="n"/>
-      <c r="H32" s="46" t="n"/>
-      <c r="I32" s="46" t="n"/>
-      <c r="J32" s="46" t="n"/>
-      <c r="K32" s="46" t="n"/>
-      <c r="L32" s="46" t="n"/>
-      <c r="M32" s="46" t="n"/>
-      <c r="N32" s="46" t="n"/>
-      <c r="O32" s="46" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D33" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B34" s="42" t="inlineStr">
-        <is>
-          <t>INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>LINE_SEQ</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="L34" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="M34" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="N34" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
-        </is>
-      </c>
-      <c r="O34" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B35" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="49" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="F35" s="49" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="G35" s="49" t="inlineStr">
-        <is>
-          <t>A-0101</t>
-        </is>
-      </c>
-      <c r="H35" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="I35" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="J35" s="49" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="K35" s="49" t="inlineStr">
-        <is>
-          <t>3126035921</t>
-        </is>
-      </c>
-      <c r="L35" s="49" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="M35" s="49" t="n"/>
-      <c r="N35" s="49" t="n"/>
-      <c r="O35" s="49" t="inlineStr">
-        <is>
-          <t>Item 001: 6 of 8, open 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
-        </is>
-      </c>
-      <c r="D37" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B38" s="42" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="C38" s="42" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="D38" s="42" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>ORDER_QTY</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>MAPPED_QTY</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B39" s="49" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="C39" s="49" t="inlineStr">
-        <is>
-          <t>3126035921</t>
-        </is>
-      </c>
-      <c r="D39" s="49" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="E39" s="49" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="F39" s="53" t="n">
-        <v>20</v>
-      </c>
-      <c r="G39" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="H39" s="49" t="inlineStr"/>
+      <c r="O39" s="64" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="45" t="inlineStr">
         <is>
-          <t>4. [Search] 16-Oct (PO1 open 14 + PO2 10) → open qty cut again from case 1</t>
+          <t>3. Supplier chooses option 1 case → [Create ASN]</t>
         </is>
       </c>
       <c r="B41" s="46" t="n"/>
@@ -16803,644 +16999,903 @@
     <row r="42">
       <c r="A42" s="35" t="inlineStr">
         <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D42" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B43" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B44" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="49" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="F44" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G44" s="49" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="H44" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I44" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J44" s="49" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="K44" s="49" t="inlineStr">
+        <is>
+          <t>3126035921</t>
+        </is>
+      </c>
+      <c r="L44" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M44" s="49" t="n"/>
+      <c r="N44" s="49" t="n"/>
+      <c r="O44" s="49" t="inlineStr">
+        <is>
+          <t>Item 001: 6 of 8, open 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
+        </is>
+      </c>
+      <c r="D46" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B47" s="42" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="C47" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="D47" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>MAPPED_QTY</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="C48" s="49" t="inlineStr">
+        <is>
+          <t>3126035921</t>
+        </is>
+      </c>
+      <c r="D48" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="E48" s="49" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="F48" s="53" t="n">
+        <v>20</v>
+      </c>
+      <c r="G48" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="H48" s="49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="45" t="inlineStr">
+        <is>
+          <t>4. [Search] 16-Oct (PO1 open 14 + PO2 10) → open qty cut again from case 1</t>
+        </is>
+      </c>
+      <c r="B50" s="46" t="n"/>
+      <c r="C50" s="46" t="n"/>
+      <c r="D50" s="46" t="n"/>
+      <c r="E50" s="46" t="n"/>
+      <c r="F50" s="46" t="n"/>
+      <c r="G50" s="46" t="n"/>
+      <c r="H50" s="46" t="n"/>
+      <c r="I50" s="46" t="n"/>
+      <c r="J50" s="46" t="n"/>
+      <c r="K50" s="46" t="n"/>
+      <c r="L50" s="46" t="n"/>
+      <c r="M50" s="46" t="n"/>
+      <c r="N50" s="46" t="n"/>
+      <c r="O50" s="46" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="35" t="inlineStr">
+        <is>
           <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
-      <c r="D42" s="47" t="inlineStr">
+      <c r="D51" s="47" t="inlineStr">
         <is>
           <t>Temporary (session)</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
+    <row r="52" ht="26" customHeight="1">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>SORT_SEQ</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>CUSTOMER_CD</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D52" s="9" t="inlineStr">
         <is>
           <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
         <is>
           <t>DESTINATION_CD</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="F52" s="9" t="inlineStr">
         <is>
           <t>PART_NO</t>
         </is>
       </c>
-      <c r="G43" s="9" t="inlineStr">
+      <c r="G52" s="9" t="inlineStr">
         <is>
           <t>OPEN_ORDER_QTY</t>
         </is>
       </c>
-      <c r="H43" s="9" t="inlineStr">
+      <c r="H52" s="9" t="inlineStr">
         <is>
           <t>PO_NO</t>
         </is>
       </c>
-      <c r="I43" s="9" t="inlineStr">
+      <c r="I52" s="9" t="inlineStr">
         <is>
           <t>ASSIGNED_QTY</t>
         </is>
       </c>
-      <c r="J43" s="9" t="inlineStr">
+      <c r="J52" s="9" t="inlineStr">
         <is>
           <t>CASE_SEQ</t>
         </is>
       </c>
-      <c r="K43" s="9" t="inlineStr">
+      <c r="K52" s="9" t="inlineStr">
         <is>
           <t>CUM_DEST_QTY</t>
         </is>
       </c>
-      <c r="L43" s="9" t="inlineStr">
+      <c r="L52" s="9" t="inlineStr">
         <is>
           <t>CUT_FLAG</t>
         </is>
       </c>
-      <c r="M43" s="9" t="inlineStr">
+      <c r="M52" s="9" t="inlineStr">
         <is>
           <t>GROUP_SEQ</t>
         </is>
       </c>
-      <c r="N43" s="9" t="inlineStr">
+      <c r="N52" s="9" t="inlineStr">
         <is>
           <t>CROSSDOCK_STATUS</t>
         </is>
       </c>
-      <c r="O43" s="9" t="inlineStr">
+      <c r="O52" s="9" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="62" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B44" s="63" t="n">
+      <c r="B53" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="C44" s="64" t="inlineStr">
+      <c r="C53" s="64" t="inlineStr">
         <is>
           <t>9715300</t>
         </is>
       </c>
-      <c r="D44" s="64" t="inlineStr">
+      <c r="D53" s="64" t="inlineStr">
         <is>
           <t>A-0101</t>
         </is>
       </c>
-      <c r="E44" s="64" t="inlineStr">
+      <c r="E53" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F44" s="64" t="inlineStr">
+      <c r="F53" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G44" s="63" t="n">
+      <c r="G53" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="H44" s="64" t="inlineStr">
+      <c r="H53" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I44" s="63" t="n">
+      <c r="I53" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J44" s="63" t="n">
+      <c r="J53" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="K44" s="63" t="n">
+      <c r="K53" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="L44" s="64" t="inlineStr">
+      <c r="L53" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M44" s="63" t="n">
+      <c r="M53" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="N44" s="49" t="inlineStr">
+      <c r="N53" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O44" s="64" t="inlineStr">
+      <c r="O53" s="64" t="inlineStr">
         <is>
           <t>Open qty 8 - 6 = 2; case 1 = the same physical case as case 2 on 15-Oct</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="62" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B45" s="63" t="n">
+      <c r="B54" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="C45" s="64" t="inlineStr">
+      <c r="C54" s="64" t="inlineStr">
         <is>
           <t>9715300</t>
         </is>
       </c>
-      <c r="D45" s="64" t="inlineStr">
+      <c r="D54" s="64" t="inlineStr">
         <is>
           <t>A-0101</t>
         </is>
       </c>
-      <c r="E45" s="64" t="inlineStr">
+      <c r="E54" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F45" s="64" t="inlineStr">
+      <c r="F54" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G45" s="63" t="n">
+      <c r="G54" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="H45" s="64" t="inlineStr">
+      <c r="H54" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I45" s="63" t="n">
+      <c r="I54" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J45" s="63" t="n">
+      <c r="J54" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="K45" s="63" t="n">
+      <c r="K54" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="L45" s="64" t="inlineStr">
+      <c r="L54" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M45" s="63" t="n">
+      <c r="M54" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="49" t="inlineStr">
+      <c r="N54" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O45" s="64" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="62" t="inlineStr">
+      <c r="O54" s="64" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B46" s="63" t="n">
+      <c r="B55" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="C46" s="64" t="inlineStr">
+      <c r="C55" s="64" t="inlineStr">
         <is>
           <t>9722D00</t>
         </is>
       </c>
-      <c r="D46" s="64" t="inlineStr">
+      <c r="D55" s="64" t="inlineStr">
         <is>
           <t>B-0102</t>
         </is>
       </c>
-      <c r="E46" s="64" t="inlineStr">
+      <c r="E55" s="64" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="F46" s="64" t="inlineStr">
+      <c r="F55" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G46" s="63" t="n">
+      <c r="G55" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="H46" s="64" t="inlineStr">
+      <c r="H55" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I46" s="63" t="n">
+      <c r="I55" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J46" s="63" t="n">
+      <c r="J55" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="K46" s="63" t="n">
+      <c r="K55" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="L46" s="64" t="inlineStr">
+      <c r="L55" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M46" s="63" t="n">
+      <c r="M55" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="N46" s="49" t="inlineStr">
+      <c r="N55" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O46" s="64" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="62" t="inlineStr">
+      <c r="O55" s="64" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B47" s="63" t="n">
+      <c r="B56" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="C47" s="64" t="inlineStr">
+      <c r="C56" s="64" t="inlineStr">
         <is>
           <t>9722D00</t>
         </is>
       </c>
-      <c r="D47" s="64" t="inlineStr">
+      <c r="D56" s="64" t="inlineStr">
         <is>
           <t>B-0102</t>
         </is>
       </c>
-      <c r="E47" s="64" t="inlineStr">
+      <c r="E56" s="64" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="F47" s="64" t="inlineStr">
+      <c r="F56" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G47" s="63" t="n">
+      <c r="G56" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="H47" s="64" t="inlineStr">
+      <c r="H56" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I47" s="63" t="n">
+      <c r="I56" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="J47" s="63" t="n">
+      <c r="J56" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="K47" s="63" t="n">
+      <c r="K56" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="L47" s="64" t="inlineStr">
+      <c r="L56" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M47" s="63" t="n">
+      <c r="M56" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="N47" s="49" t="inlineStr">
+      <c r="N56" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O47" s="64" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="62" t="inlineStr">
+      <c r="O56" s="64" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B48" s="63" t="n">
+      <c r="B57" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="C48" s="64" t="inlineStr">
+      <c r="C57" s="64" t="inlineStr">
         <is>
           <t>9730000</t>
         </is>
       </c>
-      <c r="D48" s="64" t="inlineStr">
+      <c r="D57" s="64" t="inlineStr">
         <is>
           <t>C-0103</t>
         </is>
       </c>
-      <c r="E48" s="64" t="inlineStr">
+      <c r="E57" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F48" s="64" t="inlineStr">
+      <c r="F57" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G48" s="63" t="n">
+      <c r="G57" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="H48" s="64" t="inlineStr">
+      <c r="H57" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I48" s="63" t="n">
+      <c r="I57" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J48" s="63" t="n">
+      <c r="J57" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="K48" s="63" t="n">
+      <c r="K57" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="L48" s="65" t="inlineStr">
+      <c r="L57" s="65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M48" s="63" t="n">
+      <c r="M57" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="49" t="inlineStr">
+      <c r="N57" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O48" s="64" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="62" t="inlineStr">
+      <c r="O57" s="64" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B49" s="63" t="n">
+      <c r="B58" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="C49" s="64" t="inlineStr">
+      <c r="C58" s="64" t="inlineStr">
         <is>
           <t>9730000</t>
         </is>
       </c>
-      <c r="D49" s="64" t="inlineStr">
+      <c r="D58" s="64" t="inlineStr">
         <is>
           <t>C-0103</t>
         </is>
       </c>
-      <c r="E49" s="64" t="inlineStr">
+      <c r="E58" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F49" s="64" t="inlineStr">
+      <c r="F58" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G49" s="63" t="n">
+      <c r="G58" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="H49" s="64" t="inlineStr">
+      <c r="H58" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="I49" s="63" t="n">
+      <c r="I58" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="J49" s="63" t="n">
+      <c r="J58" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="K49" s="63" t="n">
+      <c r="K58" s="63" t="n">
         <v>8</v>
       </c>
-      <c r="L49" s="64" t="inlineStr">
+      <c r="L58" s="64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M49" s="63" t="n">
+      <c r="M58" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="N49" s="49" t="inlineStr">
+      <c r="N58" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O49" s="64" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="62" t="inlineStr">
+      <c r="O58" s="64" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B50" s="63" t="n">
+      <c r="B59" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="C50" s="64" t="inlineStr">
+      <c r="C59" s="64" t="inlineStr">
         <is>
           <t>9730000</t>
         </is>
       </c>
-      <c r="D50" s="64" t="inlineStr">
+      <c r="D59" s="64" t="inlineStr">
         <is>
           <t>C-0103</t>
         </is>
       </c>
-      <c r="E50" s="64" t="inlineStr">
+      <c r="E59" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F50" s="64" t="inlineStr">
+      <c r="F59" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G50" s="63" t="n">
+      <c r="G59" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="H50" s="64" t="inlineStr">
+      <c r="H59" s="64" t="inlineStr">
         <is>
           <t>T0410021</t>
         </is>
       </c>
-      <c r="I50" s="63" t="n">
+      <c r="I59" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="J50" s="63" t="n">
+      <c r="J59" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="K50" s="63" t="n">
+      <c r="K59" s="63" t="n">
         <v>12</v>
       </c>
-      <c r="L50" s="65" t="inlineStr">
+      <c r="L59" s="65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M50" s="63" t="n">
+      <c r="M59" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="N50" s="49" t="inlineStr">
+      <c r="N59" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O50" s="64" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="62" t="inlineStr">
+      <c r="O59" s="64" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B51" s="63" t="n">
+      <c r="B60" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="C51" s="64" t="inlineStr">
+      <c r="C60" s="64" t="inlineStr">
         <is>
           <t>9730000</t>
         </is>
       </c>
-      <c r="D51" s="64" t="inlineStr">
+      <c r="D60" s="64" t="inlineStr">
         <is>
           <t>C-0103</t>
         </is>
       </c>
-      <c r="E51" s="64" t="inlineStr">
+      <c r="E60" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F51" s="64" t="inlineStr">
+      <c r="F60" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G51" s="63" t="n">
+      <c r="G60" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="H51" s="64" t="inlineStr">
+      <c r="H60" s="64" t="inlineStr">
         <is>
           <t>T0410021</t>
         </is>
       </c>
-      <c r="I51" s="63" t="n">
+      <c r="I60" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="J51" s="63" t="n">
+      <c r="J60" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="K51" s="63" t="n">
+      <c r="K60" s="63" t="n">
         <v>18</v>
       </c>
-      <c r="L51" s="65" t="inlineStr">
+      <c r="L60" s="65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M51" s="63" t="n">
+      <c r="M60" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="N51" s="49" t="inlineStr">
+      <c r="N60" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="O51" s="64" t="inlineStr">
+      <c r="O60" s="64" t="inlineStr">
         <is>
           <t>Unit 14-Oct: all 3 blocks Ready (options 2 / 3 / 4 cases)</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="62" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B52" s="63" t="n">
+      <c r="B61" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="C52" s="64" t="inlineStr">
+      <c r="C61" s="64" t="inlineStr">
         <is>
           <t>9715300</t>
         </is>
       </c>
-      <c r="D52" s="64" t="inlineStr">
+      <c r="D61" s="64" t="inlineStr">
         <is>
           <t>A-0201</t>
         </is>
       </c>
-      <c r="E52" s="64" t="inlineStr">
+      <c r="E61" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F52" s="64" t="inlineStr">
+      <c r="F61" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G52" s="63" t="n">
+      <c r="G61" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="H52" s="64" t="n"/>
-      <c r="I52" s="63" t="n">
+      <c r="H61" s="64" t="n"/>
+      <c r="I61" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="J52" s="63" t="n">
+      <c r="J61" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="K52" s="63" t="n">
+      <c r="K61" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="L52" s="65" t="inlineStr">
+      <c r="L61" s="65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M52" s="63" t="n">
+      <c r="M61" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="N52" s="66" t="inlineStr">
+      <c r="N61" s="66" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="O52" s="64" t="inlineStr">
+      <c r="O61" s="64" t="inlineStr">
         <is>
           <t>Unit 15-Oct after unit 14-Oct (way B): no PO left</t>
         </is>
@@ -34467,7 +34922,7 @@
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>PART-B, 6 pcs/case. The PK of the H0253 replicate is the 7 scan keys (Customer Code, Customer Order No, Order Date, Order Time, Destination, Detailed Item No, Serial No), so the rows are kept in scan order; the order of the whole table is global (all parts and dates), so XD09 filters the unit and reads it with ORDER BY Part, Order Date + the PK columns. SORT_SEQ = row number in this order. Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only. 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
+          <t>PART-B, 6 pcs/case. Scan order = G-System allocation order with Allocation Priority = Customer Order Date: 1) Allocation Priority, 2) Customer Code, 3) Customer Order No, 4) Order Date, 5) Order Time, 6) Destination, 7) Detailed Item No, 8) Serial No. Keys 2-8 are the PK of the H0253 replicate; XD09 reads with ORDER BY Part, Allocation Priority + the PK columns (query in XD09 Appendix). SORT_SEQ = row number per unit. Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. A-0201 (15-Oct) is in the middle of the PK order but after all 14-Oct lines in the scan order (Allocation Priority). 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only. 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SIM-8: keep only the scan-order step for the H0253 lines
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -15279,7 +15279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -15323,7 +15323,7 @@
     <row r="4">
       <c r="A4" s="34" t="inlineStr">
         <is>
-          <t>• Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. A-0201 (15-Oct) is in the middle of the PK order but after all 14-Oct lines in the scan order (Allocation Priority).</t>
+          <t>• Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. A-0201 (15-Oct) comes after all 14-Oct lines (Allocation Priority) and is the next unit.</t>
         </is>
       </c>
     </row>
@@ -15401,7 +15401,7 @@
     <row r="10">
       <c r="A10" s="45" t="inlineStr">
         <is>
-          <t>1. H0253 lines in PK order (PK = the 7 scan keys)</t>
+          <t>1. H0253 lines in scan order: ORDER BY Part, Allocation Priority (= Order Date), PK columns</t>
         </is>
       </c>
       <c r="B10" s="46" t="n"/>
@@ -15569,7 +15569,7 @@
       </c>
       <c r="N13" s="51" t="inlineStr">
         <is>
-          <t>Order time 08:00</t>
+          <t>Priority 14-Oct · SORT_SEQ 1</t>
         </is>
       </c>
     </row>
@@ -15639,7 +15639,7 @@
       </c>
       <c r="N14" s="51" t="inlineStr">
         <is>
-          <t>Order time 08:00</t>
+          <t>Priority 14-Oct · SORT_SEQ 2</t>
         </is>
       </c>
     </row>
@@ -15651,22 +15651,22 @@
       </c>
       <c r="B15" s="51" t="inlineStr">
         <is>
-          <t>9715300</t>
+          <t>9722D00</t>
         </is>
       </c>
       <c r="C15" s="51" t="inlineStr">
         <is>
-          <t>A-0201</t>
+          <t>B-0102</t>
         </is>
       </c>
       <c r="D15" s="51" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E15" s="51" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>9722D10</t>
         </is>
       </c>
       <c r="F15" s="51" t="inlineStr">
@@ -15709,7 +15709,7 @@
       </c>
       <c r="N15" s="51" t="inlineStr">
         <is>
-          <t>15-Oct between the 14-Oct lines in PK order: moved down by the Allocation Priority (1b)</t>
+          <t>Priority 14-Oct · SORT_SEQ 3</t>
         </is>
       </c>
     </row>
@@ -15721,12 +15721,12 @@
       </c>
       <c r="B16" s="51" t="inlineStr">
         <is>
-          <t>9722D00</t>
+          <t>9730000</t>
         </is>
       </c>
       <c r="C16" s="51" t="inlineStr">
         <is>
-          <t>B-0102</t>
+          <t>C-0103</t>
         </is>
       </c>
       <c r="D16" s="51" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="E16" s="51" t="inlineStr">
         <is>
-          <t>9722D10</t>
+          <t>9715310</t>
         </is>
       </c>
       <c r="F16" s="51" t="inlineStr">
@@ -15755,7 +15755,7 @@
         </is>
       </c>
       <c r="I16" s="52" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="J16" s="51" t="inlineStr">
         <is>
@@ -15779,7 +15779,7 @@
       </c>
       <c r="N16" s="51" t="inlineStr">
         <is>
-          <t>Order time 09:00</t>
+          <t>Priority 14-Oct · SORT_SEQ 4</t>
         </is>
       </c>
     </row>
@@ -15791,17 +15791,17 @@
       </c>
       <c r="B17" s="51" t="inlineStr">
         <is>
-          <t>9730000</t>
+          <t>9715300</t>
         </is>
       </c>
       <c r="C17" s="51" t="inlineStr">
         <is>
-          <t>C-0103</t>
+          <t>A-0201</t>
         </is>
       </c>
       <c r="D17" s="51" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E17" s="51" t="inlineStr">
@@ -15825,7 +15825,7 @@
         </is>
       </c>
       <c r="I17" s="52" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="J17" s="51" t="inlineStr">
         <is>
@@ -15849,14 +15849,14 @@
       </c>
       <c r="N17" s="51" t="inlineStr">
         <is>
-          <t>Order time 07:00: still last (Customer Code first)</t>
+          <t>Priority 15-Oct: after all 14-Oct lines (unit 15-Oct, SORT_SEQ 1)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="45" t="inlineStr">
         <is>
-          <t>1b. XD09 read order: ORDER BY Part, Allocation Priority (= Order Date), PK columns</t>
+          <t>2. [Search] 15-Oct (PO1 20 pcs) → XD09: SORT_SEQ, cases, blocks</t>
         </is>
       </c>
       <c r="B19" s="46" t="n"/>
@@ -15877,1108 +15877,912 @@
     <row r="20">
       <c r="A20" s="35" t="inlineStr">
         <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+          <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
       <c r="D20" s="47" t="inlineStr">
         <is>
-          <t>Replicated from DB Surrounding (G-System)</t>
+          <t>Temporary (session)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>SORT_SEQ</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>CUSTOMER_CD</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
-        <is>
-          <t>ORDER_DT</t>
-        </is>
-      </c>
-      <c r="E21" s="42" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>DESTINATION_CD</t>
         </is>
       </c>
-      <c r="F21" s="42" t="inlineStr">
-        <is>
-          <t>DETAILED_ITEM_NO</t>
-        </is>
-      </c>
-      <c r="G21" s="42" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>OPEN_ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>ASSIGNED_QTY</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>CUM_DEST_QTY</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>CUT_FLAG</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>GROUP_SEQ</t>
+        </is>
+      </c>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>CROSSDOCK_STATUS</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B22" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D22" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E22" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F22" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G22" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I22" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M22" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O22" s="64" t="inlineStr">
+        <is>
+          <t>SORT_SEQ 1 = 9715300 / A-0101 / item 001</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B23" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D23" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E23" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F23" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G23" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="H23" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I23" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="L23" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M23" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N23" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O23" s="64" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D24" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E24" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F24" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="L24" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N24" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O24" s="64" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B25" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="64" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="D25" s="64" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="E25" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F25" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G25" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I25" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L25" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M25" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N25" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O25" s="64" t="inlineStr">
+        <is>
+          <t>Case 2 = VN 2 + VN 2 + TH 2: no cut (VN 10, TH 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B26" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="64" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="D26" s="64" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="E26" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F26" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G26" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I26" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J26" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L26" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M26" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N26" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O26" s="64" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B27" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D27" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E27" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F27" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G27" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H27" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I27" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="L27" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M27" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N27" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O27" s="64" t="inlineStr">
+        <is>
+          <t>Cut: VN 12, TH 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B28" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D28" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E28" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F28" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G28" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H28" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I28" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="K28" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="L28" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M28" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="N28" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O28" s="64" t="inlineStr">
+        <is>
+          <t>Case 4: only 2 of 6 pcs with PO1 → block 3 Not Ready, block 4 too</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B29" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D29" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E29" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F29" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G29" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H29" s="64" t="n"/>
+      <c r="I29" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J29" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" s="63" t="n">
+        <v>18</v>
+      </c>
+      <c r="L29" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M29" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="N29" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O29" s="64" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B30" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D30" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E30" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F30" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G30" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H30" s="64" t="n"/>
+      <c r="I30" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J30" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="K30" s="63" t="n">
+        <v>24</v>
+      </c>
+      <c r="L30" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M30" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="N30" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O30" s="64" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="45" t="inlineStr">
+        <is>
+          <t>3. Supplier chooses option 1 case → [Create ASN]</t>
+        </is>
+      </c>
+      <c r="B32" s="46" t="n"/>
+      <c r="C32" s="46" t="n"/>
+      <c r="D32" s="46" t="n"/>
+      <c r="E32" s="46" t="n"/>
+      <c r="F32" s="46" t="n"/>
+      <c r="G32" s="46" t="n"/>
+      <c r="H32" s="46" t="n"/>
+      <c r="I32" s="46" t="n"/>
+      <c r="J32" s="46" t="n"/>
+      <c r="K32" s="46" t="n"/>
+      <c r="L32" s="46" t="n"/>
+      <c r="M32" s="46" t="n"/>
+      <c r="N32" s="46" t="n"/>
+      <c r="O32" s="46" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>SERIAL_NO</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>SHIPPING_PART_NO</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS_QTY</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>HOLD_FLAG</t>
-        </is>
-      </c>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>PO_MAPPED_FLAG</t>
-        </is>
-      </c>
-      <c r="M21" s="5" t="inlineStr">
-        <is>
-          <t>CANCEL_STATUS</t>
-        </is>
-      </c>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="50" t="inlineStr">
-        <is>
-          <t>READ</t>
-        </is>
-      </c>
-      <c r="B22" s="51" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C22" s="51" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B35" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="49" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="F35" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G35" s="49" t="inlineStr">
         <is>
           <t>A-0101</t>
         </is>
       </c>
-      <c r="D22" s="51" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E22" s="51" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F22" s="51" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G22" s="51" t="inlineStr">
+      <c r="H35" s="49" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H22" s="51" t="inlineStr">
+      <c r="I35" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J35" s="49" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="K35" s="49" t="inlineStr">
+        <is>
+          <t>3126035921</t>
+        </is>
+      </c>
+      <c r="L35" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M35" s="49" t="n"/>
+      <c r="N35" s="49" t="n"/>
+      <c r="O35" s="49" t="inlineStr">
+        <is>
+          <t>Item 001: 6 of 8, open 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B38" s="42" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="C38" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="D38" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>MAPPED_QTY</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="C39" s="49" t="inlineStr">
+        <is>
+          <t>3126035921</t>
+        </is>
+      </c>
+      <c r="D39" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="E39" s="49" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="I22" s="52" t="n">
-        <v>8</v>
-      </c>
-      <c r="J22" s="51" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K22" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L22" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M22" s="51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N22" s="51" t="inlineStr">
-        <is>
-          <t>Priority 14-Oct · SORT_SEQ 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="50" t="inlineStr">
-        <is>
-          <t>READ</t>
-        </is>
-      </c>
-      <c r="B23" s="51" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C23" s="51" t="inlineStr">
-        <is>
-          <t>A-0101</t>
-        </is>
-      </c>
-      <c r="D23" s="51" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E23" s="51" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F23" s="51" t="inlineStr">
-        <is>
-          <t>002</t>
-        </is>
-      </c>
-      <c r="G23" s="51" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H23" s="51" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="I23" s="52" t="n">
-        <v>2</v>
-      </c>
-      <c r="J23" s="51" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K23" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L23" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M23" s="51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N23" s="51" t="inlineStr">
-        <is>
-          <t>Priority 14-Oct · SORT_SEQ 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="50" t="inlineStr">
-        <is>
-          <t>READ</t>
-        </is>
-      </c>
-      <c r="B24" s="51" t="inlineStr">
-        <is>
-          <t>9722D00</t>
-        </is>
-      </c>
-      <c r="C24" s="51" t="inlineStr">
-        <is>
-          <t>B-0102</t>
-        </is>
-      </c>
-      <c r="D24" s="51" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E24" s="51" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F24" s="51" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G24" s="51" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H24" s="51" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="I24" s="52" t="n">
+      <c r="F39" s="53" t="n">
+        <v>20</v>
+      </c>
+      <c r="G39" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="J24" s="51" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K24" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L24" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M24" s="51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N24" s="51" t="inlineStr">
-        <is>
-          <t>Priority 14-Oct · SORT_SEQ 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="50" t="inlineStr">
-        <is>
-          <t>READ</t>
-        </is>
-      </c>
-      <c r="B25" s="51" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="C25" s="51" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="D25" s="51" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E25" s="51" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F25" s="51" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G25" s="51" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H25" s="51" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="I25" s="52" t="n">
-        <v>14</v>
-      </c>
-      <c r="J25" s="51" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K25" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L25" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M25" s="51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N25" s="51" t="inlineStr">
-        <is>
-          <t>Priority 14-Oct · SORT_SEQ 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="50" t="inlineStr">
-        <is>
-          <t>READ</t>
-        </is>
-      </c>
-      <c r="B26" s="51" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C26" s="51" t="inlineStr">
-        <is>
-          <t>A-0201</t>
-        </is>
-      </c>
-      <c r="D26" s="51" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E26" s="51" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F26" s="51" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G26" s="51" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H26" s="51" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="I26" s="52" t="n">
-        <v>6</v>
-      </c>
-      <c r="J26" s="51" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K26" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L26" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M26" s="51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N26" s="51" t="inlineStr">
-        <is>
-          <t>Priority 15-Oct: after all 14-Oct lines (unit 15-Oct, SORT_SEQ 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="45" t="inlineStr">
-        <is>
-          <t>2. [Search] 15-Oct (PO1 20 pcs) → XD09: SORT_SEQ, cases, blocks</t>
-        </is>
-      </c>
-      <c r="B28" s="46" t="n"/>
-      <c r="C28" s="46" t="n"/>
-      <c r="D28" s="46" t="n"/>
-      <c r="E28" s="46" t="n"/>
-      <c r="F28" s="46" t="n"/>
-      <c r="G28" s="46" t="n"/>
-      <c r="H28" s="46" t="n"/>
-      <c r="I28" s="46" t="n"/>
-      <c r="J28" s="46" t="n"/>
-      <c r="K28" s="46" t="n"/>
-      <c r="L28" s="46" t="n"/>
-      <c r="M28" s="46" t="n"/>
-      <c r="N28" s="46" t="n"/>
-      <c r="O28" s="46" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="35" t="inlineStr">
-        <is>
-          <t>#TEMP_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D29" s="47" t="inlineStr">
-        <is>
-          <t>Temporary (session)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>SORT_SEQ</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>OPEN_ORDER_QTY</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="I30" s="9" t="inlineStr">
-        <is>
-          <t>ASSIGNED_QTY</t>
-        </is>
-      </c>
-      <c r="J30" s="9" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="K30" s="9" t="inlineStr">
-        <is>
-          <t>CUM_DEST_QTY</t>
-        </is>
-      </c>
-      <c r="L30" s="9" t="inlineStr">
-        <is>
-          <t>CUT_FLAG</t>
-        </is>
-      </c>
-      <c r="M30" s="9" t="inlineStr">
-        <is>
-          <t>GROUP_SEQ</t>
-        </is>
-      </c>
-      <c r="N30" s="9" t="inlineStr">
-        <is>
-          <t>CROSSDOCK_STATUS</t>
-        </is>
-      </c>
-      <c r="O30" s="9" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B31" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" s="64" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="D31" s="64" t="inlineStr">
-        <is>
-          <t>A-0101</t>
-        </is>
-      </c>
-      <c r="E31" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F31" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G31" s="63" t="n">
-        <v>8</v>
-      </c>
-      <c r="H31" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I31" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="J31" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="K31" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="L31" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M31" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="N31" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O31" s="64" t="inlineStr">
-        <is>
-          <t>SORT_SEQ 1 = 9715300 / A-0101 / item 001</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B32" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="64" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="D32" s="64" t="inlineStr">
-        <is>
-          <t>A-0101</t>
-        </is>
-      </c>
-      <c r="E32" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F32" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G32" s="63" t="n">
-        <v>8</v>
-      </c>
-      <c r="H32" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I32" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J32" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="K32" s="63" t="n">
-        <v>8</v>
-      </c>
-      <c r="L32" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M32" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="N32" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O32" s="64" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B33" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="C33" s="64" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="D33" s="64" t="inlineStr">
-        <is>
-          <t>A-0101</t>
-        </is>
-      </c>
-      <c r="E33" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F33" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G33" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I33" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J33" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="K33" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="L33" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M33" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="N33" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O33" s="64" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B34" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="C34" s="64" t="inlineStr">
-        <is>
-          <t>9722D00</t>
-        </is>
-      </c>
-      <c r="D34" s="64" t="inlineStr">
-        <is>
-          <t>B-0102</t>
-        </is>
-      </c>
-      <c r="E34" s="64" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F34" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G34" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="H34" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I34" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J34" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="K34" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="L34" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M34" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="N34" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O34" s="64" t="inlineStr">
-        <is>
-          <t>Case 2 = VN 2 + VN 2 + TH 2: no cut (VN 10, TH 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B35" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="C35" s="64" t="inlineStr">
-        <is>
-          <t>9722D00</t>
-        </is>
-      </c>
-      <c r="D35" s="64" t="inlineStr">
-        <is>
-          <t>B-0102</t>
-        </is>
-      </c>
-      <c r="E35" s="64" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F35" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G35" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="H35" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I35" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="J35" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="K35" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="L35" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M35" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="N35" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O35" s="64" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B36" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C36" s="64" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="D36" s="64" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="E36" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F36" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G36" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="H36" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I36" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J36" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="K36" s="63" t="n">
-        <v>12</v>
-      </c>
-      <c r="L36" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M36" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="N36" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O36" s="64" t="inlineStr">
-        <is>
-          <t>Cut: VN 12, TH 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B37" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C37" s="64" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="D37" s="64" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="E37" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F37" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G37" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="H37" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I37" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J37" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="K37" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="L37" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M37" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="N37" s="66" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="O37" s="64" t="inlineStr">
-        <is>
-          <t>Case 4: only 2 of 6 pcs with PO1 → block 3 Not Ready, block 4 too</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B38" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C38" s="64" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="D38" s="64" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="E38" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F38" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G38" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="H38" s="64" t="n"/>
-      <c r="I38" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="J38" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="K38" s="63" t="n">
-        <v>18</v>
-      </c>
-      <c r="L38" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M38" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="N38" s="66" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="O38" s="64" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B39" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C39" s="64" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="D39" s="64" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="E39" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F39" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G39" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="H39" s="64" t="n"/>
-      <c r="I39" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="J39" s="63" t="n">
-        <v>5</v>
-      </c>
-      <c r="K39" s="63" t="n">
-        <v>24</v>
-      </c>
-      <c r="L39" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M39" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="N39" s="66" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="O39" s="64" t="inlineStr"/>
+      <c r="H39" s="49" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="45" t="inlineStr">
         <is>
-          <t>3. Supplier chooses option 1 case → [Create ASN]</t>
+          <t>4. [Search] 16-Oct (PO1 open 14 + PO2 10) → open qty cut again from case 1</t>
         </is>
       </c>
       <c r="B41" s="46" t="n"/>
@@ -16999,903 +16803,644 @@
     <row r="42">
       <c r="A42" s="35" t="inlineStr">
         <is>
-          <t>TB_R_INSTRUCTION</t>
+          <t>#TEMP_INSTRUCTION</t>
         </is>
       </c>
       <c r="D42" s="47" t="inlineStr">
         <is>
-          <t>New table (Crossdock)</t>
+          <t>Temporary (session)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B43" s="42" t="inlineStr">
-        <is>
-          <t>INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>SORT_SEQ</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>OPEN_ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="I43" s="9" t="inlineStr">
+        <is>
+          <t>ASSIGNED_QTY</t>
+        </is>
+      </c>
+      <c r="J43" s="9" t="inlineStr">
         <is>
           <t>CASE_SEQ</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>LINE_SEQ</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="K43" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="L43" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="M43" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="N43" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
-        </is>
-      </c>
-      <c r="O43" s="3" t="inlineStr">
+      <c r="K43" s="9" t="inlineStr">
+        <is>
+          <t>CUM_DEST_QTY</t>
+        </is>
+      </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>CUT_FLAG</t>
+        </is>
+      </c>
+      <c r="M43" s="9" t="inlineStr">
+        <is>
+          <t>GROUP_SEQ</t>
+        </is>
+      </c>
+      <c r="N43" s="9" t="inlineStr">
+        <is>
+          <t>CROSSDOCK_STATUS</t>
+        </is>
+      </c>
+      <c r="O43" s="9" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B44" s="53" t="n">
+      <c r="A44" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B44" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="C44" s="53" t="n">
+      <c r="C44" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D44" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E44" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F44" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G44" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I44" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J44" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="D44" s="53" t="n">
+      <c r="K44" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L44" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M44" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="E44" s="49" t="inlineStr">
+      <c r="N44" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O44" s="64" t="inlineStr">
+        <is>
+          <t>Open qty 8 - 6 = 2; case 1 = the same physical case as case 2 on 15-Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B45" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D45" s="64" t="inlineStr">
+        <is>
+          <t>A-0101</t>
+        </is>
+      </c>
+      <c r="E45" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F45" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="F44" s="49" t="inlineStr">
+      <c r="G45" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I45" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J45" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="L45" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M45" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N45" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O45" s="64" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B46" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" s="64" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="D46" s="64" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="E46" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F46" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G46" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H46" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I46" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J46" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L46" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M46" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N46" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O46" s="64" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B47" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" s="64" t="inlineStr">
+        <is>
+          <t>9722D00</t>
+        </is>
+      </c>
+      <c r="D47" s="64" t="inlineStr">
+        <is>
+          <t>B-0102</t>
+        </is>
+      </c>
+      <c r="E47" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F47" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G47" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H47" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I47" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J47" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K47" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L47" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M47" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N47" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O47" s="64" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B48" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C48" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D48" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E48" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="G44" s="49" t="inlineStr">
-        <is>
-          <t>A-0101</t>
-        </is>
-      </c>
-      <c r="H44" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="I44" s="53" t="n">
+      <c r="F48" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G48" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H48" s="64" t="inlineStr">
+        <is>
+          <t>T0409021</t>
+        </is>
+      </c>
+      <c r="I48" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J48" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="J44" s="49" t="inlineStr">
+      <c r="L48" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M48" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N48" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O48" s="64" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B49" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D49" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E49" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F49" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G49" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H49" s="64" t="inlineStr">
         <is>
           <t>T0409021</t>
         </is>
       </c>
-      <c r="K44" s="49" t="inlineStr">
-        <is>
-          <t>3126035921</t>
-        </is>
-      </c>
-      <c r="L44" s="49" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="M44" s="49" t="n"/>
-      <c r="N44" s="49" t="n"/>
-      <c r="O44" s="49" t="inlineStr">
-        <is>
-          <t>Item 001: 6 of 8, open 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
-        </is>
-      </c>
-      <c r="D46" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="26" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B47" s="42" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="C47" s="42" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="D47" s="42" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>ORDER_QTY</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>MAPPED_QTY</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B48" s="49" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="C48" s="49" t="inlineStr">
-        <is>
-          <t>3126035921</t>
-        </is>
-      </c>
-      <c r="D48" s="49" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="E48" s="49" t="inlineStr">
+      <c r="I49" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J49" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K49" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="L49" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M49" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N49" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O49" s="64" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B50" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D50" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E50" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F50" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="F48" s="53" t="n">
-        <v>20</v>
-      </c>
-      <c r="G48" s="53" t="n">
+      <c r="G50" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H50" s="64" t="inlineStr">
+        <is>
+          <t>T0410021</t>
+        </is>
+      </c>
+      <c r="I50" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J50" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="L50" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M50" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N50" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O50" s="64" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B51" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C51" s="64" t="inlineStr">
+        <is>
+          <t>9730000</t>
+        </is>
+      </c>
+      <c r="D51" s="64" t="inlineStr">
+        <is>
+          <t>C-0103</t>
+        </is>
+      </c>
+      <c r="E51" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F51" s="64" t="inlineStr">
+        <is>
+          <t>PART-B</t>
+        </is>
+      </c>
+      <c r="G51" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H51" s="64" t="inlineStr">
+        <is>
+          <t>T0410021</t>
+        </is>
+      </c>
+      <c r="I51" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="H48" s="49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="45" t="inlineStr">
-        <is>
-          <t>4. [Search] 16-Oct (PO1 open 14 + PO2 10) → open qty cut again from case 1</t>
-        </is>
-      </c>
-      <c r="B50" s="46" t="n"/>
-      <c r="C50" s="46" t="n"/>
-      <c r="D50" s="46" t="n"/>
-      <c r="E50" s="46" t="n"/>
-      <c r="F50" s="46" t="n"/>
-      <c r="G50" s="46" t="n"/>
-      <c r="H50" s="46" t="n"/>
-      <c r="I50" s="46" t="n"/>
-      <c r="J50" s="46" t="n"/>
-      <c r="K50" s="46" t="n"/>
-      <c r="L50" s="46" t="n"/>
-      <c r="M50" s="46" t="n"/>
-      <c r="N50" s="46" t="n"/>
-      <c r="O50" s="46" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="35" t="inlineStr">
-        <is>
-          <t>#TEMP_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D51" s="47" t="inlineStr">
-        <is>
-          <t>Temporary (session)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="26" customHeight="1">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>SORT_SEQ</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>OPEN_ORDER_QTY</t>
-        </is>
-      </c>
-      <c r="H52" s="9" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="I52" s="9" t="inlineStr">
-        <is>
-          <t>ASSIGNED_QTY</t>
-        </is>
-      </c>
-      <c r="J52" s="9" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="K52" s="9" t="inlineStr">
-        <is>
-          <t>CUM_DEST_QTY</t>
-        </is>
-      </c>
-      <c r="L52" s="9" t="inlineStr">
-        <is>
-          <t>CUT_FLAG</t>
-        </is>
-      </c>
-      <c r="M52" s="9" t="inlineStr">
-        <is>
-          <t>GROUP_SEQ</t>
-        </is>
-      </c>
-      <c r="N52" s="9" t="inlineStr">
-        <is>
-          <t>CROSSDOCK_STATUS</t>
-        </is>
-      </c>
-      <c r="O52" s="9" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="62" t="inlineStr">
+      <c r="J51" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="K51" s="63" t="n">
+        <v>18</v>
+      </c>
+      <c r="L51" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M51" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="N51" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O51" s="64" t="inlineStr">
+        <is>
+          <t>Unit 14-Oct: all 3 blocks Ready (options 2 / 3 / 4 cases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="62" t="inlineStr">
         <is>
           <t>TEMP</t>
         </is>
       </c>
-      <c r="B53" s="63" t="n">
+      <c r="B52" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="C53" s="64" t="inlineStr">
+      <c r="C52" s="64" t="inlineStr">
         <is>
           <t>9715300</t>
         </is>
       </c>
-      <c r="D53" s="64" t="inlineStr">
-        <is>
-          <t>A-0101</t>
-        </is>
-      </c>
-      <c r="E53" s="64" t="inlineStr">
+      <c r="D52" s="64" t="inlineStr">
+        <is>
+          <t>A-0201</t>
+        </is>
+      </c>
+      <c r="E52" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F53" s="64" t="inlineStr">
+      <c r="F52" s="64" t="inlineStr">
         <is>
           <t>PART-B</t>
         </is>
       </c>
-      <c r="G53" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="H53" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I53" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J53" s="63" t="n">
+      <c r="G52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H52" s="64" t="n"/>
+      <c r="I52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J52" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="K53" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="L53" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M53" s="63" t="n">
+      <c r="K52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L52" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M52" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="N53" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O53" s="64" t="inlineStr">
-        <is>
-          <t>Open qty 8 - 6 = 2; case 1 = the same physical case as case 2 on 15-Oct</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B54" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="C54" s="64" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="D54" s="64" t="inlineStr">
-        <is>
-          <t>A-0101</t>
-        </is>
-      </c>
-      <c r="E54" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F54" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G54" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="H54" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I54" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J54" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="K54" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="L54" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M54" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="N54" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O54" s="64" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B55" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="C55" s="64" t="inlineStr">
-        <is>
-          <t>9722D00</t>
-        </is>
-      </c>
-      <c r="D55" s="64" t="inlineStr">
-        <is>
-          <t>B-0102</t>
-        </is>
-      </c>
-      <c r="E55" s="64" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F55" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G55" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="H55" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I55" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J55" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="K55" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="L55" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M55" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="N55" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O55" s="64" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B56" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="C56" s="64" t="inlineStr">
-        <is>
-          <t>9722D00</t>
-        </is>
-      </c>
-      <c r="D56" s="64" t="inlineStr">
-        <is>
-          <t>B-0102</t>
-        </is>
-      </c>
-      <c r="E56" s="64" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F56" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G56" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="H56" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I56" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="J56" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="K56" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="L56" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M56" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="N56" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O56" s="64" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B57" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C57" s="64" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="D57" s="64" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="E57" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F57" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G57" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="H57" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I57" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J57" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="K57" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="L57" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M57" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="N57" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O57" s="64" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B58" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C58" s="64" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="D58" s="64" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="E58" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F58" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G58" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="H58" s="64" t="inlineStr">
-        <is>
-          <t>T0409021</t>
-        </is>
-      </c>
-      <c r="I58" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J58" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="K58" s="63" t="n">
-        <v>8</v>
-      </c>
-      <c r="L58" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M58" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="N58" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O58" s="64" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B59" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C59" s="64" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="D59" s="64" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="E59" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F59" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G59" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="H59" s="64" t="inlineStr">
-        <is>
-          <t>T0410021</t>
-        </is>
-      </c>
-      <c r="I59" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="J59" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="K59" s="63" t="n">
-        <v>12</v>
-      </c>
-      <c r="L59" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M59" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="N59" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O59" s="64" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B60" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C60" s="64" t="inlineStr">
-        <is>
-          <t>9730000</t>
-        </is>
-      </c>
-      <c r="D60" s="64" t="inlineStr">
-        <is>
-          <t>C-0103</t>
-        </is>
-      </c>
-      <c r="E60" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F60" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G60" s="63" t="n">
-        <v>14</v>
-      </c>
-      <c r="H60" s="64" t="inlineStr">
-        <is>
-          <t>T0410021</t>
-        </is>
-      </c>
-      <c r="I60" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="J60" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="K60" s="63" t="n">
-        <v>18</v>
-      </c>
-      <c r="L60" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M60" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="N60" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="O60" s="64" t="inlineStr">
-        <is>
-          <t>Unit 14-Oct: all 3 blocks Ready (options 2 / 3 / 4 cases)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B61" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="C61" s="64" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="D61" s="64" t="inlineStr">
-        <is>
-          <t>A-0201</t>
-        </is>
-      </c>
-      <c r="E61" s="64" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F61" s="64" t="inlineStr">
-        <is>
-          <t>PART-B</t>
-        </is>
-      </c>
-      <c r="G61" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="H61" s="64" t="n"/>
-      <c r="I61" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="J61" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="K61" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="L61" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M61" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="N61" s="66" t="inlineStr">
+      <c r="N52" s="66" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="O61" s="64" t="inlineStr">
+      <c r="O52" s="64" t="inlineStr">
         <is>
           <t>Unit 15-Oct after unit 14-Oct (way B): no PO left</t>
         </is>
@@ -34922,7 +34467,7 @@
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>PART-B, 6 pcs/case. Scan order = G-System allocation order with Allocation Priority = Customer Order Date: 1) Allocation Priority, 2) Customer Code, 3) Customer Order No, 4) Order Date, 5) Order Time, 6) Destination, 7) Detailed Item No, 8) Serial No. Keys 2-8 are the PK of the H0253 replicate; XD09 reads with ORDER BY Part, Allocation Priority + the PK columns (query in XD09 Appendix). SORT_SEQ = row number per unit. Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. A-0201 (15-Oct) is in the middle of the PK order but after all 14-Oct lines in the scan order (Allocation Priority). 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only. 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
+          <t>PART-B, 6 pcs/case. Scan order = G-System allocation order with Allocation Priority = Customer Order Date: 1) Allocation Priority, 2) Customer Code, 3) Customer Order No, 4) Order Date, 5) Order Time, 6) Destination, 7) Detailed Item No, 8) Serial No. Keys 2-8 are the PK of the H0253 replicate; XD09 reads with ORDER BY Part, Allocation Priority + the PK columns (query in XD09 Appendix). SORT_SEQ = row number per unit. Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. A-0201 (15-Oct) comes after all 14-Oct lines (Allocation Priority) and is the next unit. 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only. 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
XD10: check box per supplier case ending on CUT_FLAG Y (MSG10), sample H / I; ERD SIM-9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-6" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-7" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-8" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-9" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Column Definition'!$A$3:$H$468</definedName>
@@ -17573,6 +17574,1485 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:P37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SIM-9 XD10 case check boxes: cases 1-2 not possible, 1-3 sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="33" t="inlineStr">
+        <is>
+          <t>BPF F2 · Functions: XD09, XD10 (Select case, Create ASN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="34" t="inlineStr">
+        <is>
+          <t>• Same unit as SIM-7 (PART-A 14-Oct: V01 VN 10, T01 TH 6, V02 VN 14; 6 pcs/case) but all 5 cases have a PO (p1 24 + p2 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>• XD10 shows one check box per supplier case. The supplier wants cases 1 and 2 only: case 2 = VN 4 + TH 2 ends with VN 10 / TH 2 (CUT_FLAG N), so the warehouse could not close the VN and TH cases. XD10 ticks case 3 too (message no. 10): cases 1-3 = 18 pcs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>• [Create ASN] inserts the slices of cases 1-3; V01 and T01 are complete (PO_MAPPED_FLAG Y), V02 keeps 12 pcs open for a later ASN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>NEW row</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>UPD row</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>DEL row</t>
+        </is>
+      </c>
+      <c r="E7" s="39" t="inlineStr">
+        <is>
+          <t>READ row</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="inlineStr">
+        <is>
+          <t>TEMP row</t>
+        </is>
+      </c>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>Changed cell</t>
+        </is>
+      </c>
+      <c r="H7" s="42" t="inlineStr">
+        <is>
+          <t>PK column</t>
+        </is>
+      </c>
+      <c r="I7" s="36" t="inlineStr">
+        <is>
+          <t>Status OK</t>
+        </is>
+      </c>
+      <c r="J7" s="43" t="inlineStr">
+        <is>
+          <t>Status attention</t>
+        </is>
+      </c>
+      <c r="K7" s="44" t="inlineStr">
+        <is>
+          <t>Status NG / cancel</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="45" t="inlineStr">
+        <is>
+          <t>1. [Search] → XD09: all cases with PO; CUT_FLAG Y after cases 1, 3, 4, 5</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="n"/>
+      <c r="C9" s="46" t="n"/>
+      <c r="D9" s="46" t="n"/>
+      <c r="E9" s="46" t="n"/>
+      <c r="F9" s="46" t="n"/>
+      <c r="G9" s="46" t="n"/>
+      <c r="H9" s="46" t="n"/>
+      <c r="I9" s="46" t="n"/>
+      <c r="J9" s="46" t="n"/>
+      <c r="K9" s="46" t="n"/>
+      <c r="L9" s="46" t="n"/>
+      <c r="M9" s="46" t="n"/>
+      <c r="N9" s="46" t="n"/>
+      <c r="O9" s="46" t="n"/>
+      <c r="P9" s="46" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>#TEMP_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D10" s="47" t="inlineStr">
+        <is>
+          <t>Temporary (session)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>SORT_SEQ</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>OPEN_ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>ASSIGNED_QTY</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>CUM_DEST_QTY</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>SEQ_QTY</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>CUT_FLAG</t>
+        </is>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>GROUP_SEQ</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>CROSSDOCK_STATUS</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B12" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="64" t="inlineStr">
+        <is>
+          <t>CUST-A</t>
+        </is>
+      </c>
+      <c r="D12" s="64" t="inlineStr">
+        <is>
+          <t>V01</t>
+        </is>
+      </c>
+      <c r="E12" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F12" s="64" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="G12" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="H12" s="64" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="I12" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M12" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P12" s="64" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B13" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="64" t="inlineStr">
+        <is>
+          <t>CUST-A</t>
+        </is>
+      </c>
+      <c r="D13" s="64" t="inlineStr">
+        <is>
+          <t>V01</t>
+        </is>
+      </c>
+      <c r="E13" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F13" s="64" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="G13" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" s="64" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="I13" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J13" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="L13" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="M13" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P13" s="64" t="inlineStr">
+        <is>
+          <t>Case 2 = VN 4 + TH 2: CUT N (VN 10, TH 2) → cannot be the last case</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="64" t="inlineStr">
+        <is>
+          <t>CUST-B</t>
+        </is>
+      </c>
+      <c r="D14" s="64" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="E14" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F14" s="64" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="G14" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" s="64" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="I14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O14" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P14" s="64" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="64" t="inlineStr">
+        <is>
+          <t>CUST-B</t>
+        </is>
+      </c>
+      <c r="D15" s="64" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="E15" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F15" s="64" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="G15" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" s="64" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="I15" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L15" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M15" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O15" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P15" s="64" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="64" t="inlineStr">
+        <is>
+          <t>CUST-C</t>
+        </is>
+      </c>
+      <c r="D16" s="64" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
+      <c r="E16" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F16" s="64" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="G16" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H16" s="64" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="I16" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="L16" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M16" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O16" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P16" s="64" t="inlineStr">
+        <is>
+          <t>Case 3: CUT Y (VN 12, TH 6) → ticked together with case 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="64" t="inlineStr">
+        <is>
+          <t>CUST-C</t>
+        </is>
+      </c>
+      <c r="D17" s="64" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
+      <c r="E17" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F17" s="64" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="G17" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H17" s="64" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="I17" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" s="63" t="n">
+        <v>18</v>
+      </c>
+      <c r="L17" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M17" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P17" s="64" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B18" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="64" t="inlineStr">
+        <is>
+          <t>CUST-C</t>
+        </is>
+      </c>
+      <c r="D18" s="64" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
+      <c r="E18" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F18" s="64" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="G18" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H18" s="64" t="inlineStr">
+        <is>
+          <t>T0410011</t>
+        </is>
+      </c>
+      <c r="I18" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="K18" s="63" t="n">
+        <v>24</v>
+      </c>
+      <c r="L18" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M18" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="O18" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P18" s="64" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="45" t="inlineStr">
+        <is>
+          <t>2. Supplier ticks cases 1-2 → XD10 ticks case 3 too (MSG10) → [Create ASN] cases 1-3</t>
+        </is>
+      </c>
+      <c r="B20" s="46" t="n"/>
+      <c r="C20" s="46" t="n"/>
+      <c r="D20" s="46" t="n"/>
+      <c r="E20" s="46" t="n"/>
+      <c r="F20" s="46" t="n"/>
+      <c r="G20" s="46" t="n"/>
+      <c r="H20" s="46" t="n"/>
+      <c r="I20" s="46" t="n"/>
+      <c r="J20" s="46" t="n"/>
+      <c r="K20" s="46" t="n"/>
+      <c r="L20" s="46" t="n"/>
+      <c r="M20" s="46" t="n"/>
+      <c r="N20" s="46" t="n"/>
+      <c r="O20" s="46" t="n"/>
+      <c r="P20" s="46" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D21" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B23" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="49" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="F23" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G23" s="49" t="inlineStr">
+        <is>
+          <t>V01</t>
+        </is>
+      </c>
+      <c r="H23" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I23" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J23" s="49" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="K23" s="49" t="inlineStr">
+        <is>
+          <t>3126035911</t>
+        </is>
+      </c>
+      <c r="L23" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M23" s="49" t="n"/>
+      <c r="N23" s="49" t="n"/>
+      <c r="O23" s="49" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B24" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="49" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="F24" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G24" s="49" t="inlineStr">
+        <is>
+          <t>V01</t>
+        </is>
+      </c>
+      <c r="H24" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I24" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="J24" s="49" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="K24" s="49" t="inlineStr">
+        <is>
+          <t>3126035911</t>
+        </is>
+      </c>
+      <c r="L24" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M24" s="49" t="n"/>
+      <c r="N24" s="49" t="n"/>
+      <c r="O24" s="49" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B25" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="49" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="F25" s="49" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="G25" s="49" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="H25" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I25" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" s="49" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="K25" s="49" t="inlineStr">
+        <is>
+          <t>3126035911</t>
+        </is>
+      </c>
+      <c r="L25" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M25" s="49" t="n"/>
+      <c r="N25" s="49" t="n"/>
+      <c r="O25" s="49" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B26" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="49" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="F26" s="49" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="G26" s="49" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="H26" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I26" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="J26" s="49" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="K26" s="49" t="inlineStr">
+        <is>
+          <t>3126035911</t>
+        </is>
+      </c>
+      <c r="L26" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M26" s="49" t="n"/>
+      <c r="N26" s="49" t="n"/>
+      <c r="O26" s="49" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B27" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="49" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="F27" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G27" s="49" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
+      <c r="H27" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I27" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="49" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="K27" s="49" t="inlineStr">
+        <is>
+          <t>3126035911</t>
+        </is>
+      </c>
+      <c r="L27" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M27" s="49" t="n"/>
+      <c r="N27" s="49" t="n"/>
+      <c r="O27" s="49" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
+        </is>
+      </c>
+      <c r="D29" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="C30" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="D30" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>MAPPED_QTY</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>T0409011</t>
+        </is>
+      </c>
+      <c r="C31" s="49" t="inlineStr">
+        <is>
+          <t>3126035911</t>
+        </is>
+      </c>
+      <c r="D31" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="E31" s="49" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="F31" s="53" t="n">
+        <v>24</v>
+      </c>
+      <c r="G31" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="H31" s="49" t="inlineStr">
+        <is>
+          <t>18 of 24 used; 6 left for case 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C34" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D34" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E34" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F34" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G34" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>CANCEL_STATUS</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B35" s="58" t="inlineStr">
+        <is>
+          <t>CUST-A</t>
+        </is>
+      </c>
+      <c r="C35" s="58" t="inlineStr">
+        <is>
+          <t>V01</t>
+        </is>
+      </c>
+      <c r="D35" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E35" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F35" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G35" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H35" s="58" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="I35" s="59" t="n">
+        <v>10</v>
+      </c>
+      <c r="J35" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K35" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L35" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M35" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N35" s="58" t="inlineStr">
+        <is>
+          <t>Whole line in cases 1-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B36" s="58" t="inlineStr">
+        <is>
+          <t>CUST-B</t>
+        </is>
+      </c>
+      <c r="C36" s="58" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="D36" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E36" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F36" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G36" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H36" s="58" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="I36" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J36" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K36" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L36" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M36" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N36" s="58" t="inlineStr">
+        <is>
+          <t>Whole line in cases 2-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B37" s="51" t="inlineStr">
+        <is>
+          <t>CUST-C</t>
+        </is>
+      </c>
+      <c r="C37" s="51" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
+      <c r="D37" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E37" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F37" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G37" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H37" s="51" t="inlineStr">
+        <is>
+          <t>PART-A</t>
+        </is>
+      </c>
+      <c r="I37" s="52" t="n">
+        <v>14</v>
+      </c>
+      <c r="J37" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K37" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L37" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M37" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N37" s="51" t="inlineStr">
+        <is>
+          <t>2 of 14 sent: stays N, open qty 12 (cases 4-5 at the next Search)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -17895,7 +19375,7 @@
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8</t>
+          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -17955,7 +19435,7 @@
       </c>
       <c r="F14" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8</t>
+          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -17985,7 +19465,7 @@
       </c>
       <c r="F15" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-3, SIM-4, SIM-7, SIM-8</t>
+          <t>SIM-2, SIM-3, SIM-4, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -18075,7 +19555,7 @@
       </c>
       <c r="F18" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-5, SIM-6, SIM-7, SIM-8</t>
+          <t>SIM-2, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -34311,7 +35791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -34621,6 +36101,38 @@
       <c r="F12" s="32" t="inlineStr">
         <is>
           <t>PART-B, 6 pcs/case. Scan order = G-System allocation order with Allocation Priority = Customer Order Date: 1) Allocation Priority, 2) Customer Code, 3) Customer Order No, 4) Order Date, 5) Order Time, 6) Destination, 7) Detailed Item No, 8) Serial No. Keys 2-8 are the PK of the H0253 replicate; XD09 reads with ORDER BY Part, Allocation Priority + the PK columns (query in XD09 Appendix). SORT_SEQ = row number per unit. Unit 14-Oct: A-0101 item 001 VN 8 (seq 1), A-0101 item 002 VN 2 (seq 2), B-0102 TH 6 (seq 3), C-0103 VN 14 of a second VN customer 9730000 (seq 4). Order Time 07:00 of C-0103 does not move it up: Customer Code and Order No come first. A-0201 (15-Oct) comes after all 14-Oct lines (Allocation Priority) and is the next unit. 15-Oct: PO1 20 pcs → blocks 1-2 Ready, block 3 (case 4) only 2 of 6 pcs with PO → Not Ready. The supplier sends option 1 case only. 16-Oct: PO2 10 pcs. The open qty (24) is cut again from case 1 in the same SORT_SEQ: the cases are the same as before. Unit 15-Oct (A-0201) comes after unit 14-Oct (way B), so it gets no PO yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>SIM-9</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>XD10 case check boxes: cases 1-2 not possible, 1-3 sent</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>BPF F2</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>XD09, XD10 (Select case, Create ASN)</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>#TEMP_INSTRUCTION, TB_R_INSTRUCTION, TB_R_PRA_DAILY_ORDER_MAPPED, TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>Same unit as SIM-7 (PART-A 14-Oct: V01 VN 10, T01 TH 6, V02 VN 14; 6 pcs/case) but all 5 cases have a PO (p1 24 + p2 6). XD10 shows one check box per supplier case. The supplier wants cases 1 and 2 only: case 2 = VN 4 + TH 2 ends with VN 10 / TH 2 (CUT_FLAG N), so the warehouse could not close the VN and TH cases. XD10 ticks case 3 too (message no. 10): cases 1-3 = 18 pcs. [Create ASN] inserts the slices of cases 1-3; V01 and T01 are complete (PO_MAPPED_FLAG Y), V02 keeps 12 pcs open for a later ASN.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simulations: dummy PO No (PO-DMY-...) and Manifest No (MF-DMY-...)
ERD simulations, XD10 sample, XD09 / XD10 spec examples, discussion note and prototype data use
dummy PO / manifest numbers; screenshots, UISS XD10 / XD15 and BPF rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -10395,12 +10395,12 @@
       </c>
       <c r="J12" s="51" t="inlineStr">
         <is>
-          <t>T0409004</t>
+          <t>PO-DMY-09004</t>
         </is>
       </c>
       <c r="K12" s="51" t="inlineStr">
         <is>
-          <t>3126035904</t>
+          <t>MF-DMY-09004</t>
         </is>
       </c>
       <c r="L12" s="51" t="inlineStr">
@@ -10452,12 +10452,12 @@
       </c>
       <c r="J13" s="51" t="inlineStr">
         <is>
-          <t>T0409004</t>
+          <t>PO-DMY-09004</t>
         </is>
       </c>
       <c r="K13" s="51" t="inlineStr">
         <is>
-          <t>3126035904</t>
+          <t>MF-DMY-09004</t>
         </is>
       </c>
       <c r="L13" s="51" t="inlineStr">
@@ -10531,12 +10531,12 @@
       </c>
       <c r="B17" s="51" t="inlineStr">
         <is>
-          <t>T0409004</t>
+          <t>PO-DMY-09004</t>
         </is>
       </c>
       <c r="C17" s="51" t="inlineStr">
         <is>
-          <t>3126035904</t>
+          <t>MF-DMY-09004</t>
         </is>
       </c>
       <c r="D17" s="51" t="inlineStr">
@@ -10948,12 +10948,12 @@
       </c>
       <c r="J28" s="68" t="inlineStr">
         <is>
-          <t>T0409004</t>
+          <t>PO-DMY-09004</t>
         </is>
       </c>
       <c r="K28" s="68" t="inlineStr">
         <is>
-          <t>3126035904</t>
+          <t>MF-DMY-09004</t>
         </is>
       </c>
       <c r="L28" s="68" t="inlineStr">
@@ -11009,12 +11009,12 @@
       </c>
       <c r="J29" s="68" t="inlineStr">
         <is>
-          <t>T0409004</t>
+          <t>PO-DMY-09004</t>
         </is>
       </c>
       <c r="K29" s="68" t="inlineStr">
         <is>
-          <t>3126035904</t>
+          <t>MF-DMY-09004</t>
         </is>
       </c>
       <c r="L29" s="68" t="inlineStr">
@@ -11092,12 +11092,12 @@
       </c>
       <c r="B33" s="58" t="inlineStr">
         <is>
-          <t>T0409004</t>
+          <t>PO-DMY-09004</t>
         </is>
       </c>
       <c r="C33" s="58" t="inlineStr">
         <is>
-          <t>3126035904</t>
+          <t>MF-DMY-09004</t>
         </is>
       </c>
       <c r="D33" s="58" t="inlineStr">
@@ -11923,12 +11923,12 @@
       </c>
       <c r="J12" s="51" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="K12" s="51" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="L12" s="51" t="inlineStr">
@@ -12273,12 +12273,12 @@
       </c>
       <c r="J22" s="51" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="K22" s="51" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="L22" s="51" t="inlineStr">
@@ -12364,12 +12364,12 @@
       </c>
       <c r="B26" s="51" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="C26" s="51" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="D26" s="51" t="inlineStr">
@@ -13175,7 +13175,7 @@
       </c>
       <c r="B18" s="51" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="C18" s="51" t="inlineStr">
@@ -13185,7 +13185,7 @@
       </c>
       <c r="D18" s="51" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="E18" s="51" t="inlineStr">
@@ -13357,7 +13357,7 @@
       </c>
       <c r="H23" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I23" s="63" t="n">
@@ -13421,7 +13421,7 @@
       </c>
       <c r="H24" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I24" s="63" t="n">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="H25" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I25" s="63" t="n">
@@ -13553,7 +13553,7 @@
       </c>
       <c r="H26" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I26" s="63" t="n">
@@ -13617,7 +13617,7 @@
       </c>
       <c r="H27" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I27" s="63" t="n">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="H28" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I28" s="63" t="n">
@@ -13930,12 +13930,12 @@
       </c>
       <c r="J34" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K34" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L34" s="49" t="inlineStr">
@@ -13987,12 +13987,12 @@
       </c>
       <c r="J35" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K35" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L35" s="49" t="inlineStr">
@@ -14044,12 +14044,12 @@
       </c>
       <c r="J36" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K36" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L36" s="49" t="inlineStr">
@@ -14101,12 +14101,12 @@
       </c>
       <c r="J37" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K37" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L37" s="49" t="inlineStr">
@@ -14158,12 +14158,12 @@
       </c>
       <c r="J38" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K38" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L38" s="49" t="inlineStr">
@@ -14215,12 +14215,12 @@
       </c>
       <c r="J39" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K39" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L39" s="49" t="inlineStr">
@@ -14294,12 +14294,12 @@
       </c>
       <c r="B43" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="C43" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="D43" s="49" t="inlineStr">
@@ -14698,7 +14698,7 @@
       </c>
       <c r="B54" s="49" t="inlineStr">
         <is>
-          <t>3126036011</t>
+          <t>MF-DMY-10011</t>
         </is>
       </c>
       <c r="C54" s="49" t="inlineStr">
@@ -14708,7 +14708,7 @@
       </c>
       <c r="D54" s="49" t="inlineStr">
         <is>
-          <t>T0410011</t>
+          <t>PO-DMY-10011</t>
         </is>
       </c>
       <c r="E54" s="49" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="H59" s="64" t="inlineStr">
         <is>
-          <t>T0410011</t>
+          <t>PO-DMY-10011</t>
         </is>
       </c>
       <c r="I59" s="63" t="n">
@@ -15061,12 +15061,12 @@
       </c>
       <c r="J64" s="49" t="inlineStr">
         <is>
-          <t>T0410011</t>
+          <t>PO-DMY-10011</t>
         </is>
       </c>
       <c r="K64" s="49" t="inlineStr">
         <is>
-          <t>3126036011</t>
+          <t>MF-DMY-10011</t>
         </is>
       </c>
       <c r="L64" s="49" t="inlineStr">
@@ -15140,12 +15140,12 @@
       </c>
       <c r="B68" s="49" t="inlineStr">
         <is>
-          <t>T0410011</t>
+          <t>PO-DMY-10011</t>
         </is>
       </c>
       <c r="C68" s="49" t="inlineStr">
         <is>
-          <t>3126036011</t>
+          <t>MF-DMY-10011</t>
         </is>
       </c>
       <c r="D68" s="49" t="inlineStr">
@@ -16058,7 +16058,7 @@
       </c>
       <c r="H22" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I22" s="63" t="n">
@@ -16126,7 +16126,7 @@
       </c>
       <c r="H23" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I23" s="63" t="n">
@@ -16190,7 +16190,7 @@
       </c>
       <c r="H24" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I24" s="63" t="n">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="H25" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I25" s="63" t="n">
@@ -16322,7 +16322,7 @@
       </c>
       <c r="H26" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I26" s="63" t="n">
@@ -16386,7 +16386,7 @@
       </c>
       <c r="H27" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I27" s="63" t="n">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H28" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I28" s="63" t="n">
@@ -16759,12 +16759,12 @@
       </c>
       <c r="J35" s="49" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="K35" s="49" t="inlineStr">
         <is>
-          <t>3126035921</t>
+          <t>MF-DMY-09021</t>
         </is>
       </c>
       <c r="L35" s="49" t="inlineStr">
@@ -16842,12 +16842,12 @@
       </c>
       <c r="B39" s="49" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="C39" s="49" t="inlineStr">
         <is>
-          <t>3126035921</t>
+          <t>MF-DMY-09021</t>
         </is>
       </c>
       <c r="D39" s="49" t="inlineStr">
@@ -17018,7 +17018,7 @@
       </c>
       <c r="H44" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I44" s="63" t="n">
@@ -17086,7 +17086,7 @@
       </c>
       <c r="H45" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I45" s="63" t="n">
@@ -17150,7 +17150,7 @@
       </c>
       <c r="H46" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I46" s="63" t="n">
@@ -17214,7 +17214,7 @@
       </c>
       <c r="H47" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I47" s="63" t="n">
@@ -17278,7 +17278,7 @@
       </c>
       <c r="H48" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I48" s="63" t="n">
@@ -17342,7 +17342,7 @@
       </c>
       <c r="H49" s="64" t="inlineStr">
         <is>
-          <t>T0409021</t>
+          <t>PO-DMY-09021</t>
         </is>
       </c>
       <c r="I49" s="63" t="n">
@@ -17406,7 +17406,7 @@
       </c>
       <c r="H50" s="64" t="inlineStr">
         <is>
-          <t>T0410021</t>
+          <t>PO-DMY-10021</t>
         </is>
       </c>
       <c r="I50" s="63" t="n">
@@ -17470,7 +17470,7 @@
       </c>
       <c r="H51" s="64" t="inlineStr">
         <is>
-          <t>T0410021</t>
+          <t>PO-DMY-10021</t>
         </is>
       </c>
       <c r="I51" s="63" t="n">
@@ -17843,7 +17843,7 @@
       </c>
       <c r="H12" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I12" s="63" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="H13" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I13" s="63" t="n">
@@ -17975,7 +17975,7 @@
       </c>
       <c r="H14" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I14" s="63" t="n">
@@ -18039,7 +18039,7 @@
       </c>
       <c r="H15" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I15" s="63" t="n">
@@ -18103,7 +18103,7 @@
       </c>
       <c r="H16" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I16" s="63" t="n">
@@ -18171,7 +18171,7 @@
       </c>
       <c r="H17" s="64" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="I17" s="63" t="n">
@@ -18235,7 +18235,7 @@
       </c>
       <c r="H18" s="64" t="inlineStr">
         <is>
-          <t>T0410011</t>
+          <t>PO-DMY-10011</t>
         </is>
       </c>
       <c r="I18" s="63" t="n">
@@ -18416,12 +18416,12 @@
       </c>
       <c r="J23" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K23" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L23" s="49" t="inlineStr">
@@ -18473,12 +18473,12 @@
       </c>
       <c r="J24" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K24" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L24" s="49" t="inlineStr">
@@ -18530,12 +18530,12 @@
       </c>
       <c r="J25" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K25" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L25" s="49" t="inlineStr">
@@ -18587,12 +18587,12 @@
       </c>
       <c r="J26" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K26" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L26" s="49" t="inlineStr">
@@ -18644,12 +18644,12 @@
       </c>
       <c r="J27" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K27" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L27" s="49" t="inlineStr">
@@ -18723,12 +18723,12 @@
       </c>
       <c r="B31" s="49" t="inlineStr">
         <is>
-          <t>T0409011</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="C31" s="49" t="inlineStr">
         <is>
-          <t>3126035911</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="D31" s="49" t="inlineStr">
@@ -35940,7 +35940,7 @@
       </c>
       <c r="F7" s="32" t="inlineStr">
         <is>
-          <t>PART-X 14-Oct needs 24 pcs (VN 18, TH 6) but only 18 pcs of crossdock PO are released on 15-Oct (T0409001 12 + T0409002 6). Scan order VN (CO-14101..14103) then TH (CO-14104): cases 1-3 (VN) have a PO, case 4 (TH) has none. Every case ends a valid cut, so blocks 1-3 are Ready and block 4 Not Ready: the unit is Partially Ready (ASN options 1 / 2 / 3 cases). In this simulation the supplier waits: on 16-Oct a new crossdock manifest (T0410001, 6 pcs) is released → [Search] again → block 4 Ready.</t>
+          <t>PART-X 14-Oct needs 24 pcs (VN 18, TH 6) but only 18 pcs of crossdock PO are released on 15-Oct (PO-DMY-09001 12 + PO-DMY-09002 6). Scan order VN (CO-14101..14103) then TH (CO-14104): cases 1-3 (VN) have a PO, case 4 (TH) has none. Every case ends a valid cut, so blocks 1-3 are Ready and block 4 Not Ready: the unit is Partially Ready (ASN options 1 / 2 / 3 cases). In this simulation the supplier waits: on 16-Oct a new crossdock manifest (PO-DMY-10001, 6 pcs) is released → [Search] again → block 4 Ready.</t>
         </is>
       </c>
     </row>
@@ -39310,12 +39310,12 @@
       </c>
       <c r="B21" s="51" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="C21" s="51" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="D21" s="51" t="inlineStr">
@@ -39361,12 +39361,12 @@
       </c>
       <c r="B22" s="51" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="C22" s="51" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="D22" s="51" t="inlineStr">
@@ -39412,12 +39412,12 @@
       </c>
       <c r="B23" s="51" t="inlineStr">
         <is>
-          <t>3126035903</t>
+          <t>MF-DMY-09003</t>
         </is>
       </c>
       <c r="C23" s="51" t="inlineStr">
         <is>
-          <t>T0409003</t>
+          <t>PO-DMY-09003</t>
         </is>
       </c>
       <c r="D23" s="51" t="inlineStr">
@@ -39517,7 +39517,7 @@
       </c>
       <c r="B27" s="51" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="C27" s="51" t="inlineStr">
@@ -39527,7 +39527,7 @@
       </c>
       <c r="D27" s="51" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="E27" s="51" t="inlineStr">
@@ -39553,7 +39553,7 @@
       </c>
       <c r="B28" s="51" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="C28" s="51" t="inlineStr">
@@ -39563,7 +39563,7 @@
       </c>
       <c r="D28" s="51" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="E28" s="51" t="inlineStr">
@@ -39589,7 +39589,7 @@
       </c>
       <c r="B29" s="51" t="inlineStr">
         <is>
-          <t>3126035903</t>
+          <t>MF-DMY-09003</t>
         </is>
       </c>
       <c r="C29" s="51" t="inlineStr">
@@ -39599,7 +39599,7 @@
       </c>
       <c r="D29" s="51" t="inlineStr">
         <is>
-          <t>T0409003</t>
+          <t>PO-DMY-09003</t>
         </is>
       </c>
       <c r="E29" s="51" t="inlineStr">
@@ -39767,7 +39767,7 @@
       </c>
       <c r="H34" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I34" s="63" t="n">
@@ -39831,7 +39831,7 @@
       </c>
       <c r="H35" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I35" s="63" t="n">
@@ -39895,7 +39895,7 @@
       </c>
       <c r="H36" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I36" s="63" t="n">
@@ -39959,7 +39959,7 @@
       </c>
       <c r="H37" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I37" s="63" t="n">
@@ -40023,7 +40023,7 @@
       </c>
       <c r="H38" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I38" s="63" t="n">
@@ -40087,7 +40087,7 @@
       </c>
       <c r="H39" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I39" s="63" t="n">
@@ -40151,7 +40151,7 @@
       </c>
       <c r="H40" s="64" t="inlineStr">
         <is>
-          <t>T0409003</t>
+          <t>PO-DMY-09003</t>
         </is>
       </c>
       <c r="I40" s="63" t="n">
@@ -40332,12 +40332,12 @@
       </c>
       <c r="J45" s="49" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="K45" s="49" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="L45" s="49" t="inlineStr">
@@ -40389,12 +40389,12 @@
       </c>
       <c r="J46" s="49" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="K46" s="49" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="L46" s="49" t="inlineStr">
@@ -40446,12 +40446,12 @@
       </c>
       <c r="J47" s="49" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="K47" s="49" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="L47" s="49" t="inlineStr">
@@ -40503,12 +40503,12 @@
       </c>
       <c r="J48" s="49" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="K48" s="49" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="L48" s="49" t="inlineStr">
@@ -40560,12 +40560,12 @@
       </c>
       <c r="J49" s="49" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="K49" s="49" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="L49" s="49" t="inlineStr">
@@ -40617,12 +40617,12 @@
       </c>
       <c r="J50" s="49" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="K50" s="49" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="L50" s="49" t="inlineStr">
@@ -40674,12 +40674,12 @@
       </c>
       <c r="J51" s="49" t="inlineStr">
         <is>
-          <t>T0409003</t>
+          <t>PO-DMY-09003</t>
         </is>
       </c>
       <c r="K51" s="49" t="inlineStr">
         <is>
-          <t>3126035903</t>
+          <t>MF-DMY-09003</t>
         </is>
       </c>
       <c r="L51" s="49" t="inlineStr">
@@ -40753,12 +40753,12 @@
       </c>
       <c r="B55" s="49" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="C55" s="49" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="D55" s="49" t="inlineStr">
@@ -40787,12 +40787,12 @@
       </c>
       <c r="B56" s="49" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="C56" s="49" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="D56" s="49" t="inlineStr">
@@ -40821,12 +40821,12 @@
       </c>
       <c r="B57" s="49" t="inlineStr">
         <is>
-          <t>T0409003</t>
+          <t>PO-DMY-09003</t>
         </is>
       </c>
       <c r="C57" s="49" t="inlineStr">
         <is>
-          <t>3126035903</t>
+          <t>MF-DMY-09003</t>
         </is>
       </c>
       <c r="D57" s="49" t="inlineStr">
@@ -41375,12 +41375,12 @@
       </c>
       <c r="B70" s="49" t="inlineStr">
         <is>
-          <t>3126035901A1</t>
+          <t>MF-DMY-09001A1</t>
         </is>
       </c>
       <c r="C70" s="49" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="D70" s="49" t="inlineStr">
@@ -41400,7 +41400,7 @@
       </c>
       <c r="G70" s="49" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="H70" s="61" t="inlineStr">
@@ -41439,12 +41439,12 @@
       </c>
       <c r="B71" s="49" t="inlineStr">
         <is>
-          <t>3126035902A1</t>
+          <t>MF-DMY-09002A1</t>
         </is>
       </c>
       <c r="C71" s="49" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="D71" s="49" t="inlineStr">
@@ -41464,7 +41464,7 @@
       </c>
       <c r="G71" s="49" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="H71" s="61" t="inlineStr">
@@ -41503,12 +41503,12 @@
       </c>
       <c r="B72" s="49" t="inlineStr">
         <is>
-          <t>3126035903A1</t>
+          <t>MF-DMY-09003A1</t>
         </is>
       </c>
       <c r="C72" s="49" t="inlineStr">
         <is>
-          <t>3126035903</t>
+          <t>MF-DMY-09003</t>
         </is>
       </c>
       <c r="D72" s="49" t="inlineStr">
@@ -41528,7 +41528,7 @@
       </c>
       <c r="G72" s="49" t="inlineStr">
         <is>
-          <t>T0409003</t>
+          <t>PO-DMY-09003</t>
         </is>
       </c>
       <c r="H72" s="61" t="inlineStr">
@@ -41646,12 +41646,12 @@
       </c>
       <c r="B76" s="49" t="inlineStr">
         <is>
-          <t>3126035901A1</t>
+          <t>MF-DMY-09001A1</t>
         </is>
       </c>
       <c r="C76" s="49" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="D76" s="49" t="inlineStr">
@@ -41666,7 +41666,7 @@
       </c>
       <c r="F76" s="49" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="G76" s="49" t="inlineStr">
@@ -41705,12 +41705,12 @@
       </c>
       <c r="B77" s="49" t="inlineStr">
         <is>
-          <t>3126035901A1</t>
+          <t>MF-DMY-09001A1</t>
         </is>
       </c>
       <c r="C77" s="49" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="D77" s="49" t="inlineStr">
@@ -41725,7 +41725,7 @@
       </c>
       <c r="F77" s="49" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="G77" s="49" t="inlineStr">
@@ -41764,12 +41764,12 @@
       </c>
       <c r="B78" s="49" t="inlineStr">
         <is>
-          <t>3126035902A1</t>
+          <t>MF-DMY-09002A1</t>
         </is>
       </c>
       <c r="C78" s="49" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="D78" s="49" t="inlineStr">
@@ -41784,7 +41784,7 @@
       </c>
       <c r="F78" s="49" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="G78" s="49" t="inlineStr">
@@ -41823,12 +41823,12 @@
       </c>
       <c r="B79" s="49" t="inlineStr">
         <is>
-          <t>3126035902A1</t>
+          <t>MF-DMY-09002A1</t>
         </is>
       </c>
       <c r="C79" s="49" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="D79" s="49" t="inlineStr">
@@ -41843,7 +41843,7 @@
       </c>
       <c r="F79" s="49" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="G79" s="49" t="inlineStr">
@@ -41882,12 +41882,12 @@
       </c>
       <c r="B80" s="49" t="inlineStr">
         <is>
-          <t>3126035903A1</t>
+          <t>MF-DMY-09003A1</t>
         </is>
       </c>
       <c r="C80" s="49" t="inlineStr">
         <is>
-          <t>3126035903</t>
+          <t>MF-DMY-09003</t>
         </is>
       </c>
       <c r="D80" s="49" t="inlineStr">
@@ -41902,7 +41902,7 @@
       </c>
       <c r="F80" s="49" t="inlineStr">
         <is>
-          <t>T0409003</t>
+          <t>PO-DMY-09003</t>
         </is>
       </c>
       <c r="G80" s="49" t="inlineStr">
@@ -42138,12 +42138,12 @@
       </c>
       <c r="J88" s="58" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="K88" s="58" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="L88" s="58" t="inlineStr">
@@ -42203,12 +42203,12 @@
       </c>
       <c r="J89" s="58" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="K89" s="58" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="L89" s="58" t="inlineStr">
@@ -42268,12 +42268,12 @@
       </c>
       <c r="J90" s="58" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="K90" s="58" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="L90" s="58" t="inlineStr">
@@ -42333,12 +42333,12 @@
       </c>
       <c r="J91" s="58" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="K91" s="58" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="L91" s="58" t="inlineStr">
@@ -42398,12 +42398,12 @@
       </c>
       <c r="J92" s="58" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="K92" s="58" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="L92" s="58" t="inlineStr">
@@ -42463,12 +42463,12 @@
       </c>
       <c r="J93" s="58" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="K93" s="58" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="L93" s="58" t="inlineStr">
@@ -42528,12 +42528,12 @@
       </c>
       <c r="J94" s="58" t="inlineStr">
         <is>
-          <t>T0409003</t>
+          <t>PO-DMY-09003</t>
         </is>
       </c>
       <c r="K94" s="58" t="inlineStr">
         <is>
-          <t>3126035903</t>
+          <t>MF-DMY-09003</t>
         </is>
       </c>
       <c r="L94" s="58" t="inlineStr">
@@ -42603,7 +42603,7 @@
     <row r="3">
       <c r="A3" s="34" t="inlineStr">
         <is>
-          <t>• PART-X 14-Oct needs 24 pcs (VN 18, TH 6) but only 18 pcs of crossdock PO are released on 15-Oct (T0409001 12 + T0409002 6).</t>
+          <t>• PART-X 14-Oct needs 24 pcs (VN 18, TH 6) but only 18 pcs of crossdock PO are released on 15-Oct (PO-DMY-09001 12 + PO-DMY-09002 6).</t>
         </is>
       </c>
     </row>
@@ -42617,7 +42617,7 @@
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
         <is>
-          <t>• In this simulation the supplier waits: on 16-Oct a new crossdock manifest (T0410001, 6 pcs) is released → [Search] again → block 4 Ready.</t>
+          <t>• In this simulation the supplier waits: on 16-Oct a new crossdock manifest (PO-DMY-10001, 6 pcs) is released → [Search] again → block 4 Ready.</t>
         </is>
       </c>
     </row>
@@ -42762,7 +42762,7 @@
       </c>
       <c r="B12" s="51" t="inlineStr">
         <is>
-          <t>3126035901</t>
+          <t>MF-DMY-09001</t>
         </is>
       </c>
       <c r="C12" s="51" t="inlineStr">
@@ -42772,7 +42772,7 @@
       </c>
       <c r="D12" s="51" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="E12" s="51" t="inlineStr">
@@ -42798,7 +42798,7 @@
       </c>
       <c r="B13" s="51" t="inlineStr">
         <is>
-          <t>3126035902</t>
+          <t>MF-DMY-09002</t>
         </is>
       </c>
       <c r="C13" s="51" t="inlineStr">
@@ -42808,7 +42808,7 @@
       </c>
       <c r="D13" s="51" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="E13" s="51" t="inlineStr">
@@ -42976,7 +42976,7 @@
       </c>
       <c r="H18" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I18" s="63" t="n">
@@ -43040,7 +43040,7 @@
       </c>
       <c r="H19" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I19" s="63" t="n">
@@ -43104,7 +43104,7 @@
       </c>
       <c r="H20" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I20" s="63" t="n">
@@ -43168,7 +43168,7 @@
       </c>
       <c r="H21" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I21" s="63" t="n">
@@ -43232,7 +43232,7 @@
       </c>
       <c r="H22" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I22" s="63" t="n">
@@ -43425,12 +43425,12 @@
       </c>
       <c r="B28" s="49" t="inlineStr">
         <is>
-          <t>3126036001</t>
+          <t>MF-DMY-10001</t>
         </is>
       </c>
       <c r="C28" s="49" t="inlineStr">
         <is>
-          <t>T0410001</t>
+          <t>PO-DMY-10001</t>
         </is>
       </c>
       <c r="D28" s="49" t="inlineStr">
@@ -43530,7 +43530,7 @@
       </c>
       <c r="B32" s="49" t="inlineStr">
         <is>
-          <t>3126036001</t>
+          <t>MF-DMY-10001</t>
         </is>
       </c>
       <c r="C32" s="49" t="inlineStr">
@@ -43540,7 +43540,7 @@
       </c>
       <c r="D32" s="49" t="inlineStr">
         <is>
-          <t>T0410001</t>
+          <t>PO-DMY-10001</t>
         </is>
       </c>
       <c r="E32" s="49" t="inlineStr">
@@ -43708,7 +43708,7 @@
       </c>
       <c r="H37" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I37" s="63" t="n">
@@ -43772,7 +43772,7 @@
       </c>
       <c r="H38" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I38" s="63" t="n">
@@ -43836,7 +43836,7 @@
       </c>
       <c r="H39" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I39" s="63" t="n">
@@ -43900,7 +43900,7 @@
       </c>
       <c r="H40" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I40" s="63" t="n">
@@ -43964,7 +43964,7 @@
       </c>
       <c r="H41" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I41" s="63" t="n">
@@ -44028,7 +44028,7 @@
       </c>
       <c r="H42" s="60" t="inlineStr">
         <is>
-          <t>T0410001</t>
+          <t>PO-DMY-10001</t>
         </is>
       </c>
       <c r="I42" s="63" t="n">
@@ -44058,7 +44058,7 @@
       </c>
       <c r="P42" s="64" t="inlineStr">
         <is>
-          <t>PO T0410001: unit Ready</t>
+          <t>PO PO-DMY-10001: unit Ready</t>
         </is>
       </c>
     </row>
@@ -44711,7 +44711,7 @@
       </c>
       <c r="H20" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I20" s="63" t="n">
@@ -44775,7 +44775,7 @@
       </c>
       <c r="H21" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I21" s="63" t="n">
@@ -44839,7 +44839,7 @@
       </c>
       <c r="H22" s="64" t="inlineStr">
         <is>
-          <t>T0409001</t>
+          <t>PO-DMY-09001</t>
         </is>
       </c>
       <c r="I22" s="63" t="n">
@@ -44903,7 +44903,7 @@
       </c>
       <c r="H23" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I23" s="63" t="n">
@@ -44967,7 +44967,7 @@
       </c>
       <c r="H24" s="64" t="inlineStr">
         <is>
-          <t>T0409002</t>
+          <t>PO-DMY-09002</t>
         </is>
       </c>
       <c r="I24" s="63" t="n">

</xml_diff>

<commit_message>
Simulation: whole order date 17-Oct in one ASN, cancel in case 3 moved to CO-14108
simulasi_asn_rev.xlsx, ERD SIM-5, XD08 / XD11 examples and the Change Order
Number prototype follow the same story: ASN0003 = cases 1-3 of order date
17-Oct; CO-14104 cancelled in case 3 is replaced by CO-14108 (UPD_STATUS 6).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -10132,7 +10132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:P102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10149,7 +10149,8 @@
     <col width="15" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10176,21 +10177,21 @@
     <row r="4">
       <c r="A4" s="34" t="inlineStr">
         <is>
-          <t>• 15-Oct CO-14101 VN → ASN0001, CO-14102 TH on hold. 16-Oct CO-14101 received (6), CO-14102 cancelled (2, no ASN: nothing else), CO-14103 → ASN00002.</t>
+          <t>• 16-Oct CO-14101 VN → ASN0001, CO-14102 TH on hold. 17-Oct CO-14101 received (6), CO-14102 cancelled (2, no ASN: nothing else), CO-14103 → ASN0002.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
         <is>
-          <t>• 17-Oct CO-14103 received; CO-14104 TH → ASN00003. 18-Oct CO-14104 cancelled although in ASN00003, CO-14105 VN received without ASN (6, PO_MAPPED N).</t>
+          <t>• 18-Oct order date 17-Oct: scan order CO-14105, CO-14106 + CO-14107, CO-14104 (customer code 9715300 before 9722D10); all 3 cases Ready, sent together in ASN0003. CO-14108 (order date 18-Oct) gets no PO (Not Ready).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>• The D/S team moves the 6 pcs of ASN00003 from CO-14104 to CO-14105 in Change Order Number (XD11); history in TB_H_CROSSDOCK_ORDER_CHANGE.</t>
+          <t>• 19-Oct ASN0003 received; CO-14104 cancelled although in case 3, its pcs go to CO-14108 in G-System (6, PO_MAPPED N, no ASN). The D/S team moves case 3 from CO-14104 to CO-14108 in Change Order Number (XD11); history in TB_H_CROSSDOCK_ORDER_CHANGE.</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10255,7 @@
     <row r="10">
       <c r="A10" s="45" t="inlineStr">
         <is>
-          <t>1. 15-Oct XD08: first replication</t>
+          <t>1. 16-Oct XD08: first replication</t>
         </is>
       </c>
       <c r="B10" s="46" t="n"/>
@@ -10271,6 +10272,7 @@
       <c r="M10" s="46" t="n"/>
       <c r="N10" s="46" t="n"/>
       <c r="O10" s="46" t="n"/>
+      <c r="P10" s="46" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
@@ -10374,7 +10376,7 @@
       </c>
       <c r="D13" s="49" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E13" s="49" t="inlineStr">
@@ -10440,7 +10442,7 @@
       </c>
       <c r="D14" s="49" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E14" s="49" t="inlineStr">
@@ -10491,7 +10493,7 @@
     <row r="16">
       <c r="A16" s="45" t="inlineStr">
         <is>
-          <t>2. 15-Oct D/S holds CO-14102; supplier creates and submits ASN0001 (CO-14101)</t>
+          <t>2. 16-Oct D/S holds CO-14102; supplier creates and submits ASN0001 (CO-14101)</t>
         </is>
       </c>
       <c r="B16" s="46" t="n"/>
@@ -10508,6 +10510,7 @@
       <c r="M16" s="46" t="n"/>
       <c r="N16" s="46" t="n"/>
       <c r="O16" s="46" t="n"/>
+      <c r="P16" s="46" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="35" t="inlineStr">
@@ -10638,12 +10641,12 @@
       </c>
       <c r="J19" s="49" t="inlineStr">
         <is>
-          <t>PO-DMY-09051</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K19" s="49" t="inlineStr">
         <is>
-          <t>MF-DMY-09051</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L19" s="49" t="inlineStr">
@@ -10765,7 +10768,7 @@
       </c>
       <c r="D23" s="58" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E23" s="58" t="inlineStr">
@@ -10831,7 +10834,7 @@
       </c>
       <c r="D24" s="58" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E24" s="58" t="inlineStr">
@@ -10875,14 +10878,14 @@
       <c r="M24" s="58" t="n"/>
       <c r="N24" s="58" t="inlineStr">
         <is>
-          <t>Hold by D/S (screen)</t>
+          <t>Hold by D/S (screen); PO-DMY-09012 stays open</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="45" t="inlineStr">
         <is>
-          <t>3. 16-Oct XD08: source CO-14101 → 6, CO-14102 → 2, CO-14103 new</t>
+          <t>3. 17-Oct XD08: source CO-14101 → 6, CO-14102 → 2, CO-14103 new</t>
         </is>
       </c>
       <c r="B26" s="46" t="n"/>
@@ -10899,6 +10902,7 @@
       <c r="M26" s="46" t="n"/>
       <c r="N26" s="46" t="n"/>
       <c r="O26" s="46" t="n"/>
+      <c r="P26" s="46" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="35" t="inlineStr">
@@ -11002,7 +11006,7 @@
       </c>
       <c r="D29" s="58" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E29" s="58" t="inlineStr">
@@ -11072,7 +11076,7 @@
       </c>
       <c r="D30" s="58" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E30" s="58" t="inlineStr">
@@ -11193,7 +11197,7 @@
     <row r="33">
       <c r="A33" s="45" t="inlineStr">
         <is>
-          <t>4. 16-Oct CO-14103 → ASN00002</t>
+          <t>4. 17-Oct CO-14103 → ASN0002 (PO-DMY-09012)</t>
         </is>
       </c>
       <c r="B33" s="46" t="n"/>
@@ -11210,6 +11214,7 @@
       <c r="M33" s="46" t="n"/>
       <c r="N33" s="46" t="n"/>
       <c r="O33" s="46" t="n"/>
+      <c r="P33" s="46" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="35" t="inlineStr">
@@ -11340,12 +11345,12 @@
       </c>
       <c r="J36" s="49" t="inlineStr">
         <is>
-          <t>PO-DMY-10052</t>
+          <t>PO-DMY-09012</t>
         </is>
       </c>
       <c r="K36" s="49" t="inlineStr">
         <is>
-          <t>MF-DMY-10052</t>
+          <t>MF-DMY-09012</t>
         </is>
       </c>
       <c r="L36" s="49" t="inlineStr">
@@ -11355,7 +11360,7 @@
       </c>
       <c r="M36" s="49" t="inlineStr">
         <is>
-          <t>ASN00002</t>
+          <t>ASN0002</t>
         </is>
       </c>
       <c r="N36" s="49" t="inlineStr">
@@ -11514,7 +11519,7 @@
     <row r="42">
       <c r="A42" s="45" t="inlineStr">
         <is>
-          <t>5. 17-Oct XD08: CO-14103 → 6, CO-14104 and CO-14105 new; CO-14104 → ASN00003</t>
+          <t>5. 18-Oct XD08: CO-14103 → 6; CO-14104 … CO-14108 new (rows in scan order)</t>
         </is>
       </c>
       <c r="B42" s="46" t="n"/>
@@ -11531,6 +11536,7 @@
       <c r="M42" s="46" t="n"/>
       <c r="N42" s="46" t="n"/>
       <c r="O42" s="46" t="n"/>
+      <c r="P42" s="46" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="35" t="inlineStr">
@@ -11694,12 +11700,12 @@
       </c>
       <c r="B46" s="49" t="inlineStr">
         <is>
-          <t>9722D10</t>
+          <t>9715300</t>
         </is>
       </c>
       <c r="C46" s="49" t="inlineStr">
         <is>
-          <t>CO-14104</t>
+          <t>CO-14105</t>
         </is>
       </c>
       <c r="D46" s="49" t="inlineStr">
@@ -11709,7 +11715,7 @@
       </c>
       <c r="E46" s="49" t="inlineStr">
         <is>
-          <t>9722D10</t>
+          <t>9715310</t>
         </is>
       </c>
       <c r="F46" s="49" t="inlineStr">
@@ -11756,12 +11762,12 @@
       </c>
       <c r="B47" s="49" t="inlineStr">
         <is>
-          <t>9722D10</t>
+          <t>9715300</t>
         </is>
       </c>
       <c r="C47" s="49" t="inlineStr">
         <is>
-          <t>CO-14105</t>
+          <t>CO-14106</t>
         </is>
       </c>
       <c r="D47" s="49" t="inlineStr">
@@ -11790,7 +11796,7 @@
         </is>
       </c>
       <c r="I47" s="53" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J47" s="49" t="inlineStr">
         <is>
@@ -11810,816 +11816,1015 @@
       <c r="M47" s="49" t="n"/>
       <c r="N47" s="49" t="inlineStr"/>
     </row>
+    <row r="48">
+      <c r="A48" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C48" s="49" t="inlineStr">
+        <is>
+          <t>CO-14107</t>
+        </is>
+      </c>
+      <c r="D48" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E48" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F48" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G48" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H48" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I48" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="J48" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K48" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L48" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M48" s="49" t="n"/>
+      <c r="N48" s="49" t="inlineStr"/>
+    </row>
     <row r="49">
-      <c r="A49" s="35" t="inlineStr">
+      <c r="A49" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C49" s="49" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="D49" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E49" s="49" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F49" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G49" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H49" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I49" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J49" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K49" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L49" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M49" s="49" t="n"/>
+      <c r="N49" s="49" t="inlineStr">
+        <is>
+          <t>Customer code 9722D10 after 9715300</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B50" s="49" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C50" s="49" t="inlineStr">
+        <is>
+          <t>CO-14108</t>
+        </is>
+      </c>
+      <c r="D50" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E50" s="49" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F50" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G50" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H50" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I50" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J50" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K50" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L50" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M50" s="49" t="n"/>
+      <c r="N50" s="49" t="inlineStr">
+        <is>
+          <t>Order date 18-Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="45" t="inlineStr">
+        <is>
+          <t>6. 18-Oct [Search] → XD09 (unit 17-Oct: 3 cases Ready; unit 18-Oct: no PO)</t>
+        </is>
+      </c>
+      <c r="B52" s="46" t="n"/>
+      <c r="C52" s="46" t="n"/>
+      <c r="D52" s="46" t="n"/>
+      <c r="E52" s="46" t="n"/>
+      <c r="F52" s="46" t="n"/>
+      <c r="G52" s="46" t="n"/>
+      <c r="H52" s="46" t="n"/>
+      <c r="I52" s="46" t="n"/>
+      <c r="J52" s="46" t="n"/>
+      <c r="K52" s="46" t="n"/>
+      <c r="L52" s="46" t="n"/>
+      <c r="M52" s="46" t="n"/>
+      <c r="N52" s="46" t="n"/>
+      <c r="O52" s="46" t="n"/>
+      <c r="P52" s="46" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="35" t="inlineStr">
+        <is>
+          <t>#TEMP_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D53" s="47" t="inlineStr">
+        <is>
+          <t>Temporary (session)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="26" customHeight="1">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>SORT_SEQ</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>OPEN_ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="I54" s="9" t="inlineStr">
+        <is>
+          <t>ASSIGNED_QTY</t>
+        </is>
+      </c>
+      <c r="J54" s="9" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="K54" s="9" t="inlineStr">
+        <is>
+          <t>CUM_DEST_QTY</t>
+        </is>
+      </c>
+      <c r="L54" s="9" t="inlineStr">
+        <is>
+          <t>SEQ_QTY</t>
+        </is>
+      </c>
+      <c r="M54" s="9" t="inlineStr">
+        <is>
+          <t>CUT_FLAG</t>
+        </is>
+      </c>
+      <c r="N54" s="9" t="inlineStr">
+        <is>
+          <t>GROUP_SEQ</t>
+        </is>
+      </c>
+      <c r="O54" s="9" t="inlineStr">
+        <is>
+          <t>CROSSDOCK_STATUS</t>
+        </is>
+      </c>
+      <c r="P54" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B55" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D55" s="64" t="inlineStr">
+        <is>
+          <t>CO-14105</t>
+        </is>
+      </c>
+      <c r="E55" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F55" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G55" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H55" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09013</t>
+        </is>
+      </c>
+      <c r="I55" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J55" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L55" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M55" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N55" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="O55" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P55" s="64" t="inlineStr">
+        <is>
+          <t>Cases 1-3 ticked → ASN0003</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B56" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D56" s="64" t="inlineStr">
+        <is>
+          <t>CO-14106</t>
+        </is>
+      </c>
+      <c r="E56" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F56" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G56" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="H56" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="I56" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="J56" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K56" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="L56" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="M56" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N56" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O56" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P56" s="64" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B57" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D57" s="64" t="inlineStr">
+        <is>
+          <t>CO-14107</t>
+        </is>
+      </c>
+      <c r="E57" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F57" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G57" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="H57" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="I57" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="J57" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K57" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="L57" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M57" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N57" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P57" s="64" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B58" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="D58" s="64" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="E58" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F58" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G58" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H58" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="I58" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J58" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K58" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L58" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M58" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N58" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="O58" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P58" s="64" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B59" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="D59" s="64" t="inlineStr">
+        <is>
+          <t>CO-14108</t>
+        </is>
+      </c>
+      <c r="E59" s="64" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F59" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G59" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H59" s="64" t="n"/>
+      <c r="I59" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J59" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L59" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M59" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N59" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="O59" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="P59" s="64" t="inlineStr">
+        <is>
+          <t>Not Ready (no PO left)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="45" t="inlineStr">
+        <is>
+          <t>7. 18-Oct ASN0003 = cases 1-3 (whole order date 17-Oct)</t>
+        </is>
+      </c>
+      <c r="B61" s="46" t="n"/>
+      <c r="C61" s="46" t="n"/>
+      <c r="D61" s="46" t="n"/>
+      <c r="E61" s="46" t="n"/>
+      <c r="F61" s="46" t="n"/>
+      <c r="G61" s="46" t="n"/>
+      <c r="H61" s="46" t="n"/>
+      <c r="I61" s="46" t="n"/>
+      <c r="J61" s="46" t="n"/>
+      <c r="K61" s="46" t="n"/>
+      <c r="L61" s="46" t="n"/>
+      <c r="M61" s="46" t="n"/>
+      <c r="N61" s="46" t="n"/>
+      <c r="O61" s="46" t="n"/>
+      <c r="P61" s="46" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="35" t="inlineStr">
         <is>
           <t>TB_R_INSTRUCTION</t>
         </is>
       </c>
-      <c r="D49" s="47" t="inlineStr">
+      <c r="D62" s="47" t="inlineStr">
         <is>
           <t>New table (Crossdock)</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="26" customHeight="1">
-      <c r="A50" s="3" t="inlineStr">
+    <row r="63" ht="26" customHeight="1">
+      <c r="A63" s="3" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B50" s="42" t="inlineStr">
+      <c r="B63" s="42" t="inlineStr">
         <is>
           <t>INSTRUCTION_ID</t>
         </is>
       </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>CASE_SEQ</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>LINE_SEQ</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="E63" s="3" t="inlineStr">
         <is>
           <t>PART_NO</t>
         </is>
       </c>
-      <c r="F50" s="3" t="inlineStr">
+      <c r="F63" s="3" t="inlineStr">
         <is>
           <t>DESTINATION_CD</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr">
+      <c r="G63" s="3" t="inlineStr">
         <is>
           <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="H50" s="3" t="inlineStr">
+      <c r="H63" s="3" t="inlineStr">
         <is>
           <t>SERIAL_NO</t>
         </is>
       </c>
-      <c r="I50" s="3" t="inlineStr">
+      <c r="I63" s="3" t="inlineStr">
         <is>
           <t>QTY</t>
         </is>
       </c>
-      <c r="J50" s="3" t="inlineStr">
+      <c r="J63" s="3" t="inlineStr">
         <is>
           <t>PO_NO</t>
         </is>
       </c>
-      <c r="K50" s="3" t="inlineStr">
+      <c r="K63" s="3" t="inlineStr">
         <is>
           <t>MANIFEST_NO</t>
         </is>
       </c>
-      <c r="L50" s="3" t="inlineStr">
+      <c r="L63" s="3" t="inlineStr">
         <is>
           <t>MANIFEST_ITEM</t>
         </is>
       </c>
-      <c r="M50" s="3" t="inlineStr">
+      <c r="M63" s="3" t="inlineStr">
         <is>
           <t>ASN_NO</t>
         </is>
       </c>
-      <c r="N50" s="3" t="inlineStr">
+      <c r="N63" s="3" t="inlineStr">
         <is>
           <t>CASE_NO</t>
         </is>
       </c>
-      <c r="O50" s="3" t="inlineStr">
+      <c r="O63" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="48" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="48" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="B51" s="53" t="n">
+      <c r="B64" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="C51" s="53" t="n">
+      <c r="C64" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="D51" s="53" t="n">
+      <c r="D64" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E51" s="49" t="inlineStr">
+      <c r="E64" s="49" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="F51" s="49" t="inlineStr">
+      <c r="F64" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G64" s="49" t="inlineStr">
+        <is>
+          <t>CO-14105</t>
+        </is>
+      </c>
+      <c r="H64" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I64" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J64" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09013</t>
+        </is>
+      </c>
+      <c r="K64" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09013</t>
+        </is>
+      </c>
+      <c r="L64" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M64" s="49" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N64" s="49" t="inlineStr">
+        <is>
+          <t>C-0003-01</t>
+        </is>
+      </c>
+      <c r="O64" s="49" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B65" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F65" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G65" s="49" t="inlineStr">
+        <is>
+          <t>CO-14106</t>
+        </is>
+      </c>
+      <c r="H65" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I65" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="J65" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="K65" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09014</t>
+        </is>
+      </c>
+      <c r="L65" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M65" s="49" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N65" s="49" t="inlineStr">
+        <is>
+          <t>C-0003-02</t>
+        </is>
+      </c>
+      <c r="O65" s="49" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B66" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F66" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G66" s="49" t="inlineStr">
+        <is>
+          <t>CO-14107</t>
+        </is>
+      </c>
+      <c r="H66" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I66" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="J66" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="K66" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09014</t>
+        </is>
+      </c>
+      <c r="L66" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M66" s="49" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N66" s="49" t="inlineStr">
+        <is>
+          <t>C-0003-02</t>
+        </is>
+      </c>
+      <c r="O66" s="49" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B67" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C67" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D67" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F67" s="49" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="G51" s="49" t="inlineStr">
+      <c r="G67" s="49" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
       </c>
-      <c r="H51" s="49" t="inlineStr">
+      <c r="H67" s="49" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="I51" s="53" t="n">
+      <c r="I67" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="J51" s="49" t="inlineStr">
-        <is>
-          <t>PO-DMY-10053</t>
-        </is>
-      </c>
-      <c r="K51" s="49" t="inlineStr">
-        <is>
-          <t>MF-DMY-10053</t>
-        </is>
-      </c>
-      <c r="L51" s="49" t="inlineStr">
+      <c r="J67" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="K67" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09014</t>
+        </is>
+      </c>
+      <c r="L67" s="49" t="inlineStr">
         <is>
           <t>0001</t>
         </is>
       </c>
-      <c r="M51" s="49" t="inlineStr">
-        <is>
-          <t>ASN00003</t>
-        </is>
-      </c>
-      <c r="N51" s="49" t="inlineStr">
-        <is>
-          <t>C-0003-01</t>
-        </is>
-      </c>
-      <c r="O51" s="49" t="inlineStr">
-        <is>
-          <t>CO-14105: no PO yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="45" t="inlineStr">
-        <is>
-          <t>6. 18-Oct XD08: CO-14104 → 2 (in ASN00003), CO-14105 → 6</t>
-        </is>
-      </c>
-      <c r="B53" s="46" t="n"/>
-      <c r="C53" s="46" t="n"/>
-      <c r="D53" s="46" t="n"/>
-      <c r="E53" s="46" t="n"/>
-      <c r="F53" s="46" t="n"/>
-      <c r="G53" s="46" t="n"/>
-      <c r="H53" s="46" t="n"/>
-      <c r="I53" s="46" t="n"/>
-      <c r="J53" s="46" t="n"/>
-      <c r="K53" s="46" t="n"/>
-      <c r="L53" s="46" t="n"/>
-      <c r="M53" s="46" t="n"/>
-      <c r="N53" s="46" t="n"/>
-      <c r="O53" s="46" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
-        </is>
-      </c>
-      <c r="D54" s="47" t="inlineStr">
-        <is>
-          <t>Replicated from DB Surrounding (G-System)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B55" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="C55" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="D55" s="42" t="inlineStr">
-        <is>
-          <t>ORDER_DT</t>
-        </is>
-      </c>
-      <c r="E55" s="42" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F55" s="42" t="inlineStr">
-        <is>
-          <t>DETAILED_ITEM_NO</t>
-        </is>
-      </c>
-      <c r="G55" s="42" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="H55" s="5" t="inlineStr">
-        <is>
-          <t>SHIPPING_PART_NO</t>
-        </is>
-      </c>
-      <c r="I55" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS_QTY</t>
-        </is>
-      </c>
-      <c r="J55" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS</t>
-        </is>
-      </c>
-      <c r="K55" s="5" t="inlineStr">
-        <is>
-          <t>HOLD_FLAG</t>
-        </is>
-      </c>
-      <c r="L55" s="5" t="inlineStr">
-        <is>
-          <t>PO_MAPPED_FLAG</t>
-        </is>
-      </c>
-      <c r="M55" s="5" t="inlineStr">
-        <is>
-          <t>UPD_STATUS</t>
-        </is>
-      </c>
-      <c r="N55" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B56" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C56" s="58" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="D56" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E56" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F56" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G56" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H56" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I56" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="J56" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K56" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L56" s="58" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M56" s="60" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N56" s="58" t="inlineStr">
-        <is>
-          <t>Cancel after ASN: LOG5, listed in XD11; ASN not changed</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B57" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C57" s="58" t="inlineStr">
-        <is>
-          <t>CO-14105</t>
-        </is>
-      </c>
-      <c r="D57" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E57" s="58" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F57" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G57" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H57" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I57" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="J57" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K57" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L57" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M57" s="60" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N57" s="58" t="inlineStr">
-        <is>
-          <t>Received without ASN (allocated by G-System): candidate</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="45" t="inlineStr">
-        <is>
-          <t>7. 18-Oct XD11 Change Order Number: ASN00003 6 pcs → CO-14105</t>
-        </is>
-      </c>
-      <c r="B59" s="46" t="n"/>
-      <c r="C59" s="46" t="n"/>
-      <c r="D59" s="46" t="n"/>
-      <c r="E59" s="46" t="n"/>
-      <c r="F59" s="46" t="n"/>
-      <c r="G59" s="46" t="n"/>
-      <c r="H59" s="46" t="n"/>
-      <c r="I59" s="46" t="n"/>
-      <c r="J59" s="46" t="n"/>
-      <c r="K59" s="46" t="n"/>
-      <c r="L59" s="46" t="n"/>
-      <c r="M59" s="46" t="n"/>
-      <c r="N59" s="46" t="n"/>
-      <c r="O59" s="46" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D60" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="26" customHeight="1">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B61" s="42" t="inlineStr">
-        <is>
-          <t>INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>LINE_SEQ</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="K61" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="L61" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="M61" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="N61" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
-        </is>
-      </c>
-      <c r="O61" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B62" s="59" t="n">
-        <v>3</v>
-      </c>
-      <c r="C62" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="F62" s="60" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="G62" s="60" t="inlineStr">
-        <is>
-          <t>CO-14105</t>
-        </is>
-      </c>
-      <c r="H62" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="I62" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="J62" s="58" t="inlineStr">
-        <is>
-          <t>PO-DMY-10053</t>
-        </is>
-      </c>
-      <c r="K62" s="58" t="inlineStr">
-        <is>
-          <t>MF-DMY-10053</t>
-        </is>
-      </c>
-      <c r="L62" s="58" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="M62" s="58" t="inlineStr">
-        <is>
-          <t>ASN00003</t>
-        </is>
-      </c>
-      <c r="N62" s="58" t="inlineStr">
-        <is>
-          <t>C-0003-01</t>
-        </is>
-      </c>
-      <c r="O62" s="58" t="inlineStr">
-        <is>
-          <t>Whole row moved; case, PO and ASN not changed</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
-        </is>
-      </c>
-      <c r="D64" s="47" t="inlineStr">
-        <is>
-          <t>Replicated from DB Surrounding (G-System)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="26" customHeight="1">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B65" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="C65" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="D65" s="42" t="inlineStr">
-        <is>
-          <t>ORDER_DT</t>
-        </is>
-      </c>
-      <c r="E65" s="42" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F65" s="42" t="inlineStr">
-        <is>
-          <t>DETAILED_ITEM_NO</t>
-        </is>
-      </c>
-      <c r="G65" s="42" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="H65" s="5" t="inlineStr">
-        <is>
-          <t>SHIPPING_PART_NO</t>
-        </is>
-      </c>
-      <c r="I65" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS_QTY</t>
-        </is>
-      </c>
-      <c r="J65" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS</t>
-        </is>
-      </c>
-      <c r="K65" s="5" t="inlineStr">
-        <is>
-          <t>HOLD_FLAG</t>
-        </is>
-      </c>
-      <c r="L65" s="5" t="inlineStr">
-        <is>
-          <t>PO_MAPPED_FLAG</t>
-        </is>
-      </c>
-      <c r="M65" s="5" t="inlineStr">
-        <is>
-          <t>UPD_STATUS</t>
-        </is>
-      </c>
-      <c r="N65" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="50" t="inlineStr">
-        <is>
-          <t>READ</t>
-        </is>
-      </c>
-      <c r="B66" s="51" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C66" s="51" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="D66" s="51" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E66" s="51" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F66" s="51" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G66" s="51" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H66" s="51" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I66" s="52" t="n">
-        <v>6</v>
-      </c>
-      <c r="J66" s="51" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K66" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L66" s="51" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M66" s="66" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N66" s="51" t="inlineStr">
-        <is>
-          <t>Not changed (PO_MAPPED_FLAG stays Y)</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B67" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C67" s="58" t="inlineStr">
-        <is>
-          <t>CO-14105</t>
-        </is>
-      </c>
-      <c r="D67" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E67" s="58" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F67" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G67" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H67" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I67" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="J67" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K67" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L67" s="60" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="M67" s="49" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N67" s="58" t="inlineStr">
-        <is>
-          <t>PO and ASN through ASN00003</t>
-        </is>
-      </c>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N67" s="49" t="inlineStr">
+        <is>
+          <t>C-0003-03</t>
+        </is>
+      </c>
+      <c r="O67" s="49" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="35" t="inlineStr">
         <is>
-          <t>TB_H_CROSSDOCK_ORDER_CHANGE</t>
+          <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
         </is>
       </c>
       <c r="D69" s="47" t="inlineStr">
@@ -12636,17 +12841,17 @@
       </c>
       <c r="B70" s="42" t="inlineStr">
         <is>
-          <t>HIST_ID</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="C70" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="D70" s="42" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
@@ -12656,40 +12861,15 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>FROM_CUSTOMER_ORDER_NO</t>
+          <t>ORDER_QTY</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>FROM_SERIAL_NO</t>
+          <t>MAPPED_QTY</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>TO_CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="I70" s="3" t="inlineStr">
-        <is>
-          <t>TO_DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="J70" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="K70" s="3" t="inlineStr">
-        <is>
-          <t>FROM_INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="L70" s="3" t="inlineStr">
-        <is>
-          <t>TO_INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="M70" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -12701,54 +12881,1393 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="B71" s="53" t="n">
+      <c r="B71" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09013</t>
+        </is>
+      </c>
+      <c r="C71" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09013</t>
+        </is>
+      </c>
+      <c r="D71" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="E71" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F71" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="G71" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="H71" s="49" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B72" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="C72" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09014</t>
+        </is>
+      </c>
+      <c r="D72" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="E72" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F72" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="G72" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="H72" s="49" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D74" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="26" customHeight="1">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B75" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C75" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D75" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E75" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F75" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G75" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K75" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L75" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M75" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N75" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B76" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C76" s="58" t="inlineStr">
+        <is>
+          <t>CO-14105</t>
+        </is>
+      </c>
+      <c r="D76" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E76" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F76" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G76" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H76" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I76" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J76" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K76" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L76" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M76" s="58" t="n"/>
+      <c r="N76" s="58" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B77" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C77" s="58" t="inlineStr">
+        <is>
+          <t>CO-14106</t>
+        </is>
+      </c>
+      <c r="D77" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E77" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F77" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G77" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H77" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I77" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="J77" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K77" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L77" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M77" s="58" t="n"/>
+      <c r="N77" s="58" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B78" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C78" s="58" t="inlineStr">
+        <is>
+          <t>CO-14107</t>
+        </is>
+      </c>
+      <c r="D78" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E78" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F78" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G78" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H78" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I78" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="J78" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K78" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L78" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M78" s="58" t="n"/>
+      <c r="N78" s="58" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B79" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C79" s="58" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="D79" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E79" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F79" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G79" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H79" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I79" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J79" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K79" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L79" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M79" s="58" t="n"/>
+      <c r="N79" s="58" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="45" t="inlineStr">
+        <is>
+          <t>8. 19-Oct XD08: ASN0003 received, CO-14104 → 2 (in case 3), CO-14108 → 6</t>
+        </is>
+      </c>
+      <c r="B81" s="46" t="n"/>
+      <c r="C81" s="46" t="n"/>
+      <c r="D81" s="46" t="n"/>
+      <c r="E81" s="46" t="n"/>
+      <c r="F81" s="46" t="n"/>
+      <c r="G81" s="46" t="n"/>
+      <c r="H81" s="46" t="n"/>
+      <c r="I81" s="46" t="n"/>
+      <c r="J81" s="46" t="n"/>
+      <c r="K81" s="46" t="n"/>
+      <c r="L81" s="46" t="n"/>
+      <c r="M81" s="46" t="n"/>
+      <c r="N81" s="46" t="n"/>
+      <c r="O81" s="46" t="n"/>
+      <c r="P81" s="46" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D82" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="26" customHeight="1">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B83" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C83" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D83" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E83" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F83" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G83" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K83" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L83" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M83" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N83" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B84" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C84" s="58" t="inlineStr">
+        <is>
+          <t>CO-14105</t>
+        </is>
+      </c>
+      <c r="D84" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E84" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F84" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G84" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H84" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I84" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J84" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K84" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L84" s="58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M84" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N84" s="58" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B85" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C85" s="58" t="inlineStr">
+        <is>
+          <t>CO-14106</t>
+        </is>
+      </c>
+      <c r="D85" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E85" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F85" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G85" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H85" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I85" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="J85" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K85" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L85" s="58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M85" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N85" s="58" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B86" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C86" s="58" t="inlineStr">
+        <is>
+          <t>CO-14107</t>
+        </is>
+      </c>
+      <c r="D86" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E86" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F86" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G86" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H86" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I86" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="J86" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K86" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L86" s="58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M86" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N86" s="58" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B87" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C87" s="58" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="D87" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E87" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F87" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G87" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H87" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I87" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J87" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K87" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L87" s="58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M87" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N87" s="58" t="inlineStr">
+        <is>
+          <t>Cancel after ASN: LOG5, listed in XD11; ASN not changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B88" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C88" s="58" t="inlineStr">
+        <is>
+          <t>CO-14108</t>
+        </is>
+      </c>
+      <c r="D88" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E88" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F88" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G88" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H88" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I88" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J88" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K88" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L88" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M88" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N88" s="58" t="inlineStr">
+        <is>
+          <t>Received without ASN (pcs of case 3 allocated by G-System): candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="45" t="inlineStr">
+        <is>
+          <t>9. 19-Oct XD11 Change Order Number: ASN0003 case 3 → CO-14108</t>
+        </is>
+      </c>
+      <c r="B90" s="46" t="n"/>
+      <c r="C90" s="46" t="n"/>
+      <c r="D90" s="46" t="n"/>
+      <c r="E90" s="46" t="n"/>
+      <c r="F90" s="46" t="n"/>
+      <c r="G90" s="46" t="n"/>
+      <c r="H90" s="46" t="n"/>
+      <c r="I90" s="46" t="n"/>
+      <c r="J90" s="46" t="n"/>
+      <c r="K90" s="46" t="n"/>
+      <c r="L90" s="46" t="n"/>
+      <c r="M90" s="46" t="n"/>
+      <c r="N90" s="46" t="n"/>
+      <c r="O90" s="46" t="n"/>
+      <c r="P90" s="46" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D91" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="26" customHeight="1">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B92" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L92" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N92" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O92" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B93" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="C93" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D93" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="C71" s="49" t="inlineStr">
-        <is>
-          <t>ASN00003</t>
-        </is>
-      </c>
-      <c r="D71" s="49" t="inlineStr">
-        <is>
-          <t>C-0003-01</t>
-        </is>
-      </c>
-      <c r="E71" s="49" t="inlineStr">
+      <c r="E93" s="58" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="F71" s="49" t="inlineStr">
+      <c r="F93" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="G93" s="60" t="inlineStr">
+        <is>
+          <t>CO-14108</t>
+        </is>
+      </c>
+      <c r="H93" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I93" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J93" s="58" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="K93" s="58" t="inlineStr">
+        <is>
+          <t>MF-DMY-09014</t>
+        </is>
+      </c>
+      <c r="L93" s="58" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M93" s="58" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N93" s="58" t="inlineStr">
+        <is>
+          <t>C-0003-03</t>
+        </is>
+      </c>
+      <c r="O93" s="58" t="inlineStr">
+        <is>
+          <t>Whole row moved; case, PO and ASN not changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D95" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="26" customHeight="1">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B96" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C96" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D96" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E96" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F96" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G96" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J96" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K96" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L96" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M96" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N96" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B97" s="51" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C97" s="51" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
       </c>
-      <c r="G71" s="49" t="inlineStr">
+      <c r="D97" s="51" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E97" s="51" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F97" s="51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G97" s="51" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H71" s="49" t="inlineStr">
-        <is>
-          <t>CO-14105</t>
-        </is>
-      </c>
-      <c r="I71" s="49" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="J71" s="53" t="n">
+      <c r="H97" s="51" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I97" s="52" t="n">
         <v>6</v>
       </c>
-      <c r="K71" s="53" t="n">
-        <v>3</v>
-      </c>
-      <c r="L71" s="53" t="n">
-        <v>3</v>
-      </c>
-      <c r="M71" s="49" t="inlineStr"/>
+      <c r="J97" s="51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K97" s="51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L97" s="51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M97" s="66" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N97" s="51" t="inlineStr">
+        <is>
+          <t>Not changed (PO_MAPPED_FLAG stays Y)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B98" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C98" s="58" t="inlineStr">
+        <is>
+          <t>CO-14108</t>
+        </is>
+      </c>
+      <c r="D98" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E98" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F98" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G98" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H98" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I98" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J98" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K98" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L98" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M98" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N98" s="58" t="inlineStr">
+        <is>
+          <t>PO and ASN through ASN0003</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="35" t="inlineStr">
+        <is>
+          <t>TB_H_CROSSDOCK_ORDER_CHANGE</t>
+        </is>
+      </c>
+      <c r="D100" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="26" customHeight="1">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B101" s="42" t="inlineStr">
+        <is>
+          <t>HIST_ID</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>FROM_CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>FROM_SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>TO_CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>TO_DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr">
+        <is>
+          <t>FROM_INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="L101" s="3" t="inlineStr">
+        <is>
+          <t>TO_INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="M101" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B102" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" s="49" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="D102" s="49" t="inlineStr">
+        <is>
+          <t>C-0003-03</t>
+        </is>
+      </c>
+      <c r="E102" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F102" s="49" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="G102" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H102" s="49" t="inlineStr">
+        <is>
+          <t>CO-14108</t>
+        </is>
+      </c>
+      <c r="I102" s="49" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="J102" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="K102" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="L102" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="M102" s="49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21984,7 +23503,7 @@
       </c>
       <c r="F15" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-3, SIM-4, SIM-7, SIM-8, SIM-9</t>
+          <t>SIM-2, SIM-3, SIM-4, SIM-5, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -22074,7 +23593,7 @@
       </c>
       <c r="F18" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-6, SIM-7, SIM-8, SIM-9</t>
+          <t>SIM-2, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -38534,12 +40053,12 @@
       </c>
       <c r="E9" s="32" t="inlineStr">
         <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE, TB_R_INSTRUCTION, TB_H_CROSSDOCK_ORDER_CHANGE</t>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE, TB_R_INSTRUCTION, #TEMP_INSTRUCTION, TB_R_PRA_DAILY_ORDER_MAPPED, TB_H_CROSSDOCK_ORDER_CHANGE</t>
         </is>
       </c>
       <c r="F9" s="32" t="inlineStr">
         <is>
-          <t>PART-X, 6 pcs/case. ORDER_STATUS of the replicate keeps the first value (7); a change in G-System is written to UPD_STATUS: 6 received, 2 cancel. 15-Oct CO-14101 VN → ASN0001, CO-14102 TH on hold. 16-Oct CO-14101 received (6), CO-14102 cancelled (2, no ASN: nothing else), CO-14103 → ASN00002. 17-Oct CO-14103 received; CO-14104 TH → ASN00003. 18-Oct CO-14104 cancelled although in ASN00003, CO-14105 VN received without ASN (6, PO_MAPPED N). The D/S team moves the 6 pcs of ASN00003 from CO-14104 to CO-14105 in Change Order Number (XD11); history in TB_H_CROSSDOCK_ORDER_CHANGE.</t>
+          <t>PART-X, 6 pcs/case. ORDER_STATUS of the replicate keeps the first value (7); a change in G-System is written to UPD_STATUS: 6 received, 2 cancel. 16-Oct CO-14101 VN → ASN0001, CO-14102 TH on hold. 17-Oct CO-14101 received (6), CO-14102 cancelled (2, no ASN: nothing else), CO-14103 → ASN0002. 18-Oct order date 17-Oct: scan order CO-14105, CO-14106 + CO-14107, CO-14104 (customer code 9715300 before 9722D10); all 3 cases Ready, sent together in ASN0003. CO-14108 (order date 18-Oct) gets no PO (Not Ready). 19-Oct ASN0003 received; CO-14104 cancelled although in case 3, its pcs go to CO-14108 in G-System (6, PO_MAPPED N, no ASN). The D/S team moves case 3 from CO-14104 to CO-14108 in Change Order Number (XD11); history in TB_H_CROSSDOCK_ORDER_CHANGE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simulation: one PO per order date, short PO split, 4 destinations, middle-row cancel
simulasi_asn_rev.xlsx gets a PO check per customer order date (PO_DT = order
date + 1, abnormal when PO qty < order qty, rest in a split PO), destinations
9811110 and 982220, and CO-14104 cancelled in the middle of ASN0003 and moved
to CO-14111. ERD SIM-5, XD08 / XD11 examples and the Change Order Number
prototype follow the same story.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -10132,7 +10132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P102"/>
+  <dimension ref="A1:P95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10156,7 +10156,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SIM-5 UPD_STATUS day by day; cancel after ASN → Change Order Number (simulasi_asn.xlsx)</t>
+          <t>SIM-5 One PO per order date (short PO → split PO); cancel of a middle row after ASN → Change Order Number (simulasi_asn.xlsx)</t>
         </is>
       </c>
     </row>
@@ -10170,28 +10170,28 @@
     <row r="3">
       <c r="A3" s="34" t="inlineStr">
         <is>
-          <t>• PART-X, 6 pcs/case. ORDER_STATUS of the replicate keeps the first value (7); a change in G-System is written to UPD_STATUS: 6 received, 2 cancel.</t>
+          <t>• PART-X, 6 pcs/case. One PO per customer order date: PO_DT = order date + 1, qty = total order qty of the date (all destinations). PO qty &lt; order qty is an abnormality: the rest comes in a split PO. ORDER_STATUS of the replicate keeps 7; changes go to UPD_STATUS.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="34" t="inlineStr">
         <is>
-          <t>• 16-Oct CO-14101 VN → ASN0001, CO-14102 TH on hold. 17-Oct CO-14101 received (6), CO-14102 cancelled (2, no ASN: nothing else), CO-14103 → ASN0002.</t>
+          <t>• Order date 15-Oct (12) → PO-DMY-09011; CO-14102 on hold then cancelled, so its 6 pcs of PO-DMY-09011 go to CO-14103 (older PO_DT first).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
         <is>
-          <t>• 18-Oct order date 17-Oct: scan order CO-14105, CO-14106 + CO-14107, CO-14104 (customer code 9715300 before 9722D10); all 3 cases Ready, sent together in ASN0003. CO-14108 (order date 18-Oct) gets no PO (Not Ready).</t>
+          <t>• Order date 17-Oct: 4 destinations, 30 pcs, PO-DMY-09013 only 18 (abnormal) → case 5 Not Ready until the split PO-DMY-09014 (12, 19-Oct). Cases 1-4 → ASN0003; CO-14104 (middle row, case 3) is cancelled after the ASN.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>• 19-Oct ASN0003 received; CO-14104 cancelled although in case 3, its pcs go to CO-14108 in G-System (6, PO_MAPPED N, no ASN). The D/S team moves case 3 from CO-14104 to CO-14108 in Change Order Number (XD11); history in TB_H_CROSSDOCK_ORDER_CHANGE.</t>
+          <t>• 21-Oct G-System allocates the pcs of case 3 to CO-14111 (UPD_STATUS 6, no ASN): the D/S team moves case 3 to CO-14111 (XD11). Open PO qty at the end (12) = cancelled qty (CO-14102 + CO-14104).</t>
         </is>
       </c>
     </row>
@@ -10255,7 +10255,7 @@
     <row r="10">
       <c r="A10" s="45" t="inlineStr">
         <is>
-          <t>1. 16-Oct XD08: first replication</t>
+          <t>1. 16-Oct XD08 (order date 15-Oct; PO-DMY-09011 PO_DT 16-Oct, 12)</t>
         </is>
       </c>
       <c r="B10" s="46" t="n"/>
@@ -10418,11 +10418,7 @@
         </is>
       </c>
       <c r="M13" s="49" t="n"/>
-      <c r="N13" s="49" t="inlineStr">
-        <is>
-          <t>Source status 7</t>
-        </is>
-      </c>
+      <c r="N13" s="49" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="48" t="inlineStr">
@@ -10484,16 +10480,12 @@
         </is>
       </c>
       <c r="M14" s="49" t="n"/>
-      <c r="N14" s="49" t="inlineStr">
-        <is>
-          <t>Source status 7</t>
-        </is>
-      </c>
+      <c r="N14" s="49" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="45" t="inlineStr">
         <is>
-          <t>2. 16-Oct D/S holds CO-14102; supplier creates and submits ASN0001 (CO-14101)</t>
+          <t>2. 16-Oct D/S holds CO-14102; CO-14101 → ASN0001</t>
         </is>
       </c>
       <c r="B16" s="46" t="n"/>
@@ -10810,11 +10802,7 @@
         </is>
       </c>
       <c r="M23" s="58" t="n"/>
-      <c r="N23" s="58" t="inlineStr">
-        <is>
-          <t>In ASN0001</t>
-        </is>
-      </c>
+      <c r="N23" s="58" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="57" t="inlineStr">
@@ -10878,14 +10866,14 @@
       <c r="M24" s="58" t="n"/>
       <c r="N24" s="58" t="inlineStr">
         <is>
-          <t>Hold by D/S (screen); PO-DMY-09012 stays open</t>
+          <t>6 pcs of PO-DMY-09011 stay open</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="45" t="inlineStr">
         <is>
-          <t>3. 17-Oct XD08: source CO-14101 → 6, CO-14102 → 2, CO-14103 new</t>
+          <t>3. 17-Oct XD08: CO-14101 → 6, CO-14102 → 2, CO-14103 new (PO-DMY-09012 PO_DT 17-Oct, 6)</t>
         </is>
       </c>
       <c r="B26" s="46" t="n"/>
@@ -11054,7 +11042,7 @@
       </c>
       <c r="N29" s="58" t="inlineStr">
         <is>
-          <t>Received in G-System; ORDER_STATUS stays 7</t>
+          <t>Received</t>
         </is>
       </c>
     </row>
@@ -11124,7 +11112,7 @@
       </c>
       <c r="N30" s="58" t="inlineStr">
         <is>
-          <t>Cancelled, no ASN: ignored (PO_MAPPED_FLAG stays N)</t>
+          <t>Cancelled, no ASN (PO_MAPPED_FLAG stays N)</t>
         </is>
       </c>
     </row>
@@ -11188,16 +11176,12 @@
         </is>
       </c>
       <c r="M31" s="49" t="n"/>
-      <c r="N31" s="49" t="inlineStr">
-        <is>
-          <t>Source status 7</t>
-        </is>
-      </c>
+      <c r="N31" s="49" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="45" t="inlineStr">
         <is>
-          <t>4. 17-Oct CO-14103 → ASN0002 (PO-DMY-09012)</t>
+          <t>4. 17-Oct CO-14103 → ASN0002 with the rest of PO-DMY-09011 (older PO_DT)</t>
         </is>
       </c>
       <c r="B33" s="46" t="n"/>
@@ -11345,12 +11329,12 @@
       </c>
       <c r="J36" s="49" t="inlineStr">
         <is>
-          <t>PO-DMY-09012</t>
+          <t>PO-DMY-09011</t>
         </is>
       </c>
       <c r="K36" s="49" t="inlineStr">
         <is>
-          <t>MF-DMY-09012</t>
+          <t>MF-DMY-09011</t>
         </is>
       </c>
       <c r="L36" s="49" t="inlineStr">
@@ -11368,327 +11352,437 @@
           <t>C-0002-01</t>
         </is>
       </c>
-      <c r="O36" s="49" t="inlineStr"/>
+      <c r="O36" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09012 stays open</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="35" t="inlineStr">
+      <c r="A38" s="45" t="inlineStr">
+        <is>
+          <t>5. 18-Oct XD08: order date 17-Oct, 4 destinations, 30 pcs; PO-DMY-09013 only 18 (abnormal)</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="n"/>
+      <c r="C38" s="46" t="n"/>
+      <c r="D38" s="46" t="n"/>
+      <c r="E38" s="46" t="n"/>
+      <c r="F38" s="46" t="n"/>
+      <c r="G38" s="46" t="n"/>
+      <c r="H38" s="46" t="n"/>
+      <c r="I38" s="46" t="n"/>
+      <c r="J38" s="46" t="n"/>
+      <c r="K38" s="46" t="n"/>
+      <c r="L38" s="46" t="n"/>
+      <c r="M38" s="46" t="n"/>
+      <c r="N38" s="46" t="n"/>
+      <c r="O38" s="46" t="n"/>
+      <c r="P38" s="46" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr">
         <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
-      <c r="D38" s="47" t="inlineStr">
+      <c r="D39" s="47" t="inlineStr">
         <is>
           <t>Replicated from DB Surrounding (G-System)</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="40" ht="26" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B39" s="42" t="inlineStr">
+      <c r="B40" s="42" t="inlineStr">
         <is>
           <t>CUSTOMER_CD</t>
         </is>
       </c>
-      <c r="C39" s="42" t="inlineStr">
+      <c r="C40" s="42" t="inlineStr">
         <is>
           <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="D39" s="42" t="inlineStr">
+      <c r="D40" s="42" t="inlineStr">
         <is>
           <t>ORDER_DT</t>
         </is>
       </c>
-      <c r="E39" s="42" t="inlineStr">
+      <c r="E40" s="42" t="inlineStr">
         <is>
           <t>DESTINATION_CD</t>
         </is>
       </c>
-      <c r="F39" s="42" t="inlineStr">
+      <c r="F40" s="42" t="inlineStr">
         <is>
           <t>DETAILED_ITEM_NO</t>
         </is>
       </c>
-      <c r="G39" s="42" t="inlineStr">
+      <c r="G40" s="42" t="inlineStr">
         <is>
           <t>SERIAL_NO</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>SHIPPING_PART_NO</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="I40" s="5" t="inlineStr">
         <is>
           <t>ORDER_STATUS_QTY</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr">
+      <c r="J40" s="5" t="inlineStr">
         <is>
           <t>ORDER_STATUS</t>
         </is>
       </c>
-      <c r="K39" s="5" t="inlineStr">
+      <c r="K40" s="5" t="inlineStr">
         <is>
           <t>HOLD_FLAG</t>
         </is>
       </c>
-      <c r="L39" s="5" t="inlineStr">
+      <c r="L40" s="5" t="inlineStr">
         <is>
           <t>PO_MAPPED_FLAG</t>
         </is>
       </c>
-      <c r="M39" s="5" t="inlineStr">
+      <c r="M40" s="5" t="inlineStr">
         <is>
           <t>UPD_STATUS</t>
         </is>
       </c>
-      <c r="N39" s="5" t="inlineStr">
+      <c r="N40" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="57" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="57" t="inlineStr">
         <is>
           <t>UPD</t>
         </is>
       </c>
-      <c r="B40" s="58" t="inlineStr">
+      <c r="B41" s="58" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="C40" s="58" t="inlineStr">
+      <c r="C41" s="58" t="inlineStr">
         <is>
           <t>CO-14103</t>
         </is>
       </c>
-      <c r="D40" s="58" t="inlineStr">
+      <c r="D41" s="58" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E40" s="58" t="inlineStr">
+      <c r="E41" s="58" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="F40" s="58" t="inlineStr">
+      <c r="F41" s="58" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="G40" s="58" t="inlineStr">
+      <c r="G41" s="58" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H40" s="58" t="inlineStr">
+      <c r="H41" s="58" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="I40" s="59" t="n">
+      <c r="I41" s="59" t="n">
         <v>6</v>
       </c>
-      <c r="J40" s="58" t="inlineStr">
+      <c r="J41" s="58" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="K40" s="58" t="inlineStr">
+      <c r="K41" s="58" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L40" s="60" t="inlineStr">
+      <c r="L41" s="58" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M40" s="58" t="n"/>
-      <c r="N40" s="58" t="inlineStr"/>
+      <c r="M41" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N41" s="58" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="45" t="inlineStr">
-        <is>
-          <t>5. 18-Oct XD08: CO-14103 → 6; CO-14104 … CO-14108 new (rows in scan order)</t>
-        </is>
-      </c>
-      <c r="B42" s="46" t="n"/>
-      <c r="C42" s="46" t="n"/>
-      <c r="D42" s="46" t="n"/>
-      <c r="E42" s="46" t="n"/>
-      <c r="F42" s="46" t="n"/>
-      <c r="G42" s="46" t="n"/>
-      <c r="H42" s="46" t="n"/>
-      <c r="I42" s="46" t="n"/>
-      <c r="J42" s="46" t="n"/>
-      <c r="K42" s="46" t="n"/>
-      <c r="L42" s="46" t="n"/>
-      <c r="M42" s="46" t="n"/>
-      <c r="N42" s="46" t="n"/>
-      <c r="O42" s="46" t="n"/>
-      <c r="P42" s="46" t="n"/>
+      <c r="A42" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C42" s="49" t="inlineStr">
+        <is>
+          <t>CO-14105</t>
+        </is>
+      </c>
+      <c r="D42" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E42" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F42" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G42" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H42" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I42" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J42" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K42" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L42" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M42" s="49" t="n"/>
+      <c r="N42" s="49" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
-        </is>
-      </c>
-      <c r="D43" s="47" t="inlineStr">
-        <is>
-          <t>Replicated from DB Surrounding (G-System)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B44" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="C44" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="D44" s="42" t="inlineStr">
-        <is>
-          <t>ORDER_DT</t>
-        </is>
-      </c>
-      <c r="E44" s="42" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F44" s="42" t="inlineStr">
-        <is>
-          <t>DETAILED_ITEM_NO</t>
-        </is>
-      </c>
-      <c r="G44" s="42" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>SHIPPING_PART_NO</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS_QTY</t>
-        </is>
-      </c>
-      <c r="J44" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS</t>
-        </is>
-      </c>
-      <c r="K44" s="5" t="inlineStr">
-        <is>
-          <t>HOLD_FLAG</t>
-        </is>
-      </c>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t>PO_MAPPED_FLAG</t>
-        </is>
-      </c>
-      <c r="M44" s="5" t="inlineStr">
-        <is>
-          <t>UPD_STATUS</t>
-        </is>
-      </c>
-      <c r="N44" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
+      <c r="A43" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C43" s="49" t="inlineStr">
+        <is>
+          <t>CO-14106</t>
+        </is>
+      </c>
+      <c r="D43" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E43" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F43" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G43" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H43" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I43" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="J43" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K43" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L43" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M43" s="49" t="n"/>
+      <c r="N43" s="49" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C44" s="49" t="inlineStr">
+        <is>
+          <t>CO-14107</t>
+        </is>
+      </c>
+      <c r="D44" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E44" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F44" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G44" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H44" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I44" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="J44" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K44" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L44" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M44" s="49" t="n"/>
+      <c r="N44" s="49" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B45" s="58" t="inlineStr">
+      <c r="A45" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B45" s="49" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="C45" s="58" t="inlineStr">
-        <is>
-          <t>CO-14103</t>
-        </is>
-      </c>
-      <c r="D45" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="E45" s="58" t="inlineStr">
+      <c r="C45" s="49" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="D45" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E45" s="49" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="F45" s="58" t="inlineStr">
+      <c r="F45" s="49" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="G45" s="58" t="inlineStr">
+      <c r="G45" s="49" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H45" s="58" t="inlineStr">
+      <c r="H45" s="49" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="I45" s="59" t="n">
+      <c r="I45" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="J45" s="58" t="inlineStr">
+      <c r="J45" s="49" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="K45" s="58" t="inlineStr">
+      <c r="K45" s="49" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L45" s="58" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M45" s="60" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N45" s="58" t="inlineStr">
-        <is>
-          <t>Received</t>
+      <c r="L45" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M45" s="49" t="n"/>
+      <c r="N45" s="49" t="inlineStr">
+        <is>
+          <t>Middle row</t>
         </is>
       </c>
     </row>
@@ -11700,12 +11794,12 @@
       </c>
       <c r="B46" s="49" t="inlineStr">
         <is>
-          <t>9715300</t>
+          <t>9811100</t>
         </is>
       </c>
       <c r="C46" s="49" t="inlineStr">
         <is>
-          <t>CO-14105</t>
+          <t>CO-14109</t>
         </is>
       </c>
       <c r="D46" s="49" t="inlineStr">
@@ -11715,7 +11809,7 @@
       </c>
       <c r="E46" s="49" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>9811110</t>
         </is>
       </c>
       <c r="F46" s="49" t="inlineStr">
@@ -11762,12 +11856,12 @@
       </c>
       <c r="B47" s="49" t="inlineStr">
         <is>
-          <t>9715300</t>
+          <t>982200</t>
         </is>
       </c>
       <c r="C47" s="49" t="inlineStr">
         <is>
-          <t>CO-14106</t>
+          <t>CO-14110</t>
         </is>
       </c>
       <c r="D47" s="49" t="inlineStr">
@@ -11777,7 +11871,7 @@
       </c>
       <c r="E47" s="49" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>982220</t>
         </is>
       </c>
       <c r="F47" s="49" t="inlineStr">
@@ -11796,7 +11890,7 @@
         </is>
       </c>
       <c r="I47" s="53" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J47" s="49" t="inlineStr">
         <is>
@@ -11816,315 +11910,317 @@
       <c r="M47" s="49" t="n"/>
       <c r="N47" s="49" t="inlineStr"/>
     </row>
-    <row r="48">
-      <c r="A48" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B48" s="49" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="45" t="inlineStr">
+        <is>
+          <t>6. 18-Oct [Search] → XD09: 24 of 30 pcs with PO, case 5 Not Ready</t>
+        </is>
+      </c>
+      <c r="B49" s="46" t="n"/>
+      <c r="C49" s="46" t="n"/>
+      <c r="D49" s="46" t="n"/>
+      <c r="E49" s="46" t="n"/>
+      <c r="F49" s="46" t="n"/>
+      <c r="G49" s="46" t="n"/>
+      <c r="H49" s="46" t="n"/>
+      <c r="I49" s="46" t="n"/>
+      <c r="J49" s="46" t="n"/>
+      <c r="K49" s="46" t="n"/>
+      <c r="L49" s="46" t="n"/>
+      <c r="M49" s="46" t="n"/>
+      <c r="N49" s="46" t="n"/>
+      <c r="O49" s="46" t="n"/>
+      <c r="P49" s="46" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>#TEMP_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D50" s="47" t="inlineStr">
+        <is>
+          <t>Temporary (session)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>SORT_SEQ</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>OPEN_ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="inlineStr">
+        <is>
+          <t>ASSIGNED_QTY</t>
+        </is>
+      </c>
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="K51" s="9" t="inlineStr">
+        <is>
+          <t>CUM_DEST_QTY</t>
+        </is>
+      </c>
+      <c r="L51" s="9" t="inlineStr">
+        <is>
+          <t>SEQ_QTY</t>
+        </is>
+      </c>
+      <c r="M51" s="9" t="inlineStr">
+        <is>
+          <t>CUT_FLAG</t>
+        </is>
+      </c>
+      <c r="N51" s="9" t="inlineStr">
+        <is>
+          <t>GROUP_SEQ</t>
+        </is>
+      </c>
+      <c r="O51" s="9" t="inlineStr">
+        <is>
+          <t>CROSSDOCK_STATUS</t>
+        </is>
+      </c>
+      <c r="P51" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B52" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="64" t="inlineStr">
         <is>
           <t>9715300</t>
         </is>
       </c>
-      <c r="C48" s="49" t="inlineStr">
+      <c r="D52" s="64" t="inlineStr">
+        <is>
+          <t>CO-14105</t>
+        </is>
+      </c>
+      <c r="E52" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F52" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H52" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09012</t>
+        </is>
+      </c>
+      <c r="I52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J52" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L52" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M52" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N52" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P52" s="64" t="inlineStr">
+        <is>
+          <t>Cases 1-4 ticked → ASN0003</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B53" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D53" s="64" t="inlineStr">
+        <is>
+          <t>CO-14106</t>
+        </is>
+      </c>
+      <c r="E53" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F53" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G53" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="H53" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09013</t>
+        </is>
+      </c>
+      <c r="I53" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="J53" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K53" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="L53" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="M53" s="64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N53" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O53" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P53" s="64" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B54" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D54" s="64" t="inlineStr">
         <is>
           <t>CO-14107</t>
         </is>
       </c>
-      <c r="D48" s="49" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E48" s="49" t="inlineStr">
+      <c r="E54" s="64" t="inlineStr">
         <is>
           <t>9715310</t>
         </is>
       </c>
-      <c r="F48" s="49" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G48" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H48" s="49" t="inlineStr">
+      <c r="F54" s="64" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="I48" s="53" t="n">
+      <c r="G54" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="J48" s="49" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K48" s="49" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L48" s="49" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M48" s="49" t="n"/>
-      <c r="N48" s="49" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B49" s="49" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C49" s="49" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="D49" s="49" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E49" s="49" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F49" s="49" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G49" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H49" s="49" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I49" s="53" t="n">
+      <c r="H54" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09013</t>
+        </is>
+      </c>
+      <c r="I54" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="J54" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K54" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="L54" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="J49" s="49" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K49" s="49" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L49" s="49" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M49" s="49" t="n"/>
-      <c r="N49" s="49" t="inlineStr">
-        <is>
-          <t>Customer code 9722D10 after 9715300</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B50" s="49" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C50" s="49" t="inlineStr">
-        <is>
-          <t>CO-14108</t>
-        </is>
-      </c>
-      <c r="D50" s="49" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="E50" s="49" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F50" s="49" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G50" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H50" s="49" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I50" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="J50" s="49" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K50" s="49" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L50" s="49" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M50" s="49" t="n"/>
-      <c r="N50" s="49" t="inlineStr">
-        <is>
-          <t>Order date 18-Oct</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="45" t="inlineStr">
-        <is>
-          <t>6. 18-Oct [Search] → XD09 (unit 17-Oct: 3 cases Ready; unit 18-Oct: no PO)</t>
-        </is>
-      </c>
-      <c r="B52" s="46" t="n"/>
-      <c r="C52" s="46" t="n"/>
-      <c r="D52" s="46" t="n"/>
-      <c r="E52" s="46" t="n"/>
-      <c r="F52" s="46" t="n"/>
-      <c r="G52" s="46" t="n"/>
-      <c r="H52" s="46" t="n"/>
-      <c r="I52" s="46" t="n"/>
-      <c r="J52" s="46" t="n"/>
-      <c r="K52" s="46" t="n"/>
-      <c r="L52" s="46" t="n"/>
-      <c r="M52" s="46" t="n"/>
-      <c r="N52" s="46" t="n"/>
-      <c r="O52" s="46" t="n"/>
-      <c r="P52" s="46" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="35" t="inlineStr">
-        <is>
-          <t>#TEMP_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D53" s="47" t="inlineStr">
-        <is>
-          <t>Temporary (session)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="26" customHeight="1">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>SORT_SEQ</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="G54" s="9" t="inlineStr">
-        <is>
-          <t>OPEN_ORDER_QTY</t>
-        </is>
-      </c>
-      <c r="H54" s="9" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="I54" s="9" t="inlineStr">
-        <is>
-          <t>ASSIGNED_QTY</t>
-        </is>
-      </c>
-      <c r="J54" s="9" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="K54" s="9" t="inlineStr">
-        <is>
-          <t>CUM_DEST_QTY</t>
-        </is>
-      </c>
-      <c r="L54" s="9" t="inlineStr">
-        <is>
-          <t>SEQ_QTY</t>
-        </is>
-      </c>
-      <c r="M54" s="9" t="inlineStr">
-        <is>
-          <t>CUT_FLAG</t>
-        </is>
-      </c>
-      <c r="N54" s="9" t="inlineStr">
-        <is>
-          <t>GROUP_SEQ</t>
-        </is>
-      </c>
-      <c r="O54" s="9" t="inlineStr">
-        <is>
-          <t>CROSSDOCK_STATUS</t>
-        </is>
-      </c>
-      <c r="P54" s="9" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
+      <c r="M54" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N54" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O54" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P54" s="64" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="62" t="inlineStr">
@@ -12133,21 +12229,21 @@
         </is>
       </c>
       <c r="B55" s="63" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C55" s="64" t="inlineStr">
         <is>
-          <t>9715300</t>
+          <t>9722D10</t>
         </is>
       </c>
       <c r="D55" s="64" t="inlineStr">
         <is>
-          <t>CO-14105</t>
+          <t>CO-14104</t>
         </is>
       </c>
       <c r="E55" s="64" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>9722D10</t>
         </is>
       </c>
       <c r="F55" s="64" t="inlineStr">
@@ -12167,7 +12263,7 @@
         <v>6</v>
       </c>
       <c r="J55" s="63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K55" s="63" t="n">
         <v>6</v>
@@ -12181,7 +12277,7 @@
         </is>
       </c>
       <c r="N55" s="63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O55" s="49" t="inlineStr">
         <is>
@@ -12190,7 +12286,7 @@
       </c>
       <c r="P55" s="64" t="inlineStr">
         <is>
-          <t>Cases 1-3 ticked → ASN0003</t>
+          <t>Middle row</t>
         </is>
       </c>
     </row>
@@ -12201,21 +12297,21 @@
         </is>
       </c>
       <c r="B56" s="63" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C56" s="64" t="inlineStr">
         <is>
-          <t>9715300</t>
+          <t>9811100</t>
         </is>
       </c>
       <c r="D56" s="64" t="inlineStr">
         <is>
-          <t>CO-14106</t>
+          <t>CO-14109</t>
         </is>
       </c>
       <c r="E56" s="64" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>9811110</t>
         </is>
       </c>
       <c r="F56" s="64" t="inlineStr">
@@ -12224,32 +12320,32 @@
         </is>
       </c>
       <c r="G56" s="63" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H56" s="64" t="inlineStr">
         <is>
-          <t>PO-DMY-09014</t>
+          <t>PO-DMY-09013</t>
         </is>
       </c>
       <c r="I56" s="63" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J56" s="63" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K56" s="63" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L56" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="M56" s="64" t="inlineStr">
-        <is>
-          <t>N</t>
+        <v>6</v>
+      </c>
+      <c r="M56" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="N56" s="63" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O56" s="49" t="inlineStr">
         <is>
@@ -12265,21 +12361,21 @@
         </is>
       </c>
       <c r="B57" s="63" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C57" s="64" t="inlineStr">
         <is>
-          <t>9715300</t>
+          <t>982200</t>
         </is>
       </c>
       <c r="D57" s="64" t="inlineStr">
         <is>
-          <t>CO-14107</t>
+          <t>CO-14110</t>
         </is>
       </c>
       <c r="E57" s="64" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>982220</t>
         </is>
       </c>
       <c r="F57" s="64" t="inlineStr">
@@ -12288,21 +12384,17 @@
         </is>
       </c>
       <c r="G57" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="H57" s="64" t="inlineStr">
-        <is>
-          <t>PO-DMY-09014</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="H57" s="64" t="n"/>
       <c r="I57" s="63" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J57" s="63" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K57" s="63" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L57" s="63" t="n">
         <v>6</v>
@@ -12313,253 +12405,259 @@
         </is>
       </c>
       <c r="N57" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="O57" s="66" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="P57" s="64" t="inlineStr">
+        <is>
+          <t>Not Ready (PO short)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="45" t="inlineStr">
+        <is>
+          <t>7. 18-Oct ASN0003 = cases 1-4</t>
+        </is>
+      </c>
+      <c r="B59" s="46" t="n"/>
+      <c r="C59" s="46" t="n"/>
+      <c r="D59" s="46" t="n"/>
+      <c r="E59" s="46" t="n"/>
+      <c r="F59" s="46" t="n"/>
+      <c r="G59" s="46" t="n"/>
+      <c r="H59" s="46" t="n"/>
+      <c r="I59" s="46" t="n"/>
+      <c r="J59" s="46" t="n"/>
+      <c r="K59" s="46" t="n"/>
+      <c r="L59" s="46" t="n"/>
+      <c r="M59" s="46" t="n"/>
+      <c r="N59" s="46" t="n"/>
+      <c r="O59" s="46" t="n"/>
+      <c r="P59" s="46" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D60" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="26" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B61" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N61" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O61" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B62" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C62" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F62" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G62" s="49" t="inlineStr">
+        <is>
+          <t>CO-14105</t>
+        </is>
+      </c>
+      <c r="H62" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I62" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J62" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09012</t>
+        </is>
+      </c>
+      <c r="K62" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09012</t>
+        </is>
+      </c>
+      <c r="L62" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M62" s="49" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N62" s="49" t="inlineStr">
+        <is>
+          <t>C-0003-01</t>
+        </is>
+      </c>
+      <c r="O62" s="49" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B63" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="C63" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="O57" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="P57" s="64" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B58" s="63" t="n">
-        <v>4</v>
-      </c>
-      <c r="C58" s="64" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="D58" s="64" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="E58" s="64" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F58" s="64" t="inlineStr">
+      <c r="D63" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="49" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="G58" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="H58" s="64" t="inlineStr">
-        <is>
-          <t>PO-DMY-09014</t>
-        </is>
-      </c>
-      <c r="I58" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="J58" s="63" t="n">
+      <c r="F63" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G63" s="49" t="inlineStr">
+        <is>
+          <t>CO-14106</t>
+        </is>
+      </c>
+      <c r="H63" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I63" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="K58" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="L58" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="M58" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N58" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="O58" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="P58" s="64" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="62" t="inlineStr">
-        <is>
-          <t>TEMP</t>
-        </is>
-      </c>
-      <c r="B59" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="C59" s="64" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="D59" s="64" t="inlineStr">
-        <is>
-          <t>CO-14108</t>
-        </is>
-      </c>
-      <c r="E59" s="64" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F59" s="64" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="G59" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="H59" s="64" t="n"/>
-      <c r="I59" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="J59" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="K59" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="L59" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="M59" s="65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N59" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="O59" s="66" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="P59" s="64" t="inlineStr">
-        <is>
-          <t>Not Ready (no PO left)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="45" t="inlineStr">
-        <is>
-          <t>7. 18-Oct ASN0003 = cases 1-3 (whole order date 17-Oct)</t>
-        </is>
-      </c>
-      <c r="B61" s="46" t="n"/>
-      <c r="C61" s="46" t="n"/>
-      <c r="D61" s="46" t="n"/>
-      <c r="E61" s="46" t="n"/>
-      <c r="F61" s="46" t="n"/>
-      <c r="G61" s="46" t="n"/>
-      <c r="H61" s="46" t="n"/>
-      <c r="I61" s="46" t="n"/>
-      <c r="J61" s="46" t="n"/>
-      <c r="K61" s="46" t="n"/>
-      <c r="L61" s="46" t="n"/>
-      <c r="M61" s="46" t="n"/>
-      <c r="N61" s="46" t="n"/>
-      <c r="O61" s="46" t="n"/>
-      <c r="P61" s="46" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D62" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B63" s="42" t="inlineStr">
-        <is>
-          <t>INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>LINE_SEQ</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="I63" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="K63" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="L63" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="M63" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="N63" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
-        </is>
-      </c>
-      <c r="O63" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
+      <c r="J63" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09013</t>
+        </is>
+      </c>
+      <c r="K63" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09013</t>
+        </is>
+      </c>
+      <c r="L63" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M63" s="49" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N63" s="49" t="inlineStr">
+        <is>
+          <t>C-0003-02</t>
+        </is>
+      </c>
+      <c r="O63" s="49" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="48" t="inlineStr">
@@ -12568,37 +12666,37 @@
         </is>
       </c>
       <c r="B64" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="C64" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F64" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G64" s="49" t="inlineStr">
+        <is>
+          <t>CO-14107</t>
+        </is>
+      </c>
+      <c r="H64" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I64" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="C64" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" s="49" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="F64" s="49" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="G64" s="49" t="inlineStr">
-        <is>
-          <t>CO-14105</t>
-        </is>
-      </c>
-      <c r="H64" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="I64" s="53" t="n">
-        <v>6</v>
-      </c>
       <c r="J64" s="49" t="inlineStr">
         <is>
           <t>PO-DMY-09013</t>
@@ -12621,7 +12719,7 @@
       </c>
       <c r="N64" s="49" t="inlineStr">
         <is>
-          <t>C-0003-01</t>
+          <t>C-0003-02</t>
         </is>
       </c>
       <c r="O64" s="49" t="inlineStr"/>
@@ -12633,10 +12731,10 @@
         </is>
       </c>
       <c r="B65" s="53" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C65" s="53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D65" s="53" t="n">
         <v>1</v>
@@ -12648,12 +12746,12 @@
       </c>
       <c r="F65" s="49" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>9722D10</t>
         </is>
       </c>
       <c r="G65" s="49" t="inlineStr">
         <is>
-          <t>CO-14106</t>
+          <t>CO-14104</t>
         </is>
       </c>
       <c r="H65" s="49" t="inlineStr">
@@ -12662,16 +12760,16 @@
         </is>
       </c>
       <c r="I65" s="53" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J65" s="49" t="inlineStr">
         <is>
-          <t>PO-DMY-09014</t>
+          <t>PO-DMY-09013</t>
         </is>
       </c>
       <c r="K65" s="49" t="inlineStr">
         <is>
-          <t>MF-DMY-09014</t>
+          <t>MF-DMY-09013</t>
         </is>
       </c>
       <c r="L65" s="49" t="inlineStr">
@@ -12686,7 +12784,7 @@
       </c>
       <c r="N65" s="49" t="inlineStr">
         <is>
-          <t>C-0003-02</t>
+          <t>C-0003-03</t>
         </is>
       </c>
       <c r="O65" s="49" t="inlineStr"/>
@@ -12698,13 +12796,13 @@
         </is>
       </c>
       <c r="B66" s="53" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C66" s="53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D66" s="53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E66" s="49" t="inlineStr">
         <is>
@@ -12713,12 +12811,12 @@
       </c>
       <c r="F66" s="49" t="inlineStr">
         <is>
-          <t>9715310</t>
+          <t>9811110</t>
         </is>
       </c>
       <c r="G66" s="49" t="inlineStr">
         <is>
-          <t>CO-14107</t>
+          <t>CO-14109</t>
         </is>
       </c>
       <c r="H66" s="49" t="inlineStr">
@@ -12727,16 +12825,16 @@
         </is>
       </c>
       <c r="I66" s="53" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J66" s="49" t="inlineStr">
         <is>
-          <t>PO-DMY-09014</t>
+          <t>PO-DMY-09013</t>
         </is>
       </c>
       <c r="K66" s="49" t="inlineStr">
         <is>
-          <t>MF-DMY-09014</t>
+          <t>MF-DMY-09013</t>
         </is>
       </c>
       <c r="L66" s="49" t="inlineStr">
@@ -12751,773 +12849,651 @@
       </c>
       <c r="N66" s="49" t="inlineStr">
         <is>
-          <t>C-0003-02</t>
+          <t>C-0003-04</t>
         </is>
       </c>
       <c r="O66" s="49" t="inlineStr"/>
     </row>
-    <row r="67">
-      <c r="A67" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B67" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="C67" s="53" t="n">
-        <v>3</v>
-      </c>
-      <c r="D67" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E67" s="49" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="F67" s="49" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="G67" s="49" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="H67" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="I67" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="J67" s="49" t="inlineStr">
-        <is>
-          <t>PO-DMY-09014</t>
-        </is>
-      </c>
-      <c r="K67" s="49" t="inlineStr">
-        <is>
-          <t>MF-DMY-09014</t>
-        </is>
-      </c>
-      <c r="L67" s="49" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="M67" s="49" t="inlineStr">
-        <is>
-          <t>ASN0003</t>
-        </is>
-      </c>
-      <c r="N67" s="49" t="inlineStr">
-        <is>
-          <t>C-0003-03</t>
-        </is>
-      </c>
-      <c r="O67" s="49" t="inlineStr"/>
+    <row r="68">
+      <c r="A68" s="45" t="inlineStr">
+        <is>
+          <t>8. 19-Oct XD08: ASN0003 received, CO-14104 → 2 (middle row, in case 3); split PO-DMY-09014 (PO_DT 19-Oct, 12)</t>
+        </is>
+      </c>
+      <c r="B68" s="46" t="n"/>
+      <c r="C68" s="46" t="n"/>
+      <c r="D68" s="46" t="n"/>
+      <c r="E68" s="46" t="n"/>
+      <c r="F68" s="46" t="n"/>
+      <c r="G68" s="46" t="n"/>
+      <c r="H68" s="46" t="n"/>
+      <c r="I68" s="46" t="n"/>
+      <c r="J68" s="46" t="n"/>
+      <c r="K68" s="46" t="n"/>
+      <c r="L68" s="46" t="n"/>
+      <c r="M68" s="46" t="n"/>
+      <c r="N68" s="46" t="n"/>
+      <c r="O68" s="46" t="n"/>
+      <c r="P68" s="46" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="35" t="inlineStr">
         <is>
-          <t>TB_R_PRA_DAILY_ORDER_MAPPED</t>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
       <c r="D69" s="47" t="inlineStr">
         <is>
-          <t>New table (Crossdock)</t>
+          <t>Replicated from DB Surrounding (G-System)</t>
         </is>
       </c>
     </row>
     <row r="70" ht="26" customHeight="1">
-      <c r="A70" s="3" t="inlineStr">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
       <c r="B70" s="42" t="inlineStr">
         <is>
-          <t>PO_NO</t>
+          <t>CUSTOMER_CD</t>
         </is>
       </c>
       <c r="C70" s="42" t="inlineStr">
         <is>
-          <t>MANIFEST_NO</t>
+          <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
       <c r="D70" s="42" t="inlineStr">
         <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>ORDER_QTY</t>
-        </is>
-      </c>
-      <c r="G70" s="3" t="inlineStr">
-        <is>
-          <t>MAPPED_QTY</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E70" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F70" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G70" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M70" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N70" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B71" s="49" t="inlineStr">
-        <is>
-          <t>PO-DMY-09013</t>
-        </is>
-      </c>
-      <c r="C71" s="49" t="inlineStr">
-        <is>
-          <t>MF-DMY-09013</t>
-        </is>
-      </c>
-      <c r="D71" s="49" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="E71" s="49" t="inlineStr">
+      <c r="A71" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B71" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C71" s="58" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="D71" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E71" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F71" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G71" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H71" s="58" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="F71" s="53" t="n">
+      <c r="I71" s="59" t="n">
         <v>6</v>
       </c>
-      <c r="G71" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="H71" s="49" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B72" s="49" t="inlineStr">
-        <is>
-          <t>PO-DMY-09014</t>
-        </is>
-      </c>
-      <c r="C72" s="49" t="inlineStr">
-        <is>
-          <t>MF-DMY-09014</t>
-        </is>
-      </c>
-      <c r="D72" s="49" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="E72" s="49" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="F72" s="53" t="n">
-        <v>12</v>
-      </c>
-      <c r="G72" s="53" t="n">
-        <v>12</v>
-      </c>
-      <c r="H72" s="49" t="inlineStr"/>
+      <c r="J71" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K71" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L71" s="58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M71" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N71" s="58" t="inlineStr">
+        <is>
+          <t>Cancel after ASN: LOG5, listed in XD11 (waiting for a candidate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="45" t="inlineStr">
+        <is>
+          <t>9. 19-Oct CO-14110 → ASN0004 with the split PO</t>
+        </is>
+      </c>
+      <c r="B73" s="46" t="n"/>
+      <c r="C73" s="46" t="n"/>
+      <c r="D73" s="46" t="n"/>
+      <c r="E73" s="46" t="n"/>
+      <c r="F73" s="46" t="n"/>
+      <c r="G73" s="46" t="n"/>
+      <c r="H73" s="46" t="n"/>
+      <c r="I73" s="46" t="n"/>
+      <c r="J73" s="46" t="n"/>
+      <c r="K73" s="46" t="n"/>
+      <c r="L73" s="46" t="n"/>
+      <c r="M73" s="46" t="n"/>
+      <c r="N73" s="46" t="n"/>
+      <c r="O73" s="46" t="n"/>
+      <c r="P73" s="46" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="35" t="inlineStr">
         <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D74" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="26" customHeight="1">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B75" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N75" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O75" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B76" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="C76" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F76" s="49" t="inlineStr">
+        <is>
+          <t>982220</t>
+        </is>
+      </c>
+      <c r="G76" s="49" t="inlineStr">
+        <is>
+          <t>CO-14110</t>
+        </is>
+      </c>
+      <c r="H76" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I76" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J76" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="K76" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09014</t>
+        </is>
+      </c>
+      <c r="L76" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M76" s="49" t="inlineStr">
+        <is>
+          <t>ASN0004</t>
+        </is>
+      </c>
+      <c r="N76" s="49" t="inlineStr">
+        <is>
+          <t>C-0004-01</t>
+        </is>
+      </c>
+      <c r="O76" s="49" t="inlineStr">
+        <is>
+          <t>6 pcs of the split PO stay open</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="45" t="inlineStr">
+        <is>
+          <t>10. 20-Oct XD08: CO-14111 new (order date 19-Oct, PO-DMY-09015); 21-Oct → 6 (pcs of case 3 allocated by G-System)</t>
+        </is>
+      </c>
+      <c r="B78" s="46" t="n"/>
+      <c r="C78" s="46" t="n"/>
+      <c r="D78" s="46" t="n"/>
+      <c r="E78" s="46" t="n"/>
+      <c r="F78" s="46" t="n"/>
+      <c r="G78" s="46" t="n"/>
+      <c r="H78" s="46" t="n"/>
+      <c r="I78" s="46" t="n"/>
+      <c r="J78" s="46" t="n"/>
+      <c r="K78" s="46" t="n"/>
+      <c r="L78" s="46" t="n"/>
+      <c r="M78" s="46" t="n"/>
+      <c r="N78" s="46" t="n"/>
+      <c r="O78" s="46" t="n"/>
+      <c r="P78" s="46" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="35" t="inlineStr">
+        <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
-      <c r="D74" s="47" t="inlineStr">
+      <c r="D79" s="47" t="inlineStr">
         <is>
           <t>Replicated from DB Surrounding (G-System)</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="5" t="inlineStr">
+    <row r="80" ht="26" customHeight="1">
+      <c r="A80" s="5" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B75" s="42" t="inlineStr">
+      <c r="B80" s="42" t="inlineStr">
         <is>
           <t>CUSTOMER_CD</t>
         </is>
       </c>
-      <c r="C75" s="42" t="inlineStr">
+      <c r="C80" s="42" t="inlineStr">
         <is>
           <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="D75" s="42" t="inlineStr">
+      <c r="D80" s="42" t="inlineStr">
         <is>
           <t>ORDER_DT</t>
         </is>
       </c>
-      <c r="E75" s="42" t="inlineStr">
+      <c r="E80" s="42" t="inlineStr">
         <is>
           <t>DESTINATION_CD</t>
         </is>
       </c>
-      <c r="F75" s="42" t="inlineStr">
+      <c r="F80" s="42" t="inlineStr">
         <is>
           <t>DETAILED_ITEM_NO</t>
         </is>
       </c>
-      <c r="G75" s="42" t="inlineStr">
+      <c r="G80" s="42" t="inlineStr">
         <is>
           <t>SERIAL_NO</t>
         </is>
       </c>
-      <c r="H75" s="5" t="inlineStr">
+      <c r="H80" s="5" t="inlineStr">
         <is>
           <t>SHIPPING_PART_NO</t>
         </is>
       </c>
-      <c r="I75" s="5" t="inlineStr">
+      <c r="I80" s="5" t="inlineStr">
         <is>
           <t>ORDER_STATUS_QTY</t>
         </is>
       </c>
-      <c r="J75" s="5" t="inlineStr">
+      <c r="J80" s="5" t="inlineStr">
         <is>
           <t>ORDER_STATUS</t>
         </is>
       </c>
-      <c r="K75" s="5" t="inlineStr">
+      <c r="K80" s="5" t="inlineStr">
         <is>
           <t>HOLD_FLAG</t>
         </is>
       </c>
-      <c r="L75" s="5" t="inlineStr">
+      <c r="L80" s="5" t="inlineStr">
         <is>
           <t>PO_MAPPED_FLAG</t>
         </is>
       </c>
-      <c r="M75" s="5" t="inlineStr">
+      <c r="M80" s="5" t="inlineStr">
         <is>
           <t>UPD_STATUS</t>
         </is>
       </c>
-      <c r="N75" s="5" t="inlineStr">
+      <c r="N80" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="57" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="57" t="inlineStr">
         <is>
           <t>UPD</t>
         </is>
       </c>
-      <c r="B76" s="58" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C76" s="58" t="inlineStr">
-        <is>
-          <t>CO-14105</t>
-        </is>
-      </c>
-      <c r="D76" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E76" s="58" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F76" s="58" t="inlineStr">
+      <c r="B81" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C81" s="58" t="inlineStr">
+        <is>
+          <t>CO-14111</t>
+        </is>
+      </c>
+      <c r="D81" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E81" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F81" s="58" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="G76" s="58" t="inlineStr">
+      <c r="G81" s="58" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H76" s="58" t="inlineStr">
+      <c r="H81" s="58" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="I76" s="59" t="n">
+      <c r="I81" s="59" t="n">
         <v>6</v>
       </c>
-      <c r="J76" s="58" t="inlineStr">
+      <c r="J81" s="58" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="K76" s="58" t="inlineStr">
+      <c r="K81" s="58" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L76" s="60" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M76" s="58" t="n"/>
-      <c r="N76" s="58" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B77" s="58" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C77" s="58" t="inlineStr">
-        <is>
-          <t>CO-14106</t>
-        </is>
-      </c>
-      <c r="D77" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E77" s="58" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F77" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G77" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H77" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I77" s="59" t="n">
-        <v>3</v>
-      </c>
-      <c r="J77" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K77" s="58" t="inlineStr">
+      <c r="L81" s="58" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L77" s="60" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M77" s="58" t="n"/>
-      <c r="N77" s="58" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B78" s="58" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C78" s="58" t="inlineStr">
-        <is>
-          <t>CO-14107</t>
-        </is>
-      </c>
-      <c r="D78" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E78" s="58" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F78" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G78" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H78" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I78" s="59" t="n">
-        <v>3</v>
-      </c>
-      <c r="J78" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K78" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L78" s="60" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M78" s="58" t="n"/>
-      <c r="N78" s="58" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B79" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C79" s="58" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="D79" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E79" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F79" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G79" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H79" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I79" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="J79" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K79" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L79" s="60" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M79" s="58" t="n"/>
-      <c r="N79" s="58" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="45" t="inlineStr">
-        <is>
-          <t>8. 19-Oct XD08: ASN0003 received, CO-14104 → 2 (in case 3), CO-14108 → 6</t>
-        </is>
-      </c>
-      <c r="B81" s="46" t="n"/>
-      <c r="C81" s="46" t="n"/>
-      <c r="D81" s="46" t="n"/>
-      <c r="E81" s="46" t="n"/>
-      <c r="F81" s="46" t="n"/>
-      <c r="G81" s="46" t="n"/>
-      <c r="H81" s="46" t="n"/>
-      <c r="I81" s="46" t="n"/>
-      <c r="J81" s="46" t="n"/>
-      <c r="K81" s="46" t="n"/>
-      <c r="L81" s="46" t="n"/>
-      <c r="M81" s="46" t="n"/>
-      <c r="N81" s="46" t="n"/>
-      <c r="O81" s="46" t="n"/>
-      <c r="P81" s="46" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
-        </is>
-      </c>
-      <c r="D82" s="47" t="inlineStr">
-        <is>
-          <t>Replicated from DB Surrounding (G-System)</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="26" customHeight="1">
-      <c r="A83" s="5" t="inlineStr">
+      <c r="M81" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N81" s="58" t="inlineStr">
+        <is>
+          <t>Received without ASN: candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="45" t="inlineStr">
+        <is>
+          <t>11. 21-Oct XD11 Change Order Number: ASN0003 case 3 → CO-14111</t>
+        </is>
+      </c>
+      <c r="B83" s="46" t="n"/>
+      <c r="C83" s="46" t="n"/>
+      <c r="D83" s="46" t="n"/>
+      <c r="E83" s="46" t="n"/>
+      <c r="F83" s="46" t="n"/>
+      <c r="G83" s="46" t="n"/>
+      <c r="H83" s="46" t="n"/>
+      <c r="I83" s="46" t="n"/>
+      <c r="J83" s="46" t="n"/>
+      <c r="K83" s="46" t="n"/>
+      <c r="L83" s="46" t="n"/>
+      <c r="M83" s="46" t="n"/>
+      <c r="N83" s="46" t="n"/>
+      <c r="O83" s="46" t="n"/>
+      <c r="P83" s="46" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D84" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="26" customHeight="1">
+      <c r="A85" s="3" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B83" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="C83" s="42" t="inlineStr">
+      <c r="B85" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
         <is>
           <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="D83" s="42" t="inlineStr">
-        <is>
-          <t>ORDER_DT</t>
-        </is>
-      </c>
-      <c r="E83" s="42" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F83" s="42" t="inlineStr">
-        <is>
-          <t>DETAILED_ITEM_NO</t>
-        </is>
-      </c>
-      <c r="G83" s="42" t="inlineStr">
+      <c r="H85" s="3" t="inlineStr">
         <is>
           <t>SERIAL_NO</t>
         </is>
       </c>
-      <c r="H83" s="5" t="inlineStr">
-        <is>
-          <t>SHIPPING_PART_NO</t>
-        </is>
-      </c>
-      <c r="I83" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS_QTY</t>
-        </is>
-      </c>
-      <c r="J83" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS</t>
-        </is>
-      </c>
-      <c r="K83" s="5" t="inlineStr">
-        <is>
-          <t>HOLD_FLAG</t>
-        </is>
-      </c>
-      <c r="L83" s="5" t="inlineStr">
-        <is>
-          <t>PO_MAPPED_FLAG</t>
-        </is>
-      </c>
-      <c r="M83" s="5" t="inlineStr">
-        <is>
-          <t>UPD_STATUS</t>
-        </is>
-      </c>
-      <c r="N83" s="5" t="inlineStr">
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L85" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M85" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N85" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O85" s="3" t="inlineStr">
         <is>
           <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B84" s="58" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C84" s="58" t="inlineStr">
-        <is>
-          <t>CO-14105</t>
-        </is>
-      </c>
-      <c r="D84" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E84" s="58" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F84" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G84" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H84" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I84" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="J84" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K84" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L84" s="58" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M84" s="60" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N84" s="58" t="inlineStr">
-        <is>
-          <t>Received</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B85" s="58" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C85" s="58" t="inlineStr">
-        <is>
-          <t>CO-14106</t>
-        </is>
-      </c>
-      <c r="D85" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E85" s="58" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F85" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G85" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H85" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I85" s="59" t="n">
-        <v>3</v>
-      </c>
-      <c r="J85" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K85" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L85" s="58" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M85" s="60" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N85" s="58" t="inlineStr">
-        <is>
-          <t>Received</t>
         </is>
       </c>
     </row>
@@ -13527,747 +13503,426 @@
           <t>UPD</t>
         </is>
       </c>
-      <c r="B86" s="58" t="inlineStr">
-        <is>
-          <t>9715300</t>
-        </is>
-      </c>
-      <c r="C86" s="58" t="inlineStr">
-        <is>
-          <t>CO-14107</t>
-        </is>
-      </c>
-      <c r="D86" s="58" t="inlineStr">
+      <c r="B86" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="C86" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D86" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F86" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="G86" s="60" t="inlineStr">
+        <is>
+          <t>CO-14111</t>
+        </is>
+      </c>
+      <c r="H86" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I86" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J86" s="58" t="inlineStr">
+        <is>
+          <t>PO-DMY-09013</t>
+        </is>
+      </c>
+      <c r="K86" s="58" t="inlineStr">
+        <is>
+          <t>MF-DMY-09013</t>
+        </is>
+      </c>
+      <c r="L86" s="58" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M86" s="58" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N86" s="58" t="inlineStr">
+        <is>
+          <t>C-0003-03</t>
+        </is>
+      </c>
+      <c r="O86" s="58" t="inlineStr">
+        <is>
+          <t>Whole row moved; case, PO and ASN not changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D88" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="26" customHeight="1">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B89" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C89" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D89" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E89" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F89" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G89" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J89" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K89" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L89" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M89" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N89" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B90" s="51" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C90" s="51" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="D90" s="51" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="E86" s="58" t="inlineStr">
-        <is>
-          <t>9715310</t>
-        </is>
-      </c>
-      <c r="F86" s="58" t="inlineStr">
+      <c r="E90" s="51" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F90" s="51" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="G86" s="58" t="inlineStr">
+      <c r="G90" s="51" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H86" s="58" t="inlineStr">
+      <c r="H90" s="51" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="I86" s="59" t="n">
-        <v>3</v>
-      </c>
-      <c r="J86" s="58" t="inlineStr">
+      <c r="I90" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="J90" s="51" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="K86" s="58" t="inlineStr">
+      <c r="K90" s="51" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L86" s="58" t="inlineStr">
+      <c r="L90" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M86" s="60" t="inlineStr">
+      <c r="M90" s="66" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N90" s="51" t="inlineStr">
+        <is>
+          <t>Not changed (PO_MAPPED_FLAG stays Y)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B91" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C91" s="58" t="inlineStr">
+        <is>
+          <t>CO-14111</t>
+        </is>
+      </c>
+      <c r="D91" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E91" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F91" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G91" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H91" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I91" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J91" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K91" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L91" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M91" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="N86" s="58" t="inlineStr">
-        <is>
-          <t>Received</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B87" s="58" t="inlineStr">
+      <c r="N91" s="58" t="inlineStr">
+        <is>
+          <t>PO and ASN through ASN0003</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="35" t="inlineStr">
+        <is>
+          <t>TB_H_CROSSDOCK_ORDER_CHANGE</t>
+        </is>
+      </c>
+      <c r="D93" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="26" customHeight="1">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B94" s="42" t="inlineStr">
+        <is>
+          <t>HIST_ID</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>FROM_CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>FROM_SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>TO_CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>TO_DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr">
+        <is>
+          <t>FROM_INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="L94" s="3" t="inlineStr">
+        <is>
+          <t>TO_INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B95" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" s="49" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="D95" s="49" t="inlineStr">
+        <is>
+          <t>C-0003-03</t>
+        </is>
+      </c>
+      <c r="E95" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F95" s="49" t="inlineStr">
+        <is>
+          <t>CO-14104</t>
+        </is>
+      </c>
+      <c r="G95" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H95" s="49" t="inlineStr">
+        <is>
+          <t>CO-14111</t>
+        </is>
+      </c>
+      <c r="I95" s="49" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="C87" s="58" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="D87" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E87" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F87" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G87" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H87" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I87" s="59" t="n">
+      <c r="J95" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="J87" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K87" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L87" s="58" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M87" s="60" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N87" s="58" t="inlineStr">
-        <is>
-          <t>Cancel after ASN: LOG5, listed in XD11; ASN not changed</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B88" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C88" s="58" t="inlineStr">
-        <is>
-          <t>CO-14108</t>
-        </is>
-      </c>
-      <c r="D88" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="E88" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F88" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G88" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H88" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I88" s="59" t="n">
+      <c r="K95" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="J88" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K88" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L88" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M88" s="60" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N88" s="58" t="inlineStr">
-        <is>
-          <t>Received without ASN (pcs of case 3 allocated by G-System): candidate</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="45" t="inlineStr">
-        <is>
-          <t>9. 19-Oct XD11 Change Order Number: ASN0003 case 3 → CO-14108</t>
-        </is>
-      </c>
-      <c r="B90" s="46" t="n"/>
-      <c r="C90" s="46" t="n"/>
-      <c r="D90" s="46" t="n"/>
-      <c r="E90" s="46" t="n"/>
-      <c r="F90" s="46" t="n"/>
-      <c r="G90" s="46" t="n"/>
-      <c r="H90" s="46" t="n"/>
-      <c r="I90" s="46" t="n"/>
-      <c r="J90" s="46" t="n"/>
-      <c r="K90" s="46" t="n"/>
-      <c r="L90" s="46" t="n"/>
-      <c r="M90" s="46" t="n"/>
-      <c r="N90" s="46" t="n"/>
-      <c r="O90" s="46" t="n"/>
-      <c r="P90" s="46" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D91" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="26" customHeight="1">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B92" s="42" t="inlineStr">
-        <is>
-          <t>INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="C92" s="3" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>LINE_SEQ</t>
-        </is>
-      </c>
-      <c r="E92" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F92" s="3" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="G92" s="3" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="H92" s="3" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="I92" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="J92" s="3" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="K92" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="L92" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="M92" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="N92" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
-        </is>
-      </c>
-      <c r="O92" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B93" s="59" t="n">
+      <c r="L95" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="C93" s="59" t="n">
-        <v>3</v>
-      </c>
-      <c r="D93" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E93" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="F93" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="G93" s="60" t="inlineStr">
-        <is>
-          <t>CO-14108</t>
-        </is>
-      </c>
-      <c r="H93" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="I93" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="J93" s="58" t="inlineStr">
-        <is>
-          <t>PO-DMY-09014</t>
-        </is>
-      </c>
-      <c r="K93" s="58" t="inlineStr">
-        <is>
-          <t>MF-DMY-09014</t>
-        </is>
-      </c>
-      <c r="L93" s="58" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="M93" s="58" t="inlineStr">
-        <is>
-          <t>ASN0003</t>
-        </is>
-      </c>
-      <c r="N93" s="58" t="inlineStr">
-        <is>
-          <t>C-0003-03</t>
-        </is>
-      </c>
-      <c r="O93" s="58" t="inlineStr">
-        <is>
-          <t>Whole row moved; case, PO and ASN not changed</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
-        </is>
-      </c>
-      <c r="D95" s="47" t="inlineStr">
-        <is>
-          <t>Replicated from DB Surrounding (G-System)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="26" customHeight="1">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B96" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="C96" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="D96" s="42" t="inlineStr">
-        <is>
-          <t>ORDER_DT</t>
-        </is>
-      </c>
-      <c r="E96" s="42" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F96" s="42" t="inlineStr">
-        <is>
-          <t>DETAILED_ITEM_NO</t>
-        </is>
-      </c>
-      <c r="G96" s="42" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="H96" s="5" t="inlineStr">
-        <is>
-          <t>SHIPPING_PART_NO</t>
-        </is>
-      </c>
-      <c r="I96" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS_QTY</t>
-        </is>
-      </c>
-      <c r="J96" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS</t>
-        </is>
-      </c>
-      <c r="K96" s="5" t="inlineStr">
-        <is>
-          <t>HOLD_FLAG</t>
-        </is>
-      </c>
-      <c r="L96" s="5" t="inlineStr">
-        <is>
-          <t>PO_MAPPED_FLAG</t>
-        </is>
-      </c>
-      <c r="M96" s="5" t="inlineStr">
-        <is>
-          <t>UPD_STATUS</t>
-        </is>
-      </c>
-      <c r="N96" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="50" t="inlineStr">
-        <is>
-          <t>READ</t>
-        </is>
-      </c>
-      <c r="B97" s="51" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C97" s="51" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="D97" s="51" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E97" s="51" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F97" s="51" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G97" s="51" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H97" s="51" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I97" s="52" t="n">
-        <v>6</v>
-      </c>
-      <c r="J97" s="51" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K97" s="51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L97" s="51" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M97" s="66" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N97" s="51" t="inlineStr">
-        <is>
-          <t>Not changed (PO_MAPPED_FLAG stays Y)</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B98" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C98" s="58" t="inlineStr">
-        <is>
-          <t>CO-14108</t>
-        </is>
-      </c>
-      <c r="D98" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="E98" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F98" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G98" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H98" s="58" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="I98" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="J98" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K98" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L98" s="60" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M98" s="49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N98" s="58" t="inlineStr">
-        <is>
-          <t>PO and ASN through ASN0003</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="35" t="inlineStr">
-        <is>
-          <t>TB_H_CROSSDOCK_ORDER_CHANGE</t>
-        </is>
-      </c>
-      <c r="D100" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="26" customHeight="1">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B101" s="42" t="inlineStr">
-        <is>
-          <t>HIST_ID</t>
-        </is>
-      </c>
-      <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
-        </is>
-      </c>
-      <c r="E101" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F101" s="3" t="inlineStr">
-        <is>
-          <t>FROM_CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="G101" s="3" t="inlineStr">
-        <is>
-          <t>FROM_SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="H101" s="3" t="inlineStr">
-        <is>
-          <t>TO_CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="I101" s="3" t="inlineStr">
-        <is>
-          <t>TO_DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="J101" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="K101" s="3" t="inlineStr">
-        <is>
-          <t>FROM_INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="L101" s="3" t="inlineStr">
-        <is>
-          <t>TO_INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="M101" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="48" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B102" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="C102" s="49" t="inlineStr">
-        <is>
-          <t>ASN0003</t>
-        </is>
-      </c>
-      <c r="D102" s="49" t="inlineStr">
-        <is>
-          <t>C-0003-03</t>
-        </is>
-      </c>
-      <c r="E102" s="49" t="inlineStr">
-        <is>
-          <t>PART-X</t>
-        </is>
-      </c>
-      <c r="F102" s="49" t="inlineStr">
-        <is>
-          <t>CO-14104</t>
-        </is>
-      </c>
-      <c r="G102" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H102" s="49" t="inlineStr">
-        <is>
-          <t>CO-14108</t>
-        </is>
-      </c>
-      <c r="I102" s="49" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="J102" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="K102" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="L102" s="53" t="n">
-        <v>6</v>
-      </c>
-      <c r="M102" s="49" t="inlineStr"/>
+      <c r="M95" s="49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23593,7 +23248,7 @@
       </c>
       <c r="F18" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
+          <t>SIM-2, SIM-6, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -40038,7 +39693,7 @@
       </c>
       <c r="B9" s="32" t="inlineStr">
         <is>
-          <t>UPD_STATUS day by day; cancel after ASN → Change Order Number (simulasi_asn.xlsx)</t>
+          <t>One PO per order date (short PO → split PO); cancel of a middle row after ASN → Change Order Number (simulasi_asn.xlsx)</t>
         </is>
       </c>
       <c r="C9" s="32" t="inlineStr">
@@ -40053,12 +39708,12 @@
       </c>
       <c r="E9" s="32" t="inlineStr">
         <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE, TB_R_INSTRUCTION, #TEMP_INSTRUCTION, TB_R_PRA_DAILY_ORDER_MAPPED, TB_H_CROSSDOCK_ORDER_CHANGE</t>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE, TB_R_INSTRUCTION, #TEMP_INSTRUCTION, TB_H_CROSSDOCK_ORDER_CHANGE</t>
         </is>
       </c>
       <c r="F9" s="32" t="inlineStr">
         <is>
-          <t>PART-X, 6 pcs/case. ORDER_STATUS of the replicate keeps the first value (7); a change in G-System is written to UPD_STATUS: 6 received, 2 cancel. 16-Oct CO-14101 VN → ASN0001, CO-14102 TH on hold. 17-Oct CO-14101 received (6), CO-14102 cancelled (2, no ASN: nothing else), CO-14103 → ASN0002. 18-Oct order date 17-Oct: scan order CO-14105, CO-14106 + CO-14107, CO-14104 (customer code 9715300 before 9722D10); all 3 cases Ready, sent together in ASN0003. CO-14108 (order date 18-Oct) gets no PO (Not Ready). 19-Oct ASN0003 received; CO-14104 cancelled although in case 3, its pcs go to CO-14108 in G-System (6, PO_MAPPED N, no ASN). The D/S team moves case 3 from CO-14104 to CO-14108 in Change Order Number (XD11); history in TB_H_CROSSDOCK_ORDER_CHANGE.</t>
+          <t>PART-X, 6 pcs/case. One PO per customer order date: PO_DT = order date + 1, qty = total order qty of the date (all destinations). PO qty &lt; order qty is an abnormality: the rest comes in a split PO. ORDER_STATUS of the replicate keeps 7; changes go to UPD_STATUS. Order date 15-Oct (12) → PO-DMY-09011; CO-14102 on hold then cancelled, so its 6 pcs of PO-DMY-09011 go to CO-14103 (older PO_DT first). Order date 17-Oct: 4 destinations, 30 pcs, PO-DMY-09013 only 18 (abnormal) → case 5 Not Ready until the split PO-DMY-09014 (12, 19-Oct). Cases 1-4 → ASN0003; CO-14104 (middle row, case 3) is cancelled after the ASN. 21-Oct G-System allocates the pcs of case 3 to CO-14111 (UPD_STATUS 6, no ASN): the D/S team moves case 3 to CO-14111 (XD11). Open PO qty at the end (12) = cancelled qty (CO-14102 + CO-14104).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simulation: add order date 18-Oct with 3 destinations (ASN0005)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -10132,7 +10132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P95"/>
+  <dimension ref="A1:P112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10184,7 +10184,7 @@
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
         <is>
-          <t>• Order date 17-Oct: 4 destinations, 30 pcs, PO-DMY-09013 only 18 (abnormal) → case 5 Not Ready until the split PO-DMY-09014 (12, 19-Oct). Cases 1-4 → ASN0003; CO-14104 (middle row, case 3) is cancelled after the ASN.</t>
+          <t>• Order date 17-Oct: 4 destinations, 30 pcs, PO-DMY-09013 only 18 (abnormal) → case 5 Not Ready until the split PO-DMY-09014 (12, 19-Oct). Cases 1-4 → ASN0003; CO-14104 (middle row, case 3) is cancelled after the ASN. Order date 18-Oct: 3 destinations, 18 pcs, PO-DMY-09015 18 (OK) → ASN0005.</t>
         </is>
       </c>
     </row>
@@ -12857,7 +12857,7 @@
     <row r="68">
       <c r="A68" s="45" t="inlineStr">
         <is>
-          <t>8. 19-Oct XD08: ASN0003 received, CO-14104 → 2 (middle row, in case 3); split PO-DMY-09014 (PO_DT 19-Oct, 12)</t>
+          <t>8. 19-Oct XD08: ASN0003 received, CO-14104 → 2 (middle row, in case 3); split PO-DMY-09014 (PO_DT 19-Oct, 12); order date 18-Oct new</t>
         </is>
       </c>
       <c r="B68" s="46" t="n"/>
@@ -13031,113 +13031,152 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="45" t="inlineStr">
-        <is>
-          <t>9. 19-Oct CO-14110 → ASN0004 with the split PO</t>
-        </is>
-      </c>
-      <c r="B73" s="46" t="n"/>
-      <c r="C73" s="46" t="n"/>
-      <c r="D73" s="46" t="n"/>
-      <c r="E73" s="46" t="n"/>
-      <c r="F73" s="46" t="n"/>
-      <c r="G73" s="46" t="n"/>
-      <c r="H73" s="46" t="n"/>
-      <c r="I73" s="46" t="n"/>
-      <c r="J73" s="46" t="n"/>
-      <c r="K73" s="46" t="n"/>
-      <c r="L73" s="46" t="n"/>
-      <c r="M73" s="46" t="n"/>
-      <c r="N73" s="46" t="n"/>
-      <c r="O73" s="46" t="n"/>
-      <c r="P73" s="46" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D74" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="3" t="inlineStr">
+      <c r="A73" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D73" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="26" customHeight="1">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B75" s="42" t="inlineStr">
-        <is>
-          <t>INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>LINE_SEQ</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F75" s="3" t="inlineStr">
+      <c r="B74" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C74" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D74" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E74" s="42" t="inlineStr">
         <is>
           <t>DESTINATION_CD</t>
         </is>
       </c>
-      <c r="G75" s="3" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="H75" s="3" t="inlineStr">
+      <c r="F74" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G74" s="42" t="inlineStr">
         <is>
           <t>SERIAL_NO</t>
         </is>
       </c>
-      <c r="I75" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="J75" s="3" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="K75" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="L75" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="M75" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="N75" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
-        </is>
-      </c>
-      <c r="O75" s="3" t="inlineStr">
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M74" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N74" s="5" t="inlineStr">
         <is>
           <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B75" s="49" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C75" s="49" t="inlineStr">
+        <is>
+          <t>CO-14112</t>
+        </is>
+      </c>
+      <c r="D75" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E75" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F75" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G75" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H75" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I75" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J75" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K75" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L75" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M75" s="49" t="n"/>
+      <c r="N75" s="49" t="inlineStr">
+        <is>
+          <t>Order date 18-Oct, 3 destinations (PO-DMY-09015, PO_DT 19-Oct, 18)</t>
         </is>
       </c>
     </row>
@@ -13147,33 +13186,39 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="B76" s="53" t="n">
-        <v>8</v>
-      </c>
-      <c r="C76" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D76" s="53" t="n">
-        <v>1</v>
+      <c r="B76" s="49" t="inlineStr">
+        <is>
+          <t>9811100</t>
+        </is>
+      </c>
+      <c r="C76" s="49" t="inlineStr">
+        <is>
+          <t>CO-14113</t>
+        </is>
+      </c>
+      <c r="D76" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
       </c>
       <c r="E76" s="49" t="inlineStr">
         <is>
+          <t>9811110</t>
+        </is>
+      </c>
+      <c r="F76" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G76" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H76" s="49" t="inlineStr">
+        <is>
           <t>PART-X</t>
-        </is>
-      </c>
-      <c r="F76" s="49" t="inlineStr">
-        <is>
-          <t>982220</t>
-        </is>
-      </c>
-      <c r="G76" s="49" t="inlineStr">
-        <is>
-          <t>CO-14110</t>
-        </is>
-      </c>
-      <c r="H76" s="49" t="inlineStr">
-        <is>
-          <t>0000001</t>
         </is>
       </c>
       <c r="I76" s="53" t="n">
@@ -13181,748 +13226,1556 @@
       </c>
       <c r="J76" s="49" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K76" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L76" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M76" s="49" t="n"/>
+      <c r="N76" s="49" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B77" s="49" t="inlineStr">
+        <is>
+          <t>982200</t>
+        </is>
+      </c>
+      <c r="C77" s="49" t="inlineStr">
+        <is>
+          <t>CO-14114</t>
+        </is>
+      </c>
+      <c r="D77" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E77" s="49" t="inlineStr">
+        <is>
+          <t>982220</t>
+        </is>
+      </c>
+      <c r="F77" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G77" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H77" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I77" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J77" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K77" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L77" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M77" s="49" t="n"/>
+      <c r="N77" s="49" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="45" t="inlineStr">
+        <is>
+          <t>9. 19-Oct [Search] → XD09: rest of 17-Oct with the split PO, then 18-Oct</t>
+        </is>
+      </c>
+      <c r="B79" s="46" t="n"/>
+      <c r="C79" s="46" t="n"/>
+      <c r="D79" s="46" t="n"/>
+      <c r="E79" s="46" t="n"/>
+      <c r="F79" s="46" t="n"/>
+      <c r="G79" s="46" t="n"/>
+      <c r="H79" s="46" t="n"/>
+      <c r="I79" s="46" t="n"/>
+      <c r="J79" s="46" t="n"/>
+      <c r="K79" s="46" t="n"/>
+      <c r="L79" s="46" t="n"/>
+      <c r="M79" s="46" t="n"/>
+      <c r="N79" s="46" t="n"/>
+      <c r="O79" s="46" t="n"/>
+      <c r="P79" s="46" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="35" t="inlineStr">
+        <is>
+          <t>#TEMP_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D80" s="47" t="inlineStr">
+        <is>
+          <t>Temporary (session)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="26" customHeight="1">
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B81" s="9" t="inlineStr">
+        <is>
+          <t>SORT_SEQ</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>OPEN_ORDER_QTY</t>
+        </is>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="I81" s="9" t="inlineStr">
+        <is>
+          <t>ASSIGNED_QTY</t>
+        </is>
+      </c>
+      <c r="J81" s="9" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="K81" s="9" t="inlineStr">
+        <is>
+          <t>CUM_DEST_QTY</t>
+        </is>
+      </c>
+      <c r="L81" s="9" t="inlineStr">
+        <is>
+          <t>SEQ_QTY</t>
+        </is>
+      </c>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>CUT_FLAG</t>
+        </is>
+      </c>
+      <c r="N81" s="9" t="inlineStr">
+        <is>
+          <t>GROUP_SEQ</t>
+        </is>
+      </c>
+      <c r="O81" s="9" t="inlineStr">
+        <is>
+          <t>CROSSDOCK_STATUS</t>
+        </is>
+      </c>
+      <c r="P81" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B82" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" s="64" t="inlineStr">
+        <is>
+          <t>982200</t>
+        </is>
+      </c>
+      <c r="D82" s="64" t="inlineStr">
+        <is>
+          <t>CO-14110</t>
+        </is>
+      </c>
+      <c r="E82" s="64" t="inlineStr">
+        <is>
+          <t>982220</t>
+        </is>
+      </c>
+      <c r="F82" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G82" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="H82" s="64" t="inlineStr">
+        <is>
           <t>PO-DMY-09014</t>
         </is>
       </c>
-      <c r="K76" s="49" t="inlineStr">
-        <is>
-          <t>MF-DMY-09014</t>
-        </is>
-      </c>
-      <c r="L76" s="49" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="M76" s="49" t="inlineStr">
-        <is>
-          <t>ASN0004</t>
-        </is>
-      </c>
-      <c r="N76" s="49" t="inlineStr">
-        <is>
-          <t>C-0004-01</t>
-        </is>
-      </c>
-      <c r="O76" s="49" t="inlineStr">
-        <is>
-          <t>6 pcs of the split PO stay open</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="45" t="inlineStr">
-        <is>
-          <t>10. 20-Oct XD08: CO-14111 new (order date 19-Oct, PO-DMY-09015); 21-Oct → 6 (pcs of case 3 allocated by G-System)</t>
-        </is>
-      </c>
-      <c r="B78" s="46" t="n"/>
-      <c r="C78" s="46" t="n"/>
-      <c r="D78" s="46" t="n"/>
-      <c r="E78" s="46" t="n"/>
-      <c r="F78" s="46" t="n"/>
-      <c r="G78" s="46" t="n"/>
-      <c r="H78" s="46" t="n"/>
-      <c r="I78" s="46" t="n"/>
-      <c r="J78" s="46" t="n"/>
-      <c r="K78" s="46" t="n"/>
-      <c r="L78" s="46" t="n"/>
-      <c r="M78" s="46" t="n"/>
-      <c r="N78" s="46" t="n"/>
-      <c r="O78" s="46" t="n"/>
-      <c r="P78" s="46" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
-        </is>
-      </c>
-      <c r="D79" s="47" t="inlineStr">
-        <is>
-          <t>Replicated from DB Surrounding (G-System)</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="26" customHeight="1">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B80" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_CD</t>
-        </is>
-      </c>
-      <c r="C80" s="42" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="D80" s="42" t="inlineStr">
-        <is>
-          <t>ORDER_DT</t>
-        </is>
-      </c>
-      <c r="E80" s="42" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="F80" s="42" t="inlineStr">
-        <is>
-          <t>DETAILED_ITEM_NO</t>
-        </is>
-      </c>
-      <c r="G80" s="42" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="H80" s="5" t="inlineStr">
-        <is>
-          <t>SHIPPING_PART_NO</t>
-        </is>
-      </c>
-      <c r="I80" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS_QTY</t>
-        </is>
-      </c>
-      <c r="J80" s="5" t="inlineStr">
-        <is>
-          <t>ORDER_STATUS</t>
-        </is>
-      </c>
-      <c r="K80" s="5" t="inlineStr">
-        <is>
-          <t>HOLD_FLAG</t>
-        </is>
-      </c>
-      <c r="L80" s="5" t="inlineStr">
-        <is>
-          <t>PO_MAPPED_FLAG</t>
-        </is>
-      </c>
-      <c r="M80" s="5" t="inlineStr">
-        <is>
-          <t>UPD_STATUS</t>
-        </is>
-      </c>
-      <c r="N80" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B81" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="C81" s="58" t="inlineStr">
-        <is>
-          <t>CO-14111</t>
-        </is>
-      </c>
-      <c r="D81" s="58" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E81" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="F81" s="58" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="G81" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="H81" s="58" t="inlineStr">
+      <c r="I82" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J82" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K82" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L82" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M82" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N82" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="O82" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P82" s="64" t="inlineStr">
+        <is>
+          <t>→ ASN0004</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B83" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" s="64" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="D83" s="64" t="inlineStr">
+        <is>
+          <t>CO-14112</t>
+        </is>
+      </c>
+      <c r="E83" s="64" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F83" s="64" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="I81" s="59" t="n">
+      <c r="G83" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="J81" s="58" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="K81" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L81" s="58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M81" s="60" t="inlineStr">
+      <c r="H83" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="I83" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J83" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K83" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L83" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M83" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N83" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="O83" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="N81" s="58" t="inlineStr">
-        <is>
-          <t>Received without ASN: candidate</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="45" t="inlineStr">
-        <is>
-          <t>11. 21-Oct XD11 Change Order Number: ASN0003 case 3 → CO-14111</t>
-        </is>
-      </c>
-      <c r="B83" s="46" t="n"/>
-      <c r="C83" s="46" t="n"/>
-      <c r="D83" s="46" t="n"/>
-      <c r="E83" s="46" t="n"/>
-      <c r="F83" s="46" t="n"/>
-      <c r="G83" s="46" t="n"/>
-      <c r="H83" s="46" t="n"/>
-      <c r="I83" s="46" t="n"/>
-      <c r="J83" s="46" t="n"/>
-      <c r="K83" s="46" t="n"/>
-      <c r="L83" s="46" t="n"/>
-      <c r="M83" s="46" t="n"/>
-      <c r="N83" s="46" t="n"/>
-      <c r="O83" s="46" t="n"/>
-      <c r="P83" s="46" t="n"/>
+      <c r="P83" s="64" t="inlineStr">
+        <is>
+          <t>Rest of the split PO; cases 1-3 → ASN0005</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="35" t="inlineStr">
-        <is>
-          <t>TB_R_INSTRUCTION</t>
-        </is>
-      </c>
-      <c r="D84" s="47" t="inlineStr">
-        <is>
-          <t>New table (Crossdock)</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="26" customHeight="1">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B85" s="42" t="inlineStr">
-        <is>
-          <t>INSTRUCTION_ID</t>
-        </is>
-      </c>
-      <c r="C85" s="3" t="inlineStr">
-        <is>
-          <t>CASE_SEQ</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>LINE_SEQ</t>
-        </is>
-      </c>
-      <c r="E85" s="3" t="inlineStr">
-        <is>
-          <t>PART_NO</t>
-        </is>
-      </c>
-      <c r="F85" s="3" t="inlineStr">
-        <is>
-          <t>DESTINATION_CD</t>
-        </is>
-      </c>
-      <c r="G85" s="3" t="inlineStr">
-        <is>
-          <t>CUSTOMER_ORDER_NO</t>
-        </is>
-      </c>
-      <c r="H85" s="3" t="inlineStr">
-        <is>
-          <t>SERIAL_NO</t>
-        </is>
-      </c>
-      <c r="I85" s="3" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="J85" s="3" t="inlineStr">
-        <is>
-          <t>PO_NO</t>
-        </is>
-      </c>
-      <c r="K85" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_NO</t>
-        </is>
-      </c>
-      <c r="L85" s="3" t="inlineStr">
-        <is>
-          <t>MANIFEST_ITEM</t>
-        </is>
-      </c>
-      <c r="M85" s="3" t="inlineStr">
-        <is>
-          <t>ASN_NO</t>
-        </is>
-      </c>
-      <c r="N85" s="3" t="inlineStr">
-        <is>
-          <t>CASE_NO</t>
-        </is>
-      </c>
-      <c r="O85" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="57" t="inlineStr">
-        <is>
-          <t>UPD</t>
-        </is>
-      </c>
-      <c r="B86" s="59" t="n">
+      <c r="A84" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B84" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" s="64" t="inlineStr">
+        <is>
+          <t>9811100</t>
+        </is>
+      </c>
+      <c r="D84" s="64" t="inlineStr">
+        <is>
+          <t>CO-14113</t>
+        </is>
+      </c>
+      <c r="E84" s="64" t="inlineStr">
+        <is>
+          <t>9811110</t>
+        </is>
+      </c>
+      <c r="F84" s="64" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="G84" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="C86" s="59" t="n">
+      <c r="H84" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09015</t>
+        </is>
+      </c>
+      <c r="I84" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J84" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K84" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L84" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M84" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N84" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O84" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P84" s="64" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="62" t="inlineStr">
+        <is>
+          <t>TEMP</t>
+        </is>
+      </c>
+      <c r="B85" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="D86" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E86" s="58" t="inlineStr">
+      <c r="C85" s="64" t="inlineStr">
+        <is>
+          <t>982200</t>
+        </is>
+      </c>
+      <c r="D85" s="64" t="inlineStr">
+        <is>
+          <t>CO-14114</t>
+        </is>
+      </c>
+      <c r="E85" s="64" t="inlineStr">
+        <is>
+          <t>982220</t>
+        </is>
+      </c>
+      <c r="F85" s="64" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="F86" s="58" t="inlineStr">
-        <is>
-          <t>9722D10</t>
-        </is>
-      </c>
-      <c r="G86" s="60" t="inlineStr">
-        <is>
-          <t>CO-14111</t>
-        </is>
-      </c>
-      <c r="H86" s="58" t="inlineStr">
-        <is>
-          <t>0000001</t>
-        </is>
-      </c>
-      <c r="I86" s="59" t="n">
+      <c r="G85" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="J86" s="58" t="inlineStr">
-        <is>
-          <t>PO-DMY-09013</t>
-        </is>
-      </c>
-      <c r="K86" s="58" t="inlineStr">
-        <is>
-          <t>MF-DMY-09013</t>
-        </is>
-      </c>
-      <c r="L86" s="58" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="M86" s="58" t="inlineStr">
-        <is>
-          <t>ASN0003</t>
-        </is>
-      </c>
-      <c r="N86" s="58" t="inlineStr">
-        <is>
-          <t>C-0003-03</t>
-        </is>
-      </c>
-      <c r="O86" s="58" t="inlineStr">
-        <is>
-          <t>Whole row moved; case, PO and ASN not changed</t>
-        </is>
-      </c>
+      <c r="H85" s="64" t="inlineStr">
+        <is>
+          <t>PO-DMY-09015</t>
+        </is>
+      </c>
+      <c r="I85" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="J85" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="K85" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="L85" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="M85" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N85" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="O85" s="49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P85" s="64" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="45" t="inlineStr">
+        <is>
+          <t>10. 19-Oct ASN0004 (CO-14110) and ASN0005 (order date 18-Oct, cases 1-3)</t>
+        </is>
+      </c>
+      <c r="B87" s="46" t="n"/>
+      <c r="C87" s="46" t="n"/>
+      <c r="D87" s="46" t="n"/>
+      <c r="E87" s="46" t="n"/>
+      <c r="F87" s="46" t="n"/>
+      <c r="G87" s="46" t="n"/>
+      <c r="H87" s="46" t="n"/>
+      <c r="I87" s="46" t="n"/>
+      <c r="J87" s="46" t="n"/>
+      <c r="K87" s="46" t="n"/>
+      <c r="L87" s="46" t="n"/>
+      <c r="M87" s="46" t="n"/>
+      <c r="N87" s="46" t="n"/>
+      <c r="O87" s="46" t="n"/>
+      <c r="P87" s="46" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="35" t="inlineStr">
         <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D88" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="26" customHeight="1">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B89" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N89" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O89" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B90" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="C90" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F90" s="49" t="inlineStr">
+        <is>
+          <t>982220</t>
+        </is>
+      </c>
+      <c r="G90" s="49" t="inlineStr">
+        <is>
+          <t>CO-14110</t>
+        </is>
+      </c>
+      <c r="H90" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I90" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J90" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="K90" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09014</t>
+        </is>
+      </c>
+      <c r="L90" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M90" s="49" t="inlineStr">
+        <is>
+          <t>ASN0004</t>
+        </is>
+      </c>
+      <c r="N90" s="49" t="inlineStr">
+        <is>
+          <t>C-0004-01</t>
+        </is>
+      </c>
+      <c r="O90" s="49" t="inlineStr">
+        <is>
+          <t>Split PO</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B91" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="C91" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F91" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G91" s="49" t="inlineStr">
+        <is>
+          <t>CO-14112</t>
+        </is>
+      </c>
+      <c r="H91" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I91" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J91" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09014</t>
+        </is>
+      </c>
+      <c r="K91" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09014</t>
+        </is>
+      </c>
+      <c r="L91" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M91" s="49" t="inlineStr">
+        <is>
+          <t>ASN0005</t>
+        </is>
+      </c>
+      <c r="N91" s="49" t="inlineStr">
+        <is>
+          <t>C-0005-01</t>
+        </is>
+      </c>
+      <c r="O91" s="49" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B92" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="C92" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D92" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F92" s="49" t="inlineStr">
+        <is>
+          <t>9811110</t>
+        </is>
+      </c>
+      <c r="G92" s="49" t="inlineStr">
+        <is>
+          <t>CO-14113</t>
+        </is>
+      </c>
+      <c r="H92" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I92" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J92" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09015</t>
+        </is>
+      </c>
+      <c r="K92" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09015</t>
+        </is>
+      </c>
+      <c r="L92" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M92" s="49" t="inlineStr">
+        <is>
+          <t>ASN0005</t>
+        </is>
+      </c>
+      <c r="N92" s="49" t="inlineStr">
+        <is>
+          <t>C-0005-02</t>
+        </is>
+      </c>
+      <c r="O92" s="49" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B93" s="53" t="n">
+        <v>11</v>
+      </c>
+      <c r="C93" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D93" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F93" s="49" t="inlineStr">
+        <is>
+          <t>982220</t>
+        </is>
+      </c>
+      <c r="G93" s="49" t="inlineStr">
+        <is>
+          <t>CO-14114</t>
+        </is>
+      </c>
+      <c r="H93" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I93" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J93" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09015</t>
+        </is>
+      </c>
+      <c r="K93" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09015</t>
+        </is>
+      </c>
+      <c r="L93" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M93" s="49" t="inlineStr">
+        <is>
+          <t>ASN0005</t>
+        </is>
+      </c>
+      <c r="N93" s="49" t="inlineStr">
+        <is>
+          <t>C-0005-03</t>
+        </is>
+      </c>
+      <c r="O93" s="49" t="inlineStr">
+        <is>
+          <t>6 pcs of PO-DMY-09015 stay open</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="45" t="inlineStr">
+        <is>
+          <t>11. 20-Oct XD08: CO-14111 new (order date 19-Oct, PO-DMY-09016); 21-Oct → 6 (pcs of case 3 allocated by G-System)</t>
+        </is>
+      </c>
+      <c r="B95" s="46" t="n"/>
+      <c r="C95" s="46" t="n"/>
+      <c r="D95" s="46" t="n"/>
+      <c r="E95" s="46" t="n"/>
+      <c r="F95" s="46" t="n"/>
+      <c r="G95" s="46" t="n"/>
+      <c r="H95" s="46" t="n"/>
+      <c r="I95" s="46" t="n"/>
+      <c r="J95" s="46" t="n"/>
+      <c r="K95" s="46" t="n"/>
+      <c r="L95" s="46" t="n"/>
+      <c r="M95" s="46" t="n"/>
+      <c r="N95" s="46" t="n"/>
+      <c r="O95" s="46" t="n"/>
+      <c r="P95" s="46" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="35" t="inlineStr">
+        <is>
           <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
         </is>
       </c>
-      <c r="D88" s="47" t="inlineStr">
+      <c r="D96" s="47" t="inlineStr">
         <is>
           <t>Replicated from DB Surrounding (G-System)</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="26" customHeight="1">
-      <c r="A89" s="5" t="inlineStr">
+    <row r="97" ht="26" customHeight="1">
+      <c r="A97" s="5" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B89" s="42" t="inlineStr">
+      <c r="B97" s="42" t="inlineStr">
         <is>
           <t>CUSTOMER_CD</t>
         </is>
       </c>
-      <c r="C89" s="42" t="inlineStr">
+      <c r="C97" s="42" t="inlineStr">
         <is>
           <t>CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="D89" s="42" t="inlineStr">
+      <c r="D97" s="42" t="inlineStr">
         <is>
           <t>ORDER_DT</t>
         </is>
       </c>
-      <c r="E89" s="42" t="inlineStr">
+      <c r="E97" s="42" t="inlineStr">
         <is>
           <t>DESTINATION_CD</t>
         </is>
       </c>
-      <c r="F89" s="42" t="inlineStr">
+      <c r="F97" s="42" t="inlineStr">
         <is>
           <t>DETAILED_ITEM_NO</t>
         </is>
       </c>
-      <c r="G89" s="42" t="inlineStr">
+      <c r="G97" s="42" t="inlineStr">
         <is>
           <t>SERIAL_NO</t>
         </is>
       </c>
-      <c r="H89" s="5" t="inlineStr">
+      <c r="H97" s="5" t="inlineStr">
         <is>
           <t>SHIPPING_PART_NO</t>
         </is>
       </c>
-      <c r="I89" s="5" t="inlineStr">
+      <c r="I97" s="5" t="inlineStr">
         <is>
           <t>ORDER_STATUS_QTY</t>
         </is>
       </c>
-      <c r="J89" s="5" t="inlineStr">
+      <c r="J97" s="5" t="inlineStr">
         <is>
           <t>ORDER_STATUS</t>
         </is>
       </c>
-      <c r="K89" s="5" t="inlineStr">
+      <c r="K97" s="5" t="inlineStr">
         <is>
           <t>HOLD_FLAG</t>
         </is>
       </c>
-      <c r="L89" s="5" t="inlineStr">
+      <c r="L97" s="5" t="inlineStr">
         <is>
           <t>PO_MAPPED_FLAG</t>
         </is>
       </c>
-      <c r="M89" s="5" t="inlineStr">
+      <c r="M97" s="5" t="inlineStr">
         <is>
           <t>UPD_STATUS</t>
         </is>
       </c>
-      <c r="N89" s="5" t="inlineStr">
+      <c r="N97" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="50" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B98" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="C98" s="58" t="inlineStr">
+        <is>
+          <t>CO-14111</t>
+        </is>
+      </c>
+      <c r="D98" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E98" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="F98" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G98" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H98" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I98" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J98" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K98" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L98" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M98" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N98" s="58" t="inlineStr">
+        <is>
+          <t>Received without ASN: candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="45" t="inlineStr">
+        <is>
+          <t>12. 21-Oct XD11 Change Order Number: ASN0003 case 3 → CO-14111</t>
+        </is>
+      </c>
+      <c r="B100" s="46" t="n"/>
+      <c r="C100" s="46" t="n"/>
+      <c r="D100" s="46" t="n"/>
+      <c r="E100" s="46" t="n"/>
+      <c r="F100" s="46" t="n"/>
+      <c r="G100" s="46" t="n"/>
+      <c r="H100" s="46" t="n"/>
+      <c r="I100" s="46" t="n"/>
+      <c r="J100" s="46" t="n"/>
+      <c r="K100" s="46" t="n"/>
+      <c r="L100" s="46" t="n"/>
+      <c r="M100" s="46" t="n"/>
+      <c r="N100" s="46" t="n"/>
+      <c r="O100" s="46" t="n"/>
+      <c r="P100" s="46" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D101" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="26" customHeight="1">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B102" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L102" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N102" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O102" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B103" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="C103" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D103" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F103" s="58" t="inlineStr">
+        <is>
+          <t>9722D10</t>
+        </is>
+      </c>
+      <c r="G103" s="60" t="inlineStr">
+        <is>
+          <t>CO-14111</t>
+        </is>
+      </c>
+      <c r="H103" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I103" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J103" s="58" t="inlineStr">
+        <is>
+          <t>PO-DMY-09013</t>
+        </is>
+      </c>
+      <c r="K103" s="58" t="inlineStr">
+        <is>
+          <t>MF-DMY-09013</t>
+        </is>
+      </c>
+      <c r="L103" s="58" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M103" s="58" t="inlineStr">
+        <is>
+          <t>ASN0003</t>
+        </is>
+      </c>
+      <c r="N103" s="58" t="inlineStr">
+        <is>
+          <t>C-0003-03</t>
+        </is>
+      </c>
+      <c r="O103" s="58" t="inlineStr">
+        <is>
+          <t>Whole row moved; case, PO and ASN not changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D105" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="26" customHeight="1">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B106" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C106" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D106" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E106" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F106" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G106" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J106" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L106" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M106" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N106" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="50" t="inlineStr">
         <is>
           <t>READ</t>
         </is>
       </c>
-      <c r="B90" s="51" t="inlineStr">
+      <c r="B107" s="51" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="C90" s="51" t="inlineStr">
+      <c r="C107" s="51" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
       </c>
-      <c r="D90" s="51" t="inlineStr">
+      <c r="D107" s="51" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="E90" s="51" t="inlineStr">
+      <c r="E107" s="51" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="F90" s="51" t="inlineStr">
+      <c r="F107" s="51" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="G90" s="51" t="inlineStr">
+      <c r="G107" s="51" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H90" s="51" t="inlineStr">
+      <c r="H107" s="51" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="I90" s="52" t="n">
+      <c r="I107" s="52" t="n">
         <v>6</v>
       </c>
-      <c r="J90" s="51" t="inlineStr">
+      <c r="J107" s="51" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="K90" s="51" t="inlineStr">
+      <c r="K107" s="51" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L90" s="51" t="inlineStr">
+      <c r="L107" s="51" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M90" s="66" t="inlineStr">
+      <c r="M107" s="66" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="N90" s="51" t="inlineStr">
+      <c r="N107" s="51" t="inlineStr">
         <is>
           <t>Not changed (PO_MAPPED_FLAG stays Y)</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="57" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="57" t="inlineStr">
         <is>
           <t>UPD</t>
         </is>
       </c>
-      <c r="B91" s="58" t="inlineStr">
+      <c r="B108" s="58" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="C91" s="58" t="inlineStr">
+      <c r="C108" s="58" t="inlineStr">
         <is>
           <t>CO-14111</t>
         </is>
       </c>
-      <c r="D91" s="58" t="inlineStr">
+      <c r="D108" s="58" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E91" s="58" t="inlineStr">
+      <c r="E108" s="58" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="F91" s="58" t="inlineStr">
+      <c r="F108" s="58" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="G91" s="58" t="inlineStr">
+      <c r="G108" s="58" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H91" s="58" t="inlineStr">
+      <c r="H108" s="58" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="I91" s="59" t="n">
+      <c r="I108" s="59" t="n">
         <v>6</v>
       </c>
-      <c r="J91" s="58" t="inlineStr">
+      <c r="J108" s="58" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="K91" s="58" t="inlineStr">
+      <c r="K108" s="58" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L91" s="60" t="inlineStr">
+      <c r="L108" s="60" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M91" s="49" t="inlineStr">
+      <c r="M108" s="49" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="N91" s="58" t="inlineStr">
+      <c r="N108" s="58" t="inlineStr">
         <is>
           <t>PO and ASN through ASN0003</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="35" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="35" t="inlineStr">
         <is>
           <t>TB_H_CROSSDOCK_ORDER_CHANGE</t>
         </is>
       </c>
-      <c r="D93" s="47" t="inlineStr">
+      <c r="D110" s="47" t="inlineStr">
         <is>
           <t>New table (Crossdock)</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="26" customHeight="1">
-      <c r="A94" s="3" t="inlineStr">
+    <row r="111" ht="26" customHeight="1">
+      <c r="A111" s="3" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B94" s="42" t="inlineStr">
+      <c r="B111" s="42" t="inlineStr">
         <is>
           <t>HIST_ID</t>
         </is>
       </c>
-      <c r="C94" s="3" t="inlineStr">
+      <c r="C111" s="3" t="inlineStr">
         <is>
           <t>ASN_NO</t>
         </is>
       </c>
-      <c r="D94" s="3" t="inlineStr">
+      <c r="D111" s="3" t="inlineStr">
         <is>
           <t>CASE_NO</t>
         </is>
       </c>
-      <c r="E94" s="3" t="inlineStr">
+      <c r="E111" s="3" t="inlineStr">
         <is>
           <t>PART_NO</t>
         </is>
       </c>
-      <c r="F94" s="3" t="inlineStr">
+      <c r="F111" s="3" t="inlineStr">
         <is>
           <t>FROM_CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="G94" s="3" t="inlineStr">
+      <c r="G111" s="3" t="inlineStr">
         <is>
           <t>FROM_SERIAL_NO</t>
         </is>
       </c>
-      <c r="H94" s="3" t="inlineStr">
+      <c r="H111" s="3" t="inlineStr">
         <is>
           <t>TO_CUSTOMER_ORDER_NO</t>
         </is>
       </c>
-      <c r="I94" s="3" t="inlineStr">
+      <c r="I111" s="3" t="inlineStr">
         <is>
           <t>TO_DESTINATION_CD</t>
         </is>
       </c>
-      <c r="J94" s="3" t="inlineStr">
+      <c r="J111" s="3" t="inlineStr">
         <is>
           <t>QTY</t>
         </is>
       </c>
-      <c r="K94" s="3" t="inlineStr">
+      <c r="K111" s="3" t="inlineStr">
         <is>
           <t>FROM_INSTRUCTION_ID</t>
         </is>
       </c>
-      <c r="L94" s="3" t="inlineStr">
+      <c r="L111" s="3" t="inlineStr">
         <is>
           <t>TO_INSTRUCTION_ID</t>
         </is>
       </c>
-      <c r="M94" s="3" t="inlineStr">
+      <c r="M111" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="48" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="48" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="B95" s="53" t="n">
+      <c r="B112" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="C95" s="49" t="inlineStr">
+      <c r="C112" s="49" t="inlineStr">
         <is>
           <t>ASN0003</t>
         </is>
       </c>
-      <c r="D95" s="49" t="inlineStr">
+      <c r="D112" s="49" t="inlineStr">
         <is>
           <t>C-0003-03</t>
         </is>
       </c>
-      <c r="E95" s="49" t="inlineStr">
+      <c r="E112" s="49" t="inlineStr">
         <is>
           <t>PART-X</t>
         </is>
       </c>
-      <c r="F95" s="49" t="inlineStr">
+      <c r="F112" s="49" t="inlineStr">
         <is>
           <t>CO-14104</t>
         </is>
       </c>
-      <c r="G95" s="49" t="inlineStr">
+      <c r="G112" s="49" t="inlineStr">
         <is>
           <t>0000001</t>
         </is>
       </c>
-      <c r="H95" s="49" t="inlineStr">
+      <c r="H112" s="49" t="inlineStr">
         <is>
           <t>CO-14111</t>
         </is>
       </c>
-      <c r="I95" s="49" t="inlineStr">
+      <c r="I112" s="49" t="inlineStr">
         <is>
           <t>9722D10</t>
         </is>
       </c>
-      <c r="J95" s="53" t="n">
+      <c r="J112" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="K95" s="53" t="n">
+      <c r="K112" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="L95" s="53" t="n">
+      <c r="L112" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="M95" s="49" t="inlineStr"/>
+      <c r="M112" s="49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -39713,7 +40566,7 @@
       </c>
       <c r="F9" s="32" t="inlineStr">
         <is>
-          <t>PART-X, 6 pcs/case. One PO per customer order date: PO_DT = order date + 1, qty = total order qty of the date (all destinations). PO qty &lt; order qty is an abnormality: the rest comes in a split PO. ORDER_STATUS of the replicate keeps 7; changes go to UPD_STATUS. Order date 15-Oct (12) → PO-DMY-09011; CO-14102 on hold then cancelled, so its 6 pcs of PO-DMY-09011 go to CO-14103 (older PO_DT first). Order date 17-Oct: 4 destinations, 30 pcs, PO-DMY-09013 only 18 (abnormal) → case 5 Not Ready until the split PO-DMY-09014 (12, 19-Oct). Cases 1-4 → ASN0003; CO-14104 (middle row, case 3) is cancelled after the ASN. 21-Oct G-System allocates the pcs of case 3 to CO-14111 (UPD_STATUS 6, no ASN): the D/S team moves case 3 to CO-14111 (XD11). Open PO qty at the end (12) = cancelled qty (CO-14102 + CO-14104).</t>
+          <t>PART-X, 6 pcs/case. One PO per customer order date: PO_DT = order date + 1, qty = total order qty of the date (all destinations). PO qty &lt; order qty is an abnormality: the rest comes in a split PO. ORDER_STATUS of the replicate keeps 7; changes go to UPD_STATUS. Order date 15-Oct (12) → PO-DMY-09011; CO-14102 on hold then cancelled, so its 6 pcs of PO-DMY-09011 go to CO-14103 (older PO_DT first). Order date 17-Oct: 4 destinations, 30 pcs, PO-DMY-09013 only 18 (abnormal) → case 5 Not Ready until the split PO-DMY-09014 (12, 19-Oct). Cases 1-4 → ASN0003; CO-14104 (middle row, case 3) is cancelled after the ASN. Order date 18-Oct: 3 destinations, 18 pcs, PO-DMY-09015 18 (OK) → ASN0005. 21-Oct G-System allocates the pcs of case 3 to CO-14111 (UPD_STATUS 6, no ASN): the D/S team moves case 3 to CO-14111 (XD11). Open PO qty at the end (12) = cancelled qty (CO-14102 + CO-14104).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Serial split: one line in 2 ASNs, partial receipt, XD08 re-assigns TB_R_INSTRUCTION
simulasi_asn_rev.xlsx adds CO-14115 (12 pcs in ASN0006 + ASN0007); on 21-Oct
G-System splits it into serial 0000001 6 pcs status 6 and 0000002 6 pcs
status 7. Shows the double mapping without re-assignment and the result with
it. XD08 gets the serial split step (LOG7); ERD SIM-10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
+++ b/deliverables/function_list_v2/erd/Crossdock_ERD.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-7" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-8" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-9" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIM-10" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Column Definition'!$A$3:$H$470</definedName>
@@ -23599,6 +23600,1334 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SIM-10 One line in 2 ASNs; partial receipt splits the serial → XD08 re-assigns TB_R_INSTRUCTION (simulasi_asn.xlsx)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="33" t="inlineStr">
+        <is>
+          <t>BPF F2 · Functions: XD09, XD10, XD08 (serial split)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="34" t="inlineStr">
+        <is>
+          <t>• CO-14115 VN 12 pcs (order date 19-Oct), 6 pcs/case: case 1 → ASN0006 (rit 1), case 2 → ASN0007 (rit 2). One H0253 row, two TB_R_INSTRUCTION rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>• 21-Oct ASN0006 received: G-System splits the line into serial 0000001 6 pcs status 6 and serial 0000002 6 pcs status 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>• Upsert alone: serial 0000001 has 12 pcs in TB_R_INSTRUCTION for qty 6 and serial 0000002 looks open (6) → XD09 would map it again (double). XD08 re-assigns the rows: serial 0000001 = ASN0006 (oldest ASN = received), serial 0000002 = ASN0007; both PO_MAPPED_FLAG Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>NEW row</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>UPD row</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>DEL row</t>
+        </is>
+      </c>
+      <c r="E7" s="39" t="inlineStr">
+        <is>
+          <t>READ row</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="inlineStr">
+        <is>
+          <t>TEMP row</t>
+        </is>
+      </c>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>Changed cell</t>
+        </is>
+      </c>
+      <c r="H7" s="42" t="inlineStr">
+        <is>
+          <t>PK column</t>
+        </is>
+      </c>
+      <c r="I7" s="36" t="inlineStr">
+        <is>
+          <t>Status OK</t>
+        </is>
+      </c>
+      <c r="J7" s="43" t="inlineStr">
+        <is>
+          <t>Status attention</t>
+        </is>
+      </c>
+      <c r="K7" s="44" t="inlineStr">
+        <is>
+          <t>Status NG / cancel</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="45" t="inlineStr">
+        <is>
+          <t>1. 20-Oct ASN0006 (case 1) and ASN0007 (case 2): one line in 2 ASNs</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="n"/>
+      <c r="C9" s="46" t="n"/>
+      <c r="D9" s="46" t="n"/>
+      <c r="E9" s="46" t="n"/>
+      <c r="F9" s="46" t="n"/>
+      <c r="G9" s="46" t="n"/>
+      <c r="H9" s="46" t="n"/>
+      <c r="I9" s="46" t="n"/>
+      <c r="J9" s="46" t="n"/>
+      <c r="K9" s="46" t="n"/>
+      <c r="L9" s="46" t="n"/>
+      <c r="M9" s="46" t="n"/>
+      <c r="N9" s="46" t="n"/>
+      <c r="O9" s="46" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D10" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B12" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F12" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G12" s="49" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="H12" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I12" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09015</t>
+        </is>
+      </c>
+      <c r="K12" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09015</t>
+        </is>
+      </c>
+      <c r="L12" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M12" s="49" t="inlineStr">
+        <is>
+          <t>ASN0006</t>
+        </is>
+      </c>
+      <c r="N12" s="49" t="inlineStr">
+        <is>
+          <t>C-0006-01</t>
+        </is>
+      </c>
+      <c r="O12" s="49" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B13" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="C13" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F13" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G13" s="49" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="H13" s="49" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I13" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="49" t="inlineStr">
+        <is>
+          <t>PO-DMY-09016</t>
+        </is>
+      </c>
+      <c r="K13" s="49" t="inlineStr">
+        <is>
+          <t>MF-DMY-09016</t>
+        </is>
+      </c>
+      <c r="L13" s="49" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M13" s="49" t="inlineStr">
+        <is>
+          <t>ASN0007</t>
+        </is>
+      </c>
+      <c r="N13" s="49" t="inlineStr">
+        <is>
+          <t>C-0007-01</t>
+        </is>
+      </c>
+      <c r="O13" s="49" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C16" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E16" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F16" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G16" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B17" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C17" s="58" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="D17" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E17" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F17" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G17" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H17" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I17" s="59" t="n">
+        <v>12</v>
+      </c>
+      <c r="J17" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K17" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L17" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M17" s="58" t="n"/>
+      <c r="N17" s="58" t="inlineStr">
+        <is>
+          <t>N after ASN0006 (6 of 12), Y after ASN0007</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="45" t="inlineStr">
+        <is>
+          <t>2. 21-Oct XD08 upsert: ASN0006 received, G-System split the line</t>
+        </is>
+      </c>
+      <c r="B19" s="46" t="n"/>
+      <c r="C19" s="46" t="n"/>
+      <c r="D19" s="46" t="n"/>
+      <c r="E19" s="46" t="n"/>
+      <c r="F19" s="46" t="n"/>
+      <c r="G19" s="46" t="n"/>
+      <c r="H19" s="46" t="n"/>
+      <c r="I19" s="46" t="n"/>
+      <c r="J19" s="46" t="n"/>
+      <c r="K19" s="46" t="n"/>
+      <c r="L19" s="46" t="n"/>
+      <c r="M19" s="46" t="n"/>
+      <c r="N19" s="46" t="n"/>
+      <c r="O19" s="46" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D20" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E21" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F21" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G21" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B22" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C22" s="58" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="D22" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E22" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F22" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G22" s="58" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="H22" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I22" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K22" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L22" s="58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M22" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N22" s="58" t="inlineStr">
+        <is>
+          <t>12 → 6, received</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="48" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C23" s="49" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="D23" s="49" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E23" s="49" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F23" s="49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G23" s="49" t="inlineStr">
+        <is>
+          <t>0000002</t>
+        </is>
+      </c>
+      <c r="H23" s="49" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I23" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="J23" s="49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K23" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L23" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M23" s="49" t="n"/>
+      <c r="N23" s="49" t="inlineStr">
+        <is>
+          <t>New serial, status 7: without step 3 open qty 6 = double mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="45" t="inlineStr">
+        <is>
+          <t>3. 21-Oct XD08 serial split: rows re-assigned (LOG7)</t>
+        </is>
+      </c>
+      <c r="B25" s="46" t="n"/>
+      <c r="C25" s="46" t="n"/>
+      <c r="D25" s="46" t="n"/>
+      <c r="E25" s="46" t="n"/>
+      <c r="F25" s="46" t="n"/>
+      <c r="G25" s="46" t="n"/>
+      <c r="H25" s="46" t="n"/>
+      <c r="I25" s="46" t="n"/>
+      <c r="J25" s="46" t="n"/>
+      <c r="K25" s="46" t="n"/>
+      <c r="L25" s="46" t="n"/>
+      <c r="M25" s="46" t="n"/>
+      <c r="N25" s="46" t="n"/>
+      <c r="O25" s="46" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D26" s="47" t="inlineStr">
+        <is>
+          <t>New table (Crossdock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t>INSTRUCTION_ID</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>CASE_SEQ</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>LINE_SEQ</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>PART_NO</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>PO_NO</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_NO</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>MANIFEST_ITEM</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>ASN_NO</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>CASE_NO</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B28" s="52" t="n">
+        <v>12</v>
+      </c>
+      <c r="C28" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="51" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F28" s="51" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G28" s="51" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="H28" s="51" t="inlineStr">
+        <is>
+          <t>0000001</t>
+        </is>
+      </c>
+      <c r="I28" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="J28" s="51" t="inlineStr">
+        <is>
+          <t>PO-DMY-09015</t>
+        </is>
+      </c>
+      <c r="K28" s="51" t="inlineStr">
+        <is>
+          <t>MF-DMY-09015</t>
+        </is>
+      </c>
+      <c r="L28" s="51" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M28" s="51" t="inlineStr">
+        <is>
+          <t>ASN0006</t>
+        </is>
+      </c>
+      <c r="N28" s="51" t="inlineStr">
+        <is>
+          <t>C-0006-01</t>
+        </is>
+      </c>
+      <c r="O28" s="51" t="inlineStr">
+        <is>
+          <t>Oldest ASN → serial with status 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B29" s="59" t="n">
+        <v>13</v>
+      </c>
+      <c r="C29" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="F29" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="G29" s="58" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="H29" s="60" t="inlineStr">
+        <is>
+          <t>0000002</t>
+        </is>
+      </c>
+      <c r="I29" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J29" s="58" t="inlineStr">
+        <is>
+          <t>PO-DMY-09016</t>
+        </is>
+      </c>
+      <c r="K29" s="58" t="inlineStr">
+        <is>
+          <t>MF-DMY-09016</t>
+        </is>
+      </c>
+      <c r="L29" s="58" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="M29" s="58" t="inlineStr">
+        <is>
+          <t>ASN0007</t>
+        </is>
+      </c>
+      <c r="N29" s="58" t="inlineStr">
+        <is>
+          <t>C-0007-01</t>
+        </is>
+      </c>
+      <c r="O29" s="58" t="inlineStr">
+        <is>
+          <t>Next ASN → serial with status 7; case, PO, ASN not changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D31" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B32" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C32" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D32" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E32" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F32" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G32" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B33" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C33" s="58" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="D33" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E33" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F33" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G33" s="58" t="inlineStr">
+        <is>
+          <t>0000002</t>
+        </is>
+      </c>
+      <c r="H33" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I33" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J33" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K33" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L33" s="60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M33" s="58" t="n"/>
+      <c r="N33" s="58" t="inlineStr">
+        <is>
+          <t>Fully in TB_R_INSTRUCTION: not taken by XD09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="45" t="inlineStr">
+        <is>
+          <t>4. 22-Oct XD08: ASN0007 received</t>
+        </is>
+      </c>
+      <c r="B35" s="46" t="n"/>
+      <c r="C35" s="46" t="n"/>
+      <c r="D35" s="46" t="n"/>
+      <c r="E35" s="46" t="n"/>
+      <c r="F35" s="46" t="n"/>
+      <c r="G35" s="46" t="n"/>
+      <c r="H35" s="46" t="n"/>
+      <c r="I35" s="46" t="n"/>
+      <c r="J35" s="46" t="n"/>
+      <c r="K35" s="46" t="n"/>
+      <c r="L35" s="46" t="n"/>
+      <c r="M35" s="46" t="n"/>
+      <c r="N35" s="46" t="n"/>
+      <c r="O35" s="46" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="D36" s="47" t="inlineStr">
+        <is>
+          <t>Replicated from DB Surrounding (G-System)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B37" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_CD</t>
+        </is>
+      </c>
+      <c r="C37" s="42" t="inlineStr">
+        <is>
+          <t>CUSTOMER_ORDER_NO</t>
+        </is>
+      </c>
+      <c r="D37" s="42" t="inlineStr">
+        <is>
+          <t>ORDER_DT</t>
+        </is>
+      </c>
+      <c r="E37" s="42" t="inlineStr">
+        <is>
+          <t>DESTINATION_CD</t>
+        </is>
+      </c>
+      <c r="F37" s="42" t="inlineStr">
+        <is>
+          <t>DETAILED_ITEM_NO</t>
+        </is>
+      </c>
+      <c r="G37" s="42" t="inlineStr">
+        <is>
+          <t>SERIAL_NO</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>SHIPPING_PART_NO</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS_QTY</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>HOLD_FLAG</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>PO_MAPPED_FLAG</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>UPD_STATUS</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="57" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="B38" s="58" t="inlineStr">
+        <is>
+          <t>9715300</t>
+        </is>
+      </c>
+      <c r="C38" s="58" t="inlineStr">
+        <is>
+          <t>CO-14115</t>
+        </is>
+      </c>
+      <c r="D38" s="58" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E38" s="58" t="inlineStr">
+        <is>
+          <t>9715310</t>
+        </is>
+      </c>
+      <c r="F38" s="58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G38" s="58" t="inlineStr">
+        <is>
+          <t>0000002</t>
+        </is>
+      </c>
+      <c r="H38" s="58" t="inlineStr">
+        <is>
+          <t>PART-X</t>
+        </is>
+      </c>
+      <c r="I38" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="J38" s="58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K38" s="58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L38" s="58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M38" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N38" s="58" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -23921,7 +25250,7 @@
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
+          <t>SIM-10, SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -23981,7 +25310,7 @@
       </c>
       <c r="F14" s="32" t="inlineStr">
         <is>
-          <t>SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
+          <t>SIM-10, SIM-2, SIM-4, SIM-5, SIM-6, SIM-7, SIM-8, SIM-9</t>
         </is>
       </c>
     </row>
@@ -40353,7 +41682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -40695,6 +42024,38 @@
       <c r="F13" s="32" t="inlineStr">
         <is>
           <t>Same unit as SIM-7 (PART-A 14-Oct: V01 VN 10, T01 TH 6, V02 VN 14; 6 pcs/case) but all 5 cases have a PO (p1 24 + p2 6). XD10 shows one check box per supplier case. The supplier wants cases 1 and 2 only: case 2 = VN 4 + TH 2 ends with VN 10 / TH 2 (CUT_FLAG N), so the warehouse could not close the VN and TH cases. XD10 ticks case 3 too (message no. 10): cases 1-3 = 18 pcs. [Create ASN] inserts the slices of cases 1-3; V01 and T01 are complete (PO_MAPPED_FLAG Y), V02 keeps 12 pcs open for a later ASN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="32" t="inlineStr">
+        <is>
+          <t>SIM-10</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>One line in 2 ASNs; partial receipt splits the serial → XD08 re-assigns TB_R_INSTRUCTION (simulasi_asn.xlsx)</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>BPF F2</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>XD09, XD10, XD08 (serial split)</t>
+        </is>
+      </c>
+      <c r="E14" s="32" t="inlineStr">
+        <is>
+          <t>TB_R_INSTRUCTION, TB_R_H0253_ORDER_CONTROL_PRE</t>
+        </is>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>CO-14115 VN 12 pcs (order date 19-Oct), 6 pcs/case: case 1 → ASN0006 (rit 1), case 2 → ASN0007 (rit 2). One H0253 row, two TB_R_INSTRUCTION rows. 21-Oct ASN0006 received: G-System splits the line into serial 0000001 6 pcs status 6 and serial 0000002 6 pcs status 7. Upsert alone: serial 0000001 has 12 pcs in TB_R_INSTRUCTION for qty 6 and serial 0000002 looks open (6) → XD09 would map it again (double). XD08 re-assigns the rows: serial 0000001 = ASN0006 (oldest ASN = received), serial 0000002 = ASN0007; both PO_MAPPED_FLAG Y.</t>
         </is>
       </c>
     </row>

</xml_diff>